<commit_message>
Actualizacion Images, anotaciones, fotos,admin student, CRUD bien para Student
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C36E64-D252-4A2C-9A3E-563C19C2DD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BDCB7E-91D5-4704-A7D1-C7264655AFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="77">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -165,24 +165,9 @@
     <t>TAREA</t>
   </si>
   <si>
-    <t>Tarea 1</t>
-  </si>
-  <si>
-    <t>Tarea 2</t>
-  </si>
-  <si>
-    <t>Tarea 3</t>
-  </si>
-  <si>
-    <t>Tarea 4</t>
-  </si>
-  <si>
     <t>Tarea 5</t>
   </si>
   <si>
-    <t>Título de la fase 4</t>
-  </si>
-  <si>
     <t>Inserte nuevas filas ENCIMA de ésta</t>
   </si>
   <si>
@@ -196,9 +181,6 @@
   </si>
   <si>
     <t>INICIO</t>
-  </si>
-  <si>
-    <t>fecha</t>
   </si>
   <si>
     <t>FIN</t>
@@ -257,9 +239,6 @@
     <t>Reasignar fotos</t>
   </si>
   <si>
-    <t>Revision Paginas</t>
-  </si>
-  <si>
     <t>Estructura Organización MCV</t>
   </si>
   <si>
@@ -278,15 +257,9 @@
     <t>forms/ManageStudent.php</t>
   </si>
   <si>
-    <t>CRUD</t>
-  </si>
-  <si>
     <t>Editar Datos Est</t>
   </si>
   <si>
-    <t>Eliminar Est</t>
-  </si>
-  <si>
     <t>Crear Datos Est</t>
   </si>
   <si>
@@ -299,13 +272,100 @@
     <t>Elimina y actualiza correctamente</t>
   </si>
   <si>
-    <t>Trigger</t>
-  </si>
-  <si>
     <t>views/AnnotationTrigger.php</t>
   </si>
   <si>
-    <t>Falla</t>
+    <t>CRUD Estudiante</t>
+  </si>
+  <si>
+    <t>CRUD Profesor</t>
+  </si>
+  <si>
+    <t>Editar Datos Prof</t>
+  </si>
+  <si>
+    <t>Actualizar Datos Prof</t>
+  </si>
+  <si>
+    <t>Eliminar Datos Prof</t>
+  </si>
+  <si>
+    <t>Crear Datos Prof</t>
+  </si>
+  <si>
+    <t>Eliminar Datos Est</t>
+  </si>
+  <si>
+    <t>Trigger Est</t>
+  </si>
+  <si>
+    <t>Trigger Prof</t>
+  </si>
+  <si>
+    <t>models\TeacherModel.php</t>
+  </si>
+  <si>
+    <t>Todo se encuentra en Teacher Model</t>
+  </si>
+  <si>
+    <t>Guardado de Imágenes Prof</t>
+  </si>
+  <si>
+    <t>CRUD Anotaciones</t>
+  </si>
+  <si>
+    <t>Es un Procedure</t>
+  </si>
+  <si>
+    <t>NO IMPLEMENTADO</t>
+  </si>
+  <si>
+    <t>Revision de Permisos</t>
+  </si>
+  <si>
+    <t>config/ProtectPages.php</t>
+  </si>
+  <si>
+    <t>Revision Paginas General</t>
+  </si>
+  <si>
+    <t>templates/HomeHeader.php</t>
+  </si>
+  <si>
+    <t>Permiso paginas de Header</t>
+  </si>
+  <si>
+    <t>Profesor</t>
+  </si>
+  <si>
+    <t>Dejar campos vacios Guardado</t>
+  </si>
+  <si>
+    <t>CRUD Insert New User</t>
+  </si>
+  <si>
+    <t>Obligatorio</t>
+  </si>
+  <si>
+    <t>Se crea bien con los foreing keys</t>
+  </si>
+  <si>
+    <t>Crear Anotacion</t>
+  </si>
+  <si>
+    <t>Eliminar Anotacion</t>
+  </si>
+  <si>
+    <t>Editar Anotacion</t>
+  </si>
+  <si>
+    <t>models/AnnotationsModel.php</t>
+  </si>
+  <si>
+    <t>Bien pero falta el Trigger</t>
+  </si>
+  <si>
+    <t>Se crea bien y funciona trigger</t>
   </si>
 </sst>
 </file>
@@ -553,7 +613,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="44">
+  <fills count="46">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -799,6 +859,18 @@
         <bgColor theme="4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="17">
     <border>
@@ -1073,7 +1145,7 @@
     <xf numFmtId="0" fontId="9" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1175,13 +1247,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="7">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="11" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1288,12 +1353,42 @@
     <xf numFmtId="172" fontId="28" fillId="42" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="2" xfId="12" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="44" borderId="2" xfId="12" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="44" borderId="2" xfId="11" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="44" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="44" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="45" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="45" borderId="2" xfId="11" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="45" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1313,6 +1408,15 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="7" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="55">
     <cellStyle name="20% - Énfasis1" xfId="31" builtinId="30" customBuiltin="1"/>
@@ -1949,12 +2053,13 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BM37"/>
+  <dimension ref="A1:BM45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="32" customWidth="1"/>
     <col min="2" max="2" width="30.5703125" customWidth="1"/>
-    <col min="3" max="4" width="28" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="10.42578125" style="5" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" customWidth="1"/>
@@ -1966,12 +2071,12 @@
     <col min="70" max="71" width="10.28515625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37" t="s">
-        <v>31</v>
+      <c r="B1" s="94" t="s">
+        <v>25</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1979,15 +2084,15 @@
       <c r="F1" s="4"/>
       <c r="G1" s="31"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="69" t="s">
-        <v>30</v>
+      <c r="J1" s="66" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="92" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="35"/>
@@ -1996,601 +2101,600 @@
       <c r="A3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="39" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="82"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="81">
-        <f ca="1">TODAY()</f>
-        <v>45823</v>
-      </c>
-      <c r="G3" s="81"/>
+      <c r="B3" s="93" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="89"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="88">
+        <v>45822</v>
+      </c>
+      <c r="G3" s="88"/>
     </row>
     <row r="4" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="82" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="82"/>
-      <c r="E4" s="83"/>
+      <c r="C4" s="89" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="89"/>
+      <c r="E4" s="90"/>
       <c r="F4" s="7">
         <v>1</v>
       </c>
-      <c r="J4" s="78">
-        <f ca="1">J5</f>
+      <c r="J4" s="85">
+        <f>J5</f>
+        <v>45817</v>
+      </c>
+      <c r="K4" s="86"/>
+      <c r="L4" s="86"/>
+      <c r="M4" s="86"/>
+      <c r="N4" s="86"/>
+      <c r="O4" s="86"/>
+      <c r="P4" s="87"/>
+      <c r="Q4" s="85">
+        <f>Q5</f>
         <v>45824</v>
       </c>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-      <c r="N4" s="79"/>
-      <c r="O4" s="79"/>
-      <c r="P4" s="80"/>
-      <c r="Q4" s="78">
-        <f ca="1">Q5</f>
+      <c r="R4" s="86"/>
+      <c r="S4" s="86"/>
+      <c r="T4" s="86"/>
+      <c r="U4" s="86"/>
+      <c r="V4" s="86"/>
+      <c r="W4" s="87"/>
+      <c r="X4" s="85">
+        <f>X5</f>
         <v>45831</v>
       </c>
-      <c r="R4" s="79"/>
-      <c r="S4" s="79"/>
-      <c r="T4" s="79"/>
-      <c r="U4" s="79"/>
-      <c r="V4" s="79"/>
-      <c r="W4" s="80"/>
-      <c r="X4" s="78">
-        <f ca="1">X5</f>
+      <c r="Y4" s="86"/>
+      <c r="Z4" s="86"/>
+      <c r="AA4" s="86"/>
+      <c r="AB4" s="86"/>
+      <c r="AC4" s="86"/>
+      <c r="AD4" s="87"/>
+      <c r="AE4" s="85">
+        <f>AE5</f>
         <v>45838</v>
       </c>
-      <c r="Y4" s="79"/>
-      <c r="Z4" s="79"/>
-      <c r="AA4" s="79"/>
-      <c r="AB4" s="79"/>
-      <c r="AC4" s="79"/>
-      <c r="AD4" s="80"/>
-      <c r="AE4" s="78">
-        <f ca="1">AE5</f>
+      <c r="AF4" s="86"/>
+      <c r="AG4" s="86"/>
+      <c r="AH4" s="86"/>
+      <c r="AI4" s="86"/>
+      <c r="AJ4" s="86"/>
+      <c r="AK4" s="87"/>
+      <c r="AL4" s="85">
+        <f>AL5</f>
         <v>45845</v>
       </c>
-      <c r="AF4" s="79"/>
-      <c r="AG4" s="79"/>
-      <c r="AH4" s="79"/>
-      <c r="AI4" s="79"/>
-      <c r="AJ4" s="79"/>
-      <c r="AK4" s="80"/>
-      <c r="AL4" s="78">
-        <f ca="1">AL5</f>
+      <c r="AM4" s="86"/>
+      <c r="AN4" s="86"/>
+      <c r="AO4" s="86"/>
+      <c r="AP4" s="86"/>
+      <c r="AQ4" s="86"/>
+      <c r="AR4" s="87"/>
+      <c r="AS4" s="85">
+        <f>AS5</f>
         <v>45852</v>
       </c>
-      <c r="AM4" s="79"/>
-      <c r="AN4" s="79"/>
-      <c r="AO4" s="79"/>
-      <c r="AP4" s="79"/>
-      <c r="AQ4" s="79"/>
-      <c r="AR4" s="80"/>
-      <c r="AS4" s="78">
-        <f ca="1">AS5</f>
+      <c r="AT4" s="86"/>
+      <c r="AU4" s="86"/>
+      <c r="AV4" s="86"/>
+      <c r="AW4" s="86"/>
+      <c r="AX4" s="86"/>
+      <c r="AY4" s="87"/>
+      <c r="AZ4" s="85">
+        <f>AZ5</f>
         <v>45859</v>
       </c>
-      <c r="AT4" s="79"/>
-      <c r="AU4" s="79"/>
-      <c r="AV4" s="79"/>
-      <c r="AW4" s="79"/>
-      <c r="AX4" s="79"/>
-      <c r="AY4" s="80"/>
-      <c r="AZ4" s="78">
-        <f ca="1">AZ5</f>
+      <c r="BA4" s="86"/>
+      <c r="BB4" s="86"/>
+      <c r="BC4" s="86"/>
+      <c r="BD4" s="86"/>
+      <c r="BE4" s="86"/>
+      <c r="BF4" s="87"/>
+      <c r="BG4" s="85">
+        <f>BG5</f>
         <v>45866</v>
       </c>
-      <c r="BA4" s="79"/>
-      <c r="BB4" s="79"/>
-      <c r="BC4" s="79"/>
-      <c r="BD4" s="79"/>
-      <c r="BE4" s="79"/>
-      <c r="BF4" s="80"/>
-      <c r="BG4" s="78">
-        <f ca="1">BG5</f>
-        <v>45873</v>
-      </c>
-      <c r="BH4" s="79"/>
-      <c r="BI4" s="79"/>
-      <c r="BJ4" s="79"/>
-      <c r="BK4" s="79"/>
-      <c r="BL4" s="79"/>
-      <c r="BM4" s="80"/>
+      <c r="BH4" s="86"/>
+      <c r="BI4" s="86"/>
+      <c r="BJ4" s="86"/>
+      <c r="BK4" s="86"/>
+      <c r="BL4" s="86"/>
+      <c r="BM4" s="87"/>
     </row>
     <row r="5" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="84"/>
-      <c r="C5" s="84"/>
-      <c r="D5" s="84"/>
-      <c r="E5" s="84"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="84"/>
-      <c r="H5" s="84"/>
-      <c r="J5" s="73">
-        <f ca="1">InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
+      <c r="B5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="91"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
+      <c r="J5" s="70">
+        <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
+        <v>45817</v>
+      </c>
+      <c r="K5" s="71">
+        <f>J5+1</f>
+        <v>45818</v>
+      </c>
+      <c r="L5" s="71">
+        <f t="shared" ref="L5:AY5" si="0">K5+1</f>
+        <v>45819</v>
+      </c>
+      <c r="M5" s="71">
+        <f t="shared" si="0"/>
+        <v>45820</v>
+      </c>
+      <c r="N5" s="71">
+        <f t="shared" si="0"/>
+        <v>45821</v>
+      </c>
+      <c r="O5" s="71">
+        <f t="shared" si="0"/>
+        <v>45822</v>
+      </c>
+      <c r="P5" s="72">
+        <f t="shared" si="0"/>
+        <v>45823</v>
+      </c>
+      <c r="Q5" s="70">
+        <f>P5+1</f>
         <v>45824</v>
       </c>
-      <c r="K5" s="74">
-        <f ca="1">J5+1</f>
+      <c r="R5" s="71">
+        <f>Q5+1</f>
         <v>45825</v>
       </c>
-      <c r="L5" s="74">
-        <f t="shared" ref="L5:AY5" ca="1" si="0">K5+1</f>
+      <c r="S5" s="71">
+        <f t="shared" si="0"/>
         <v>45826</v>
       </c>
-      <c r="M5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="T5" s="71">
+        <f t="shared" si="0"/>
         <v>45827</v>
       </c>
-      <c r="N5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="U5" s="71">
+        <f t="shared" si="0"/>
         <v>45828</v>
       </c>
-      <c r="O5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="V5" s="71">
+        <f t="shared" si="0"/>
         <v>45829</v>
       </c>
-      <c r="P5" s="75">
-        <f t="shared" ca="1" si="0"/>
+      <c r="W5" s="72">
+        <f t="shared" si="0"/>
         <v>45830</v>
       </c>
-      <c r="Q5" s="73">
-        <f ca="1">P5+1</f>
+      <c r="X5" s="70">
+        <f>W5+1</f>
         <v>45831</v>
       </c>
-      <c r="R5" s="74">
-        <f ca="1">Q5+1</f>
+      <c r="Y5" s="71">
+        <f>X5+1</f>
         <v>45832</v>
       </c>
-      <c r="S5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="Z5" s="71">
+        <f t="shared" si="0"/>
         <v>45833</v>
       </c>
-      <c r="T5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AA5" s="71">
+        <f t="shared" si="0"/>
         <v>45834</v>
       </c>
-      <c r="U5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AB5" s="71">
+        <f t="shared" si="0"/>
         <v>45835</v>
       </c>
-      <c r="V5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AC5" s="71">
+        <f t="shared" si="0"/>
         <v>45836</v>
       </c>
-      <c r="W5" s="75">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AD5" s="72">
+        <f t="shared" si="0"/>
         <v>45837</v>
       </c>
-      <c r="X5" s="73">
-        <f ca="1">W5+1</f>
+      <c r="AE5" s="70">
+        <f>AD5+1</f>
         <v>45838</v>
       </c>
-      <c r="Y5" s="74">
-        <f ca="1">X5+1</f>
+      <c r="AF5" s="71">
+        <f>AE5+1</f>
         <v>45839</v>
       </c>
-      <c r="Z5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AG5" s="71">
+        <f t="shared" si="0"/>
         <v>45840</v>
       </c>
-      <c r="AA5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AH5" s="71">
+        <f t="shared" si="0"/>
         <v>45841</v>
       </c>
-      <c r="AB5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AI5" s="71">
+        <f t="shared" si="0"/>
         <v>45842</v>
       </c>
-      <c r="AC5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AJ5" s="71">
+        <f t="shared" si="0"/>
         <v>45843</v>
       </c>
-      <c r="AD5" s="75">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AK5" s="72">
+        <f t="shared" si="0"/>
         <v>45844</v>
       </c>
-      <c r="AE5" s="73">
-        <f ca="1">AD5+1</f>
+      <c r="AL5" s="70">
+        <f>AK5+1</f>
         <v>45845</v>
       </c>
-      <c r="AF5" s="74">
-        <f ca="1">AE5+1</f>
+      <c r="AM5" s="71">
+        <f>AL5+1</f>
         <v>45846</v>
       </c>
-      <c r="AG5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AN5" s="71">
+        <f t="shared" si="0"/>
         <v>45847</v>
       </c>
-      <c r="AH5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AO5" s="71">
+        <f t="shared" si="0"/>
         <v>45848</v>
       </c>
-      <c r="AI5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AP5" s="71">
+        <f t="shared" si="0"/>
         <v>45849</v>
       </c>
-      <c r="AJ5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AQ5" s="71">
+        <f t="shared" si="0"/>
         <v>45850</v>
       </c>
-      <c r="AK5" s="75">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AR5" s="72">
+        <f t="shared" si="0"/>
         <v>45851</v>
       </c>
-      <c r="AL5" s="73">
-        <f ca="1">AK5+1</f>
+      <c r="AS5" s="70">
+        <f>AR5+1</f>
         <v>45852</v>
       </c>
-      <c r="AM5" s="74">
-        <f ca="1">AL5+1</f>
+      <c r="AT5" s="71">
+        <f>AS5+1</f>
         <v>45853</v>
       </c>
-      <c r="AN5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AU5" s="71">
+        <f t="shared" si="0"/>
         <v>45854</v>
       </c>
-      <c r="AO5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AV5" s="71">
+        <f t="shared" si="0"/>
         <v>45855</v>
       </c>
-      <c r="AP5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AW5" s="71">
+        <f t="shared" si="0"/>
         <v>45856</v>
       </c>
-      <c r="AQ5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AX5" s="71">
+        <f t="shared" si="0"/>
         <v>45857</v>
       </c>
-      <c r="AR5" s="75">
-        <f t="shared" ca="1" si="0"/>
+      <c r="AY5" s="72">
+        <f t="shared" si="0"/>
         <v>45858</v>
       </c>
-      <c r="AS5" s="73">
-        <f ca="1">AR5+1</f>
+      <c r="AZ5" s="70">
+        <f>AY5+1</f>
         <v>45859</v>
       </c>
-      <c r="AT5" s="74">
-        <f ca="1">AS5+1</f>
+      <c r="BA5" s="71">
+        <f>AZ5+1</f>
         <v>45860</v>
       </c>
-      <c r="AU5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BB5" s="71">
+        <f t="shared" ref="BB5:BF5" si="1">BA5+1</f>
         <v>45861</v>
       </c>
-      <c r="AV5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BC5" s="71">
+        <f t="shared" si="1"/>
         <v>45862</v>
       </c>
-      <c r="AW5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BD5" s="71">
+        <f t="shared" si="1"/>
         <v>45863</v>
       </c>
-      <c r="AX5" s="74">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BE5" s="71">
+        <f t="shared" si="1"/>
         <v>45864</v>
       </c>
-      <c r="AY5" s="75">
-        <f t="shared" ca="1" si="0"/>
+      <c r="BF5" s="72">
+        <f t="shared" si="1"/>
         <v>45865</v>
       </c>
-      <c r="AZ5" s="73">
-        <f ca="1">AY5+1</f>
+      <c r="BG5" s="70">
+        <f>BF5+1</f>
         <v>45866</v>
       </c>
-      <c r="BA5" s="74">
-        <f ca="1">AZ5+1</f>
+      <c r="BH5" s="71">
+        <f>BG5+1</f>
         <v>45867</v>
       </c>
-      <c r="BB5" s="74">
-        <f t="shared" ref="BB5:BF5" ca="1" si="1">BA5+1</f>
+      <c r="BI5" s="71">
+        <f t="shared" ref="BI5:BM5" si="2">BH5+1</f>
         <v>45868</v>
       </c>
-      <c r="BC5" s="74">
-        <f t="shared" ca="1" si="1"/>
+      <c r="BJ5" s="71">
+        <f t="shared" si="2"/>
         <v>45869</v>
       </c>
-      <c r="BD5" s="74">
-        <f t="shared" ca="1" si="1"/>
+      <c r="BK5" s="71">
+        <f t="shared" si="2"/>
         <v>45870</v>
       </c>
-      <c r="BE5" s="74">
-        <f t="shared" ca="1" si="1"/>
+      <c r="BL5" s="71">
+        <f t="shared" si="2"/>
         <v>45871</v>
       </c>
-      <c r="BF5" s="75">
-        <f t="shared" ca="1" si="1"/>
+      <c r="BM5" s="72">
+        <f t="shared" si="2"/>
         <v>45872</v>
-      </c>
-      <c r="BG5" s="73">
-        <f ca="1">BF5+1</f>
-        <v>45873</v>
-      </c>
-      <c r="BH5" s="74">
-        <f ca="1">BG5+1</f>
-        <v>45874</v>
-      </c>
-      <c r="BI5" s="74">
-        <f t="shared" ref="BI5:BM5" ca="1" si="2">BH5+1</f>
-        <v>45875</v>
-      </c>
-      <c r="BJ5" s="74">
-        <f t="shared" ca="1" si="2"/>
-        <v>45876</v>
-      </c>
-      <c r="BK5" s="74">
-        <f t="shared" ca="1" si="2"/>
-        <v>45877</v>
-      </c>
-      <c r="BL5" s="74">
-        <f t="shared" ca="1" si="2"/>
-        <v>45878</v>
-      </c>
-      <c r="BM5" s="75">
-        <f t="shared" ca="1" si="2"/>
-        <v>45879</v>
       </c>
     </row>
     <row r="6" spans="1:65" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="70" t="s">
+      <c r="B6" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="71" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" s="71" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="71" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="71" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="71" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="71"/>
-      <c r="I6" s="71" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" s="72" t="str">
-        <f t="shared" ref="J6" ca="1" si="3">LEFT(TEXT(J5,"ddd"),1)</f>
+      <c r="C6" s="68" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="68" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="68" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="69" t="str">
+        <f t="shared" ref="J6" si="3">LEFT(TEXT(J5,"ddd"),1)</f>
         <v>l</v>
       </c>
-      <c r="K6" s="72" t="str">
-        <f t="shared" ref="K6:AS6" ca="1" si="4">LEFT(TEXT(K5,"ddd"),1)</f>
+      <c r="K6" s="69" t="str">
+        <f t="shared" ref="K6:AS6" si="4">LEFT(TEXT(K5,"ddd"),1)</f>
         <v>m</v>
       </c>
-      <c r="L6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="L6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="M6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="M6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
-      <c r="N6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="N6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
-      <c r="O6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="O6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
-      <c r="P6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="P6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
-      <c r="Q6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="Q6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
-      <c r="R6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="R6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="S6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="S6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="T6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="T6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
-      <c r="U6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="U6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
-      <c r="V6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="V6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
-      <c r="W6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="W6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
-      <c r="X6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="X6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
-      <c r="Y6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="Y6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="Z6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="Z6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AA6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AA6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
-      <c r="AB6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AB6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
-      <c r="AC6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AC6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
-      <c r="AD6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AD6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
-      <c r="AE6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AE6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
-      <c r="AF6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AF6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AG6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AG6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AH6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AH6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
-      <c r="AI6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AI6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
-      <c r="AJ6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AJ6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
-      <c r="AK6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AK6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
-      <c r="AL6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AL6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
-      <c r="AM6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AM6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AN6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AN6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AO6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AO6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
-      <c r="AP6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AP6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
-      <c r="AQ6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AQ6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
-      <c r="AR6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AR6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
-      <c r="AS6" s="72" t="str">
-        <f t="shared" ca="1" si="4"/>
+      <c r="AS6" s="69" t="str">
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
-      <c r="AT6" s="72" t="str">
-        <f t="shared" ref="AT6:BM6" ca="1" si="5">LEFT(TEXT(AT5,"ddd"),1)</f>
+      <c r="AT6" s="69" t="str">
+        <f t="shared" ref="AT6:BM6" si="5">LEFT(TEXT(AT5,"ddd"),1)</f>
         <v>m</v>
       </c>
-      <c r="AU6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="AU6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
-      <c r="AV6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="AV6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>j</v>
       </c>
-      <c r="AW6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="AW6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>v</v>
       </c>
-      <c r="AX6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="AX6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>s</v>
       </c>
-      <c r="AY6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="AY6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>d</v>
       </c>
-      <c r="AZ6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="AZ6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>l</v>
       </c>
-      <c r="BA6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BA6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
-      <c r="BB6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BB6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
-      <c r="BC6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BC6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>j</v>
       </c>
-      <c r="BD6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BD6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>v</v>
       </c>
-      <c r="BE6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BE6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>s</v>
       </c>
-      <c r="BF6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BF6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>d</v>
       </c>
-      <c r="BG6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BG6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>l</v>
       </c>
-      <c r="BH6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BH6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
-      <c r="BI6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BI6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
-      <c r="BJ6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BJ6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>j</v>
       </c>
-      <c r="BK6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BK6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>v</v>
       </c>
-      <c r="BL6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BL6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>s</v>
       </c>
-      <c r="BM6" s="72" t="str">
-        <f t="shared" ca="1" si="5"/>
+      <c r="BM6" s="69" t="str">
+        <f t="shared" si="5"/>
         <v>d</v>
       </c>
     </row>
-    <row r="7" spans="1:65" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:65" ht="15.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="32" t="s">
         <v>6</v>
       </c>
@@ -2660,19 +2764,19 @@
     </row>
     <row r="8" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="54"/>
       <c r="G8" s="55"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11" t="str">
-        <f t="shared" ref="I8:I34" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
+        <f t="shared" ref="I8:I42" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
         <v/>
       </c>
       <c r="J8" s="28"/>
@@ -2733,31 +2837,29 @@
       <c r="BM8" s="28"/>
     </row>
     <row r="9" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="41" t="s">
+      <c r="A9" s="33"/>
+      <c r="B9" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="41"/>
-      <c r="E9" s="14">
-        <v>0.5</v>
+      <c r="C9" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="40"/>
+      <c r="E9" s="17">
+        <v>0</v>
       </c>
       <c r="F9" s="56">
-        <f ca="1">InicioDelProyecto</f>
-        <v>45823</v>
+        <f>F23+1</f>
+        <v>45830</v>
       </c>
       <c r="G9" s="56">
-        <f ca="1">F9+6</f>
-        <v>45829</v>
+        <f>F9+4</f>
+        <v>45834</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>7</v>
+        <f t="shared" si="6"/>
+        <v>5</v>
       </c>
       <c r="J9" s="28"/>
       <c r="K9" s="28"/>
@@ -2817,31 +2919,29 @@
       <c r="BM9" s="28"/>
     </row>
     <row r="10" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="41"/>
-      <c r="E10" s="14">
+      <c r="A10" s="32"/>
+      <c r="B10" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="40"/>
+      <c r="E10" s="17">
         <v>0</v>
       </c>
       <c r="F10" s="56">
-        <f ca="1">G9</f>
-        <v>45829</v>
+        <f>F9+2</f>
+        <v>45832</v>
       </c>
       <c r="G10" s="56">
-        <f ca="1">F10+2</f>
-        <v>45831</v>
+        <f>F10+5</f>
+        <v>45837</v>
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+        <f t="shared" si="6"/>
+        <v>6</v>
       </c>
       <c r="J10" s="28"/>
       <c r="K10" s="28"/>
@@ -2902,28 +3002,28 @@
     </row>
     <row r="11" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="32"/>
-      <c r="B11" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="41"/>
-      <c r="E11" s="14">
+      <c r="B11" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="40"/>
+      <c r="E11" s="17">
         <v>0</v>
       </c>
       <c r="F11" s="56">
-        <f ca="1">G10</f>
-        <v>45831</v>
+        <f>G10</f>
+        <v>45837</v>
       </c>
       <c r="G11" s="56">
-        <f ca="1">F11+4</f>
-        <v>45835</v>
+        <f>F11+3</f>
+        <v>45840</v>
       </c>
       <c r="H11" s="11"/>
       <c r="I11" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>5</v>
+        <f t="shared" si="6"/>
+        <v>4</v>
       </c>
       <c r="J11" s="28"/>
       <c r="K11" s="28"/>
@@ -2952,7 +3052,7 @@
       <c r="AH11" s="28"/>
       <c r="AI11" s="28"/>
       <c r="AJ11" s="28"/>
-      <c r="AK11" s="77"/>
+      <c r="AK11" s="28"/>
       <c r="AL11" s="28"/>
       <c r="AM11" s="28"/>
       <c r="AN11" s="28"/>
@@ -2984,26 +3084,29 @@
     </row>
     <row r="12" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="32"/>
-      <c r="B12" s="49" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" s="41"/>
-      <c r="E12" s="14">
-        <v>0.5</v>
+      <c r="B12" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="40"/>
+      <c r="E12" s="17">
+        <v>0</v>
       </c>
       <c r="F12" s="56">
-        <f ca="1">G11</f>
-        <v>45835</v>
+        <f>F11</f>
+        <v>45837</v>
       </c>
       <c r="G12" s="56">
-        <f ca="1">F12+4</f>
+        <f>F12+2</f>
         <v>45839</v>
       </c>
       <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
+      <c r="I12" s="11">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
       <c r="J12" s="28"/>
       <c r="K12" s="28"/>
       <c r="L12" s="28"/>
@@ -3020,7 +3123,7 @@
       <c r="W12" s="28"/>
       <c r="X12" s="28"/>
       <c r="Y12" s="28"/>
-      <c r="Z12" s="28"/>
+      <c r="Z12" s="29"/>
       <c r="AA12" s="28"/>
       <c r="AB12" s="28"/>
       <c r="AC12" s="28"/>
@@ -3031,7 +3134,7 @@
       <c r="AH12" s="28"/>
       <c r="AI12" s="28"/>
       <c r="AJ12" s="28"/>
-      <c r="AK12" s="77"/>
+      <c r="AK12" s="28"/>
       <c r="AL12" s="28"/>
       <c r="AM12" s="28"/>
       <c r="AN12" s="28"/>
@@ -3063,28 +3166,28 @@
     </row>
     <row r="13" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="32"/>
-      <c r="B13" s="49" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="41"/>
-      <c r="E13" s="14">
+      <c r="B13" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="40"/>
+      <c r="E13" s="17">
         <v>0</v>
       </c>
       <c r="F13" s="56">
-        <f ca="1">G11</f>
-        <v>45835</v>
+        <f>F12</f>
+        <v>45837</v>
       </c>
       <c r="G13" s="56">
-        <f ca="1">F13+5</f>
+        <f>F13+3</f>
         <v>45840</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>6</v>
+        <f t="shared" si="6"/>
+        <v>4</v>
       </c>
       <c r="J13" s="28"/>
       <c r="K13" s="28"/>
@@ -3102,7 +3205,7 @@
       <c r="W13" s="28"/>
       <c r="X13" s="28"/>
       <c r="Y13" s="28"/>
-      <c r="Z13" s="29"/>
+      <c r="Z13" s="28"/>
       <c r="AA13" s="28"/>
       <c r="AB13" s="28"/>
       <c r="AC13" s="28"/>
@@ -3144,29 +3247,21 @@
       <c r="BM13" s="28"/>
     </row>
     <row r="14" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
-      <c r="B14" s="49" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="41"/>
-      <c r="E14" s="14">
-        <v>0</v>
-      </c>
-      <c r="F14" s="56">
-        <f ca="1">F10+1</f>
-        <v>45830</v>
-      </c>
-      <c r="G14" s="56">
-        <f ca="1">F14+2</f>
-        <v>45832</v>
-      </c>
+      <c r="A14" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="52"/>
       <c r="H14" s="11"/>
-      <c r="I14" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>3</v>
+      <c r="I14" s="11" t="str">
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="J14" s="28"/>
       <c r="K14" s="28"/>
@@ -3227,20 +3322,30 @@
     </row>
     <row r="15" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="58"/>
+        <v>8</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="38"/>
+      <c r="E15" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="F15" s="53">
+        <f>InicioDelProyecto</f>
+        <v>45822</v>
+      </c>
+      <c r="G15" s="53">
+        <f>F15+6</f>
+        <v>45828</v>
+      </c>
       <c r="H15" s="11"/>
-      <c r="I15" s="11" t="str">
+      <c r="I15" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>7</v>
       </c>
       <c r="J15" s="28"/>
       <c r="K15" s="28"/>
@@ -3301,29 +3406,27 @@
     </row>
     <row r="16" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
-      <c r="B16" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="43"/>
-      <c r="E16" s="17">
+      <c r="B16" s="46" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="14">
         <v>0</v>
       </c>
-      <c r="F16" s="59">
-        <f ca="1">F14+1</f>
-        <v>45831</v>
-      </c>
-      <c r="G16" s="59">
-        <f ca="1">F16+4</f>
-        <v>45835</v>
+      <c r="F16" s="53">
+        <v>45851</v>
+      </c>
+      <c r="G16" s="53">
+        <f>F16+6</f>
+        <v>45857</v>
       </c>
       <c r="H16" s="11"/>
-      <c r="I16" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>5</v>
-      </c>
+      <c r="I16" s="11"/>
       <c r="J16" s="28"/>
       <c r="K16" s="28"/>
       <c r="L16" s="28"/>
@@ -3382,30 +3485,25 @@
       <c r="BM16" s="28"/>
     </row>
     <row r="17" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="32"/>
-      <c r="B17" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="43"/>
-      <c r="E17" s="17">
-        <v>0</v>
-      </c>
-      <c r="F17" s="59">
-        <f ca="1">F16+2</f>
-        <v>45833</v>
-      </c>
-      <c r="G17" s="59">
-        <f ca="1">F17+5</f>
-        <v>45838</v>
-      </c>
+      <c r="A17" s="33"/>
+      <c r="B17" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="14">
+        <v>0.2</v>
+      </c>
+      <c r="F17" s="53">
+        <v>45837</v>
+      </c>
+      <c r="G17" s="53"/>
       <c r="H17" s="11"/>
-      <c r="I17" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>6</v>
-      </c>
+      <c r="I17" s="11"/>
       <c r="J17" s="28"/>
       <c r="K17" s="28"/>
       <c r="L17" s="28"/>
@@ -3418,8 +3516,8 @@
       <c r="S17" s="28"/>
       <c r="T17" s="28"/>
       <c r="U17" s="28"/>
-      <c r="V17" s="29"/>
-      <c r="W17" s="29"/>
+      <c r="V17" s="28"/>
+      <c r="W17" s="28"/>
       <c r="X17" s="28"/>
       <c r="Y17" s="28"/>
       <c r="Z17" s="28"/>
@@ -3464,30 +3562,25 @@
       <c r="BM17" s="28"/>
     </row>
     <row r="18" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="32"/>
-      <c r="B18" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="43"/>
-      <c r="E18" s="17">
-        <v>0</v>
-      </c>
-      <c r="F18" s="59">
-        <f ca="1">G17</f>
-        <v>45838</v>
-      </c>
-      <c r="G18" s="59">
-        <f ca="1">F18+3</f>
-        <v>45841</v>
+      <c r="A18" s="33"/>
+      <c r="B18" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="38"/>
+      <c r="E18" s="14">
+        <v>1</v>
+      </c>
+      <c r="F18" s="53">
+        <v>45837</v>
+      </c>
+      <c r="G18" s="53">
+        <v>45837</v>
       </c>
       <c r="H18" s="11"/>
-      <c r="I18" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>4</v>
-      </c>
+      <c r="I18" s="11"/>
       <c r="J18" s="28"/>
       <c r="K18" s="28"/>
       <c r="L18" s="28"/>
@@ -3546,28 +3639,30 @@
       <c r="BM18" s="28"/>
     </row>
     <row r="19" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="32"/>
-      <c r="B19" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="43"/>
-      <c r="E19" s="17">
+      <c r="A19" s="33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="38"/>
+      <c r="E19" s="14">
         <v>0</v>
       </c>
-      <c r="F19" s="59">
-        <f ca="1">F18</f>
-        <v>45838</v>
-      </c>
-      <c r="G19" s="59">
-        <f ca="1">F19+2</f>
-        <v>45840</v>
+      <c r="F19" s="53">
+        <f>G15</f>
+        <v>45828</v>
+      </c>
+      <c r="G19" s="53">
+        <f>F19+2</f>
+        <v>45830</v>
       </c>
       <c r="H19" s="11"/>
       <c r="I19" s="11">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="J19" s="28"/>
@@ -3582,11 +3677,11 @@
       <c r="S19" s="28"/>
       <c r="T19" s="28"/>
       <c r="U19" s="28"/>
-      <c r="V19" s="28"/>
-      <c r="W19" s="28"/>
+      <c r="V19" s="29"/>
+      <c r="W19" s="29"/>
       <c r="X19" s="28"/>
       <c r="Y19" s="28"/>
-      <c r="Z19" s="29"/>
+      <c r="Z19" s="28"/>
       <c r="AA19" s="28"/>
       <c r="AB19" s="28"/>
       <c r="AC19" s="28"/>
@@ -3629,28 +3724,28 @@
     </row>
     <row r="20" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="32"/>
-      <c r="B20" s="76" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="D20" s="43"/>
-      <c r="E20" s="17">
+      <c r="B20" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="38"/>
+      <c r="E20" s="14">
         <v>0</v>
       </c>
-      <c r="F20" s="59">
-        <f ca="1">F19</f>
-        <v>45838</v>
-      </c>
-      <c r="G20" s="59">
-        <f ca="1">F20+3</f>
-        <v>45841</v>
+      <c r="F20" s="53">
+        <f>G19</f>
+        <v>45830</v>
+      </c>
+      <c r="G20" s="53">
+        <f>F20+4</f>
+        <v>45834</v>
       </c>
       <c r="H20" s="11"/>
       <c r="I20" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>4</v>
+        <f t="shared" si="6"/>
+        <v>5</v>
       </c>
       <c r="J20" s="28"/>
       <c r="K20" s="28"/>
@@ -3679,7 +3774,7 @@
       <c r="AH20" s="28"/>
       <c r="AI20" s="28"/>
       <c r="AJ20" s="28"/>
-      <c r="AK20" s="28"/>
+      <c r="AK20" s="73"/>
       <c r="AL20" s="28"/>
       <c r="AM20" s="28"/>
       <c r="AN20" s="28"/>
@@ -3710,22 +3805,27 @@
       <c r="BM20" s="28"/>
     </row>
     <row r="21" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61"/>
+      <c r="A21" s="32"/>
+      <c r="B21" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="38"/>
+      <c r="E21" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="F21" s="53">
+        <f>G20</f>
+        <v>45834</v>
+      </c>
+      <c r="G21" s="53">
+        <f>F21+4</f>
+        <v>45838</v>
+      </c>
       <c r="H21" s="11"/>
-      <c r="I21" s="11" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
+      <c r="I21" s="11"/>
       <c r="J21" s="28"/>
       <c r="K21" s="28"/>
       <c r="L21" s="28"/>
@@ -3753,7 +3853,7 @@
       <c r="AH21" s="28"/>
       <c r="AI21" s="28"/>
       <c r="AJ21" s="28"/>
-      <c r="AK21" s="28"/>
+      <c r="AK21" s="73"/>
       <c r="AL21" s="28"/>
       <c r="AM21" s="28"/>
       <c r="AN21" s="28"/>
@@ -3785,27 +3885,27 @@
     </row>
     <row r="22" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="32"/>
-      <c r="B22" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="45" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" s="45"/>
-      <c r="E22" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="F22" s="62">
-        <f ca="1">F9+15</f>
-        <v>45838</v>
-      </c>
-      <c r="G22" s="62">
-        <f ca="1">F22+5</f>
-        <v>45843</v>
+      <c r="B22" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="38"/>
+      <c r="E22" s="14">
+        <v>0</v>
+      </c>
+      <c r="F22" s="53">
+        <f>G20</f>
+        <v>45834</v>
+      </c>
+      <c r="G22" s="53">
+        <f>F22+5</f>
+        <v>45839</v>
       </c>
       <c r="H22" s="11"/>
       <c r="I22" s="11">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>6</v>
       </c>
       <c r="J22" s="28"/>
@@ -3824,7 +3924,7 @@
       <c r="W22" s="28"/>
       <c r="X22" s="28"/>
       <c r="Y22" s="28"/>
-      <c r="Z22" s="28"/>
+      <c r="Z22" s="29"/>
       <c r="AA22" s="28"/>
       <c r="AB22" s="28"/>
       <c r="AC22" s="28"/>
@@ -3867,28 +3967,28 @@
     </row>
     <row r="23" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="32"/>
-      <c r="B23" s="51" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="45"/>
-      <c r="E23" s="20">
+      <c r="B23" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="38"/>
+      <c r="E23" s="14">
         <v>0</v>
       </c>
-      <c r="F23" s="62">
-        <f ca="1">G22+1</f>
-        <v>45844</v>
-      </c>
-      <c r="G23" s="62">
-        <f ca="1">F23+4</f>
-        <v>45848</v>
+      <c r="F23" s="53">
+        <f>F19+1</f>
+        <v>45829</v>
+      </c>
+      <c r="G23" s="53">
+        <f>F23+2</f>
+        <v>45831</v>
       </c>
       <c r="H23" s="11"/>
       <c r="I23" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>5</v>
+        <f t="shared" si="6"/>
+        <v>3</v>
       </c>
       <c r="J23" s="28"/>
       <c r="K23" s="28"/>
@@ -3948,31 +4048,21 @@
       <c r="BM23" s="28"/>
     </row>
     <row r="24" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="32"/>
-      <c r="B24" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="45" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" s="20">
-        <v>1</v>
-      </c>
-      <c r="F24" s="62">
-        <f ca="1">F23+5</f>
-        <v>45849</v>
-      </c>
-      <c r="G24" s="62">
-        <f ca="1">F24+5</f>
-        <v>45854</v>
-      </c>
+      <c r="A24" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" s="80" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="84"/>
       <c r="H24" s="11"/>
-      <c r="I24" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>6</v>
+      <c r="I24" s="11" t="str">
+        <f t="shared" si="6"/>
+        <v/>
       </c>
       <c r="J24" s="28"/>
       <c r="K24" s="28"/>
@@ -4033,27 +4123,24 @@
     </row>
     <row r="25" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="32"/>
-      <c r="B25" s="51" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="D25" s="45"/>
-      <c r="E25" s="20">
+      <c r="B25" s="76" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="77"/>
+      <c r="D25" s="77"/>
+      <c r="E25" s="78">
         <v>0</v>
       </c>
-      <c r="F25" s="62">
-        <f ca="1">G24+1</f>
+      <c r="F25" s="79">
+        <v>45851</v>
+      </c>
+      <c r="G25" s="79">
+        <f>F25+4</f>
         <v>45855</v>
-      </c>
-      <c r="G25" s="62">
-        <f ca="1">F25+4</f>
-        <v>45859</v>
       </c>
       <c r="H25" s="11"/>
       <c r="I25" s="11">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="J25" s="28"/>
@@ -4115,30 +4202,26 @@
     </row>
     <row r="26" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32"/>
-      <c r="B26" s="51" t="s">
-        <v>54</v>
-      </c>
-      <c r="C26" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" s="45" t="s">
-        <v>56</v>
-      </c>
-      <c r="E26" s="20">
-        <v>1</v>
-      </c>
-      <c r="F26" s="62">
-        <f ca="1">F24</f>
-        <v>45849</v>
-      </c>
-      <c r="G26" s="62">
-        <f ca="1">F26+4</f>
-        <v>45853</v>
+      <c r="B26" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="77"/>
+      <c r="D26" s="77" t="s">
+        <v>75</v>
+      </c>
+      <c r="E26" s="78">
+        <v>0.5</v>
+      </c>
+      <c r="F26" s="79">
+        <v>45829</v>
+      </c>
+      <c r="G26" s="79">
+        <v>45829</v>
       </c>
       <c r="H26" s="11"/>
       <c r="I26" s="11">
-        <f t="shared" ca="1" si="6"/>
-        <v>5</v>
+        <f t="shared" si="6"/>
+        <v>1</v>
       </c>
       <c r="J26" s="28"/>
       <c r="K26" s="28"/>
@@ -4198,21 +4281,31 @@
       <c r="BM26" s="28"/>
     </row>
     <row r="27" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="C27" s="46"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="63"/>
-      <c r="G27" s="64"/>
+      <c r="A27" s="32"/>
+      <c r="B27" s="76" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="77" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="77" t="s">
+        <v>76</v>
+      </c>
+      <c r="E27" s="78">
+        <v>1</v>
+      </c>
+      <c r="F27" s="79">
+        <f>G26+1</f>
+        <v>45830</v>
+      </c>
+      <c r="G27" s="79">
+        <f>F27+4</f>
+        <v>45834</v>
+      </c>
       <c r="H27" s="11"/>
-      <c r="I27" s="11" t="str">
+      <c r="I27" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>5</v>
       </c>
       <c r="J27" s="28"/>
       <c r="K27" s="28"/>
@@ -4273,26 +4366,26 @@
     </row>
     <row r="28" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32"/>
-      <c r="B28" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="C28" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="D28" s="47"/>
-      <c r="E28" s="23">
+      <c r="B28" s="76" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="77"/>
+      <c r="E28" s="78">
         <v>0</v>
       </c>
-      <c r="F28" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="G28" s="65" t="s">
-        <v>27</v>
+      <c r="F28" s="79">
+        <v>45829</v>
+      </c>
+      <c r="G28" s="79">
+        <v>45829</v>
       </c>
       <c r="H28" s="11"/>
-      <c r="I28" s="11" t="e">
+      <c r="I28" s="11">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v>1</v>
       </c>
       <c r="J28" s="28"/>
       <c r="K28" s="28"/>
@@ -4352,27 +4445,21 @@
       <c r="BM28" s="28"/>
     </row>
     <row r="29" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="32"/>
-      <c r="B29" s="52" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="D29" s="47"/>
-      <c r="E29" s="23">
-        <v>0</v>
-      </c>
-      <c r="F29" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="G29" s="65" t="s">
-        <v>27</v>
-      </c>
+      <c r="A29" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="58"/>
       <c r="H29" s="11"/>
-      <c r="I29" s="11" t="e">
+      <c r="I29" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v/>
       </c>
       <c r="J29" s="28"/>
       <c r="K29" s="28"/>
@@ -4433,26 +4520,28 @@
     </row>
     <row r="30" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="32"/>
-      <c r="B30" s="52" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="D30" s="47"/>
-      <c r="E30" s="23">
-        <v>0</v>
-      </c>
-      <c r="F30" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="G30" s="65" t="s">
-        <v>27</v>
+      <c r="B30" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" s="42"/>
+      <c r="E30" s="20">
+        <v>0.5</v>
+      </c>
+      <c r="F30" s="59">
+        <f>F15+15</f>
+        <v>45837</v>
+      </c>
+      <c r="G30" s="59">
+        <f>F30+5</f>
+        <v>45842</v>
       </c>
       <c r="H30" s="11"/>
-      <c r="I30" s="11" t="e">
+      <c r="I30" s="11">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v>6</v>
       </c>
       <c r="J30" s="28"/>
       <c r="K30" s="28"/>
@@ -4513,26 +4602,28 @@
     </row>
     <row r="31" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32"/>
-      <c r="B31" s="52" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="D31" s="47"/>
-      <c r="E31" s="23">
+      <c r="B31" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="42"/>
+      <c r="E31" s="20">
         <v>0</v>
       </c>
-      <c r="F31" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="G31" s="65" t="s">
-        <v>27</v>
+      <c r="F31" s="59">
+        <f>G30+1</f>
+        <v>45843</v>
+      </c>
+      <c r="G31" s="59">
+        <f>F31+4</f>
+        <v>45847</v>
       </c>
       <c r="H31" s="11"/>
-      <c r="I31" s="11" t="e">
+      <c r="I31" s="11">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v>5</v>
       </c>
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
@@ -4593,26 +4684,28 @@
     </row>
     <row r="32" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32"/>
-      <c r="B32" s="52" t="s">
-        <v>20</v>
-      </c>
-      <c r="C32" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="D32" s="47"/>
-      <c r="E32" s="23">
-        <v>0</v>
-      </c>
-      <c r="F32" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="G32" s="65" t="s">
-        <v>27</v>
+      <c r="B32" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="20">
+        <v>1</v>
+      </c>
+      <c r="F32" s="59">
+        <v>45829</v>
+      </c>
+      <c r="G32" s="59">
+        <v>45829</v>
       </c>
       <c r="H32" s="11"/>
-      <c r="I32" s="11" t="e">
+      <c r="I32" s="11">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v>1</v>
       </c>
       <c r="J32" s="28"/>
       <c r="K32" s="28"/>
@@ -4672,19 +4765,29 @@
       <c r="BM32" s="28"/>
     </row>
     <row r="33" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B33" s="53"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="66"/>
-      <c r="G33" s="66"/>
+      <c r="A33" s="32"/>
+      <c r="B33" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33" s="20">
+        <v>1</v>
+      </c>
+      <c r="F33" s="59">
+        <v>45837</v>
+      </c>
+      <c r="G33" s="59">
+        <v>45851</v>
+      </c>
       <c r="H33" s="11"/>
-      <c r="I33" s="11" t="str">
+      <c r="I33" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>15</v>
       </c>
       <c r="J33" s="28"/>
       <c r="K33" s="28"/>
@@ -4744,90 +4847,715 @@
       <c r="BM33" s="28"/>
     </row>
     <row r="34" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B34" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="67"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27" t="str">
+      <c r="A34" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="74" t="s">
+        <v>56</v>
+      </c>
+      <c r="D34" s="43"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="60"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="J34" s="30"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="30"/>
-      <c r="M34" s="30"/>
-      <c r="N34" s="30"/>
-      <c r="O34" s="30"/>
-      <c r="P34" s="30"/>
-      <c r="Q34" s="30"/>
-      <c r="R34" s="30"/>
-      <c r="S34" s="30"/>
-      <c r="T34" s="30"/>
-      <c r="U34" s="30"/>
-      <c r="V34" s="30"/>
-      <c r="W34" s="30"/>
-      <c r="X34" s="30"/>
-      <c r="Y34" s="30"/>
-      <c r="Z34" s="30"/>
-      <c r="AA34" s="30"/>
-      <c r="AB34" s="30"/>
-      <c r="AC34" s="30"/>
-      <c r="AD34" s="30"/>
-      <c r="AE34" s="30"/>
-      <c r="AF34" s="30"/>
-      <c r="AG34" s="30"/>
-      <c r="AH34" s="30"/>
-      <c r="AI34" s="30"/>
-      <c r="AJ34" s="30"/>
-      <c r="AK34" s="30"/>
-      <c r="AL34" s="30"/>
-      <c r="AM34" s="30"/>
-      <c r="AN34" s="30"/>
-      <c r="AO34" s="30"/>
-      <c r="AP34" s="30"/>
-      <c r="AQ34" s="30"/>
-      <c r="AR34" s="30"/>
-      <c r="AS34" s="30"/>
-      <c r="AT34" s="30"/>
-      <c r="AU34" s="30"/>
-      <c r="AV34" s="30"/>
-      <c r="AW34" s="30"/>
-      <c r="AX34" s="30"/>
-      <c r="AY34" s="30"/>
-      <c r="AZ34" s="30"/>
-      <c r="BA34" s="30"/>
-      <c r="BB34" s="30"/>
-      <c r="BC34" s="30"/>
-      <c r="BD34" s="30"/>
-      <c r="BE34" s="30"/>
-      <c r="BF34" s="30"/>
-      <c r="BG34" s="30"/>
-      <c r="BH34" s="30"/>
-      <c r="BI34" s="30"/>
-      <c r="BJ34" s="30"/>
-      <c r="BK34" s="30"/>
-      <c r="BL34" s="30"/>
-      <c r="BM34" s="30"/>
+      <c r="J34" s="28"/>
+      <c r="K34" s="28"/>
+      <c r="L34" s="28"/>
+      <c r="M34" s="28"/>
+      <c r="N34" s="28"/>
+      <c r="O34" s="28"/>
+      <c r="P34" s="28"/>
+      <c r="Q34" s="28"/>
+      <c r="R34" s="28"/>
+      <c r="S34" s="28"/>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
+      <c r="V34" s="28"/>
+      <c r="W34" s="28"/>
+      <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
+      <c r="Z34" s="28"/>
+      <c r="AA34" s="28"/>
+      <c r="AB34" s="28"/>
+      <c r="AC34" s="28"/>
+      <c r="AD34" s="28"/>
+      <c r="AE34" s="28"/>
+      <c r="AF34" s="28"/>
+      <c r="AG34" s="28"/>
+      <c r="AH34" s="28"/>
+      <c r="AI34" s="28"/>
+      <c r="AJ34" s="28"/>
+      <c r="AK34" s="28"/>
+      <c r="AL34" s="28"/>
+      <c r="AM34" s="28"/>
+      <c r="AN34" s="28"/>
+      <c r="AO34" s="28"/>
+      <c r="AP34" s="28"/>
+      <c r="AQ34" s="28"/>
+      <c r="AR34" s="28"/>
+      <c r="AS34" s="28"/>
+      <c r="AT34" s="28"/>
+      <c r="AU34" s="28"/>
+      <c r="AV34" s="28"/>
+      <c r="AW34" s="28"/>
+      <c r="AX34" s="28"/>
+      <c r="AY34" s="28"/>
+      <c r="AZ34" s="28"/>
+      <c r="BA34" s="28"/>
+      <c r="BB34" s="28"/>
+      <c r="BC34" s="28"/>
+      <c r="BD34" s="28"/>
+      <c r="BE34" s="28"/>
+      <c r="BF34" s="28"/>
+      <c r="BG34" s="28"/>
+      <c r="BH34" s="28"/>
+      <c r="BI34" s="28"/>
+      <c r="BJ34" s="28"/>
+      <c r="BK34" s="28"/>
+      <c r="BL34" s="28"/>
+      <c r="BM34" s="28"/>
     </row>
-    <row r="35" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H35" s="6"/>
+    <row r="35" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="32"/>
+      <c r="B35" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D35" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35" s="23">
+        <v>1</v>
+      </c>
+      <c r="F35" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G35" s="62">
+        <v>45837</v>
+      </c>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="J35" s="28"/>
+      <c r="K35" s="28"/>
+      <c r="L35" s="28"/>
+      <c r="M35" s="28"/>
+      <c r="N35" s="28"/>
+      <c r="O35" s="28"/>
+      <c r="P35" s="28"/>
+      <c r="Q35" s="28"/>
+      <c r="R35" s="28"/>
+      <c r="S35" s="28"/>
+      <c r="T35" s="28"/>
+      <c r="U35" s="28"/>
+      <c r="V35" s="28"/>
+      <c r="W35" s="28"/>
+      <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
+      <c r="Z35" s="28"/>
+      <c r="AA35" s="28"/>
+      <c r="AB35" s="28"/>
+      <c r="AC35" s="28"/>
+      <c r="AD35" s="28"/>
+      <c r="AE35" s="28"/>
+      <c r="AF35" s="28"/>
+      <c r="AG35" s="28"/>
+      <c r="AH35" s="28"/>
+      <c r="AI35" s="28"/>
+      <c r="AJ35" s="28"/>
+      <c r="AK35" s="28"/>
+      <c r="AL35" s="28"/>
+      <c r="AM35" s="28"/>
+      <c r="AN35" s="28"/>
+      <c r="AO35" s="28"/>
+      <c r="AP35" s="28"/>
+      <c r="AQ35" s="28"/>
+      <c r="AR35" s="28"/>
+      <c r="AS35" s="28"/>
+      <c r="AT35" s="28"/>
+      <c r="AU35" s="28"/>
+      <c r="AV35" s="28"/>
+      <c r="AW35" s="28"/>
+      <c r="AX35" s="28"/>
+      <c r="AY35" s="28"/>
+      <c r="AZ35" s="28"/>
+      <c r="BA35" s="28"/>
+      <c r="BB35" s="28"/>
+      <c r="BC35" s="28"/>
+      <c r="BD35" s="28"/>
+      <c r="BE35" s="28"/>
+      <c r="BF35" s="28"/>
+      <c r="BG35" s="28"/>
+      <c r="BH35" s="28"/>
+      <c r="BI35" s="28"/>
+      <c r="BJ35" s="28"/>
+      <c r="BK35" s="28"/>
+      <c r="BL35" s="28"/>
+      <c r="BM35" s="28"/>
     </row>
-    <row r="36" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="G36" s="34"/>
+    <row r="36" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="32"/>
+      <c r="B36" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D36" s="44"/>
+      <c r="E36" s="23">
+        <v>1</v>
+      </c>
+      <c r="F36" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G36" s="62">
+        <v>45837</v>
+      </c>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="28"/>
+      <c r="M36" s="28"/>
+      <c r="N36" s="28"/>
+      <c r="O36" s="28"/>
+      <c r="P36" s="28"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="28"/>
+      <c r="S36" s="28"/>
+      <c r="T36" s="28"/>
+      <c r="U36" s="28"/>
+      <c r="V36" s="28"/>
+      <c r="W36" s="28"/>
+      <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
+      <c r="Z36" s="28"/>
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28"/>
+      <c r="AC36" s="28"/>
+      <c r="AD36" s="28"/>
+      <c r="AE36" s="28"/>
+      <c r="AF36" s="28"/>
+      <c r="AG36" s="28"/>
+      <c r="AH36" s="28"/>
+      <c r="AI36" s="28"/>
+      <c r="AJ36" s="28"/>
+      <c r="AK36" s="28"/>
+      <c r="AL36" s="28"/>
+      <c r="AM36" s="28"/>
+      <c r="AN36" s="28"/>
+      <c r="AO36" s="28"/>
+      <c r="AP36" s="28"/>
+      <c r="AQ36" s="28"/>
+      <c r="AR36" s="28"/>
+      <c r="AS36" s="28"/>
+      <c r="AT36" s="28"/>
+      <c r="AU36" s="28"/>
+      <c r="AV36" s="28"/>
+      <c r="AW36" s="28"/>
+      <c r="AX36" s="28"/>
+      <c r="AY36" s="28"/>
+      <c r="AZ36" s="28"/>
+      <c r="BA36" s="28"/>
+      <c r="BB36" s="28"/>
+      <c r="BC36" s="28"/>
+      <c r="BD36" s="28"/>
+      <c r="BE36" s="28"/>
+      <c r="BF36" s="28"/>
+      <c r="BG36" s="28"/>
+      <c r="BH36" s="28"/>
+      <c r="BI36" s="28"/>
+      <c r="BJ36" s="28"/>
+      <c r="BK36" s="28"/>
+      <c r="BL36" s="28"/>
+      <c r="BM36" s="28"/>
     </row>
-    <row r="37" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
+    <row r="37" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="32"/>
+      <c r="B37" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="44"/>
+      <c r="E37" s="23">
+        <v>1</v>
+      </c>
+      <c r="F37" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G37" s="62">
+        <v>45837</v>
+      </c>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="J37" s="28"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="28"/>
+      <c r="O37" s="28"/>
+      <c r="P37" s="28"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="28"/>
+      <c r="S37" s="28"/>
+      <c r="T37" s="28"/>
+      <c r="U37" s="28"/>
+      <c r="V37" s="28"/>
+      <c r="W37" s="28"/>
+      <c r="X37" s="28"/>
+      <c r="Y37" s="28"/>
+      <c r="Z37" s="28"/>
+      <c r="AA37" s="28"/>
+      <c r="AB37" s="28"/>
+      <c r="AC37" s="28"/>
+      <c r="AD37" s="28"/>
+      <c r="AE37" s="28"/>
+      <c r="AF37" s="28"/>
+      <c r="AG37" s="28"/>
+      <c r="AH37" s="28"/>
+      <c r="AI37" s="28"/>
+      <c r="AJ37" s="28"/>
+      <c r="AK37" s="28"/>
+      <c r="AL37" s="28"/>
+      <c r="AM37" s="28"/>
+      <c r="AN37" s="28"/>
+      <c r="AO37" s="28"/>
+      <c r="AP37" s="28"/>
+      <c r="AQ37" s="28"/>
+      <c r="AR37" s="28"/>
+      <c r="AS37" s="28"/>
+      <c r="AT37" s="28"/>
+      <c r="AU37" s="28"/>
+      <c r="AV37" s="28"/>
+      <c r="AW37" s="28"/>
+      <c r="AX37" s="28"/>
+      <c r="AY37" s="28"/>
+      <c r="AZ37" s="28"/>
+      <c r="BA37" s="28"/>
+      <c r="BB37" s="28"/>
+      <c r="BC37" s="28"/>
+      <c r="BD37" s="28"/>
+      <c r="BE37" s="28"/>
+      <c r="BF37" s="28"/>
+      <c r="BG37" s="28"/>
+      <c r="BH37" s="28"/>
+      <c r="BI37" s="28"/>
+      <c r="BJ37" s="28"/>
+      <c r="BK37" s="28"/>
+      <c r="BL37" s="28"/>
+      <c r="BM37" s="28"/>
+    </row>
+    <row r="38" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="32"/>
+      <c r="B38" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D38" s="44"/>
+      <c r="E38" s="23">
+        <v>1</v>
+      </c>
+      <c r="F38" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G38" s="62">
+        <v>45837</v>
+      </c>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="J38" s="28"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="28"/>
+      <c r="M38" s="28"/>
+      <c r="N38" s="28"/>
+      <c r="O38" s="28"/>
+      <c r="P38" s="28"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="28"/>
+      <c r="S38" s="28"/>
+      <c r="T38" s="28"/>
+      <c r="U38" s="28"/>
+      <c r="V38" s="28"/>
+      <c r="W38" s="28"/>
+      <c r="X38" s="28"/>
+      <c r="Y38" s="28"/>
+      <c r="Z38" s="28"/>
+      <c r="AA38" s="28"/>
+      <c r="AB38" s="28"/>
+      <c r="AC38" s="28"/>
+      <c r="AD38" s="28"/>
+      <c r="AE38" s="28"/>
+      <c r="AF38" s="28"/>
+      <c r="AG38" s="28"/>
+      <c r="AH38" s="28"/>
+      <c r="AI38" s="28"/>
+      <c r="AJ38" s="28"/>
+      <c r="AK38" s="28"/>
+      <c r="AL38" s="28"/>
+      <c r="AM38" s="28"/>
+      <c r="AN38" s="28"/>
+      <c r="AO38" s="28"/>
+      <c r="AP38" s="28"/>
+      <c r="AQ38" s="28"/>
+      <c r="AR38" s="28"/>
+      <c r="AS38" s="28"/>
+      <c r="AT38" s="28"/>
+      <c r="AU38" s="28"/>
+      <c r="AV38" s="28"/>
+      <c r="AW38" s="28"/>
+      <c r="AX38" s="28"/>
+      <c r="AY38" s="28"/>
+      <c r="AZ38" s="28"/>
+      <c r="BA38" s="28"/>
+      <c r="BB38" s="28"/>
+      <c r="BC38" s="28"/>
+      <c r="BD38" s="28"/>
+      <c r="BE38" s="28"/>
+      <c r="BF38" s="28"/>
+      <c r="BG38" s="28"/>
+      <c r="BH38" s="28"/>
+      <c r="BI38" s="28"/>
+      <c r="BJ38" s="28"/>
+      <c r="BK38" s="28"/>
+      <c r="BL38" s="28"/>
+      <c r="BM38" s="28"/>
+    </row>
+    <row r="39" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="32"/>
+      <c r="B39" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D39" s="44"/>
+      <c r="E39" s="23">
+        <v>1</v>
+      </c>
+      <c r="F39" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G39" s="62">
+        <v>45837</v>
+      </c>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="J39" s="28"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="28"/>
+      <c r="M39" s="28"/>
+      <c r="N39" s="28"/>
+      <c r="O39" s="28"/>
+      <c r="P39" s="28"/>
+      <c r="Q39" s="28"/>
+      <c r="R39" s="28"/>
+      <c r="S39" s="28"/>
+      <c r="T39" s="28"/>
+      <c r="U39" s="28"/>
+      <c r="V39" s="28"/>
+      <c r="W39" s="28"/>
+      <c r="X39" s="28"/>
+      <c r="Y39" s="28"/>
+      <c r="Z39" s="28"/>
+      <c r="AA39" s="28"/>
+      <c r="AB39" s="28"/>
+      <c r="AC39" s="28"/>
+      <c r="AD39" s="28"/>
+      <c r="AE39" s="28"/>
+      <c r="AF39" s="28"/>
+      <c r="AG39" s="28"/>
+      <c r="AH39" s="28"/>
+      <c r="AI39" s="28"/>
+      <c r="AJ39" s="28"/>
+      <c r="AK39" s="28"/>
+      <c r="AL39" s="28"/>
+      <c r="AM39" s="28"/>
+      <c r="AN39" s="28"/>
+      <c r="AO39" s="28"/>
+      <c r="AP39" s="28"/>
+      <c r="AQ39" s="28"/>
+      <c r="AR39" s="28"/>
+      <c r="AS39" s="28"/>
+      <c r="AT39" s="28"/>
+      <c r="AU39" s="28"/>
+      <c r="AV39" s="28"/>
+      <c r="AW39" s="28"/>
+      <c r="AX39" s="28"/>
+      <c r="AY39" s="28"/>
+      <c r="AZ39" s="28"/>
+      <c r="BA39" s="28"/>
+      <c r="BB39" s="28"/>
+      <c r="BC39" s="28"/>
+      <c r="BD39" s="28"/>
+      <c r="BE39" s="28"/>
+      <c r="BF39" s="28"/>
+      <c r="BG39" s="28"/>
+      <c r="BH39" s="28"/>
+      <c r="BI39" s="28"/>
+      <c r="BJ39" s="28"/>
+      <c r="BK39" s="28"/>
+      <c r="BL39" s="28"/>
+      <c r="BM39" s="28"/>
+    </row>
+    <row r="40" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="32"/>
+      <c r="B40" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="C40" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="E40" s="23">
+        <v>0</v>
+      </c>
+      <c r="F40" s="62"/>
+      <c r="G40" s="62"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J40" s="28"/>
+      <c r="K40" s="28"/>
+      <c r="L40" s="28"/>
+      <c r="M40" s="28"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="28"/>
+      <c r="P40" s="28"/>
+      <c r="Q40" s="28"/>
+      <c r="R40" s="28"/>
+      <c r="S40" s="28"/>
+      <c r="T40" s="28"/>
+      <c r="U40" s="28"/>
+      <c r="V40" s="28"/>
+      <c r="W40" s="28"/>
+      <c r="X40" s="28"/>
+      <c r="Y40" s="28"/>
+      <c r="Z40" s="28"/>
+      <c r="AA40" s="28"/>
+      <c r="AB40" s="28"/>
+      <c r="AC40" s="28"/>
+      <c r="AD40" s="28"/>
+      <c r="AE40" s="28"/>
+      <c r="AF40" s="28"/>
+      <c r="AG40" s="28"/>
+      <c r="AH40" s="28"/>
+      <c r="AI40" s="28"/>
+      <c r="AJ40" s="28"/>
+      <c r="AK40" s="28"/>
+      <c r="AL40" s="28"/>
+      <c r="AM40" s="28"/>
+      <c r="AN40" s="28"/>
+      <c r="AO40" s="28"/>
+      <c r="AP40" s="28"/>
+      <c r="AQ40" s="28"/>
+      <c r="AR40" s="28"/>
+      <c r="AS40" s="28"/>
+      <c r="AT40" s="28"/>
+      <c r="AU40" s="28"/>
+      <c r="AV40" s="28"/>
+      <c r="AW40" s="28"/>
+      <c r="AX40" s="28"/>
+      <c r="AY40" s="28"/>
+      <c r="AZ40" s="28"/>
+      <c r="BA40" s="28"/>
+      <c r="BB40" s="28"/>
+      <c r="BC40" s="28"/>
+      <c r="BD40" s="28"/>
+      <c r="BE40" s="28"/>
+      <c r="BF40" s="28"/>
+      <c r="BG40" s="28"/>
+      <c r="BH40" s="28"/>
+      <c r="BI40" s="28"/>
+      <c r="BJ40" s="28"/>
+      <c r="BK40" s="28"/>
+      <c r="BL40" s="28"/>
+      <c r="BM40" s="28"/>
+    </row>
+    <row r="41" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" s="50"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="45"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J41" s="28"/>
+      <c r="K41" s="28"/>
+      <c r="L41" s="28"/>
+      <c r="M41" s="28"/>
+      <c r="N41" s="28"/>
+      <c r="O41" s="28"/>
+      <c r="P41" s="28"/>
+      <c r="Q41" s="28"/>
+      <c r="R41" s="28"/>
+      <c r="S41" s="28"/>
+      <c r="T41" s="28"/>
+      <c r="U41" s="28"/>
+      <c r="V41" s="28"/>
+      <c r="W41" s="28"/>
+      <c r="X41" s="28"/>
+      <c r="Y41" s="28"/>
+      <c r="Z41" s="28"/>
+      <c r="AA41" s="28"/>
+      <c r="AB41" s="28"/>
+      <c r="AC41" s="28"/>
+      <c r="AD41" s="28"/>
+      <c r="AE41" s="28"/>
+      <c r="AF41" s="28"/>
+      <c r="AG41" s="28"/>
+      <c r="AH41" s="28"/>
+      <c r="AI41" s="28"/>
+      <c r="AJ41" s="28"/>
+      <c r="AK41" s="28"/>
+      <c r="AL41" s="28"/>
+      <c r="AM41" s="28"/>
+      <c r="AN41" s="28"/>
+      <c r="AO41" s="28"/>
+      <c r="AP41" s="28"/>
+      <c r="AQ41" s="28"/>
+      <c r="AR41" s="28"/>
+      <c r="AS41" s="28"/>
+      <c r="AT41" s="28"/>
+      <c r="AU41" s="28"/>
+      <c r="AV41" s="28"/>
+      <c r="AW41" s="28"/>
+      <c r="AX41" s="28"/>
+      <c r="AY41" s="28"/>
+      <c r="AZ41" s="28"/>
+      <c r="BA41" s="28"/>
+      <c r="BB41" s="28"/>
+      <c r="BC41" s="28"/>
+      <c r="BD41" s="28"/>
+      <c r="BE41" s="28"/>
+      <c r="BF41" s="28"/>
+      <c r="BG41" s="28"/>
+      <c r="BH41" s="28"/>
+      <c r="BI41" s="28"/>
+      <c r="BJ41" s="28"/>
+      <c r="BK41" s="28"/>
+      <c r="BL41" s="28"/>
+      <c r="BM41" s="28"/>
+    </row>
+    <row r="42" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="26"/>
+      <c r="F42" s="64"/>
+      <c r="G42" s="65"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J42" s="30"/>
+      <c r="K42" s="30"/>
+      <c r="L42" s="30"/>
+      <c r="M42" s="30"/>
+      <c r="N42" s="30"/>
+      <c r="O42" s="30"/>
+      <c r="P42" s="30"/>
+      <c r="Q42" s="30"/>
+      <c r="R42" s="30"/>
+      <c r="S42" s="30"/>
+      <c r="T42" s="30"/>
+      <c r="U42" s="30"/>
+      <c r="V42" s="30"/>
+      <c r="W42" s="30"/>
+      <c r="X42" s="30"/>
+      <c r="Y42" s="30"/>
+      <c r="Z42" s="30"/>
+      <c r="AA42" s="30"/>
+      <c r="AB42" s="30"/>
+      <c r="AC42" s="30"/>
+      <c r="AD42" s="30"/>
+      <c r="AE42" s="30"/>
+      <c r="AF42" s="30"/>
+      <c r="AG42" s="30"/>
+      <c r="AH42" s="30"/>
+      <c r="AI42" s="30"/>
+      <c r="AJ42" s="30"/>
+      <c r="AK42" s="30"/>
+      <c r="AL42" s="30"/>
+      <c r="AM42" s="30"/>
+      <c r="AN42" s="30"/>
+      <c r="AO42" s="30"/>
+      <c r="AP42" s="30"/>
+      <c r="AQ42" s="30"/>
+      <c r="AR42" s="30"/>
+      <c r="AS42" s="30"/>
+      <c r="AT42" s="30"/>
+      <c r="AU42" s="30"/>
+      <c r="AV42" s="30"/>
+      <c r="AW42" s="30"/>
+      <c r="AX42" s="30"/>
+      <c r="AY42" s="30"/>
+      <c r="AZ42" s="30"/>
+      <c r="BA42" s="30"/>
+      <c r="BB42" s="30"/>
+      <c r="BC42" s="30"/>
+      <c r="BD42" s="30"/>
+      <c r="BE42" s="30"/>
+      <c r="BF42" s="30"/>
+      <c r="BG42" s="30"/>
+      <c r="BH42" s="30"/>
+      <c r="BI42" s="30"/>
+      <c r="BJ42" s="30"/>
+      <c r="BK42" s="30"/>
+      <c r="BL42" s="30"/>
+      <c r="BM42" s="30"/>
+    </row>
+    <row r="43" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H43" s="6"/>
+    </row>
+    <row r="44" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="G44" s="34"/>
+    </row>
+    <row r="45" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4844,7 +5572,7 @@
     <mergeCell ref="X4:AD4"/>
     <mergeCell ref="AE4:AK4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E34">
+  <conditionalFormatting sqref="E7:E42">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -4858,12 +5586,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:BM34">
+  <conditionalFormatting sqref="J5:BM42">
     <cfRule type="expression" dxfId="2" priority="33">
       <formula>AND(TODAY()&gt;=J$5,TODAY()&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:BM34">
+  <conditionalFormatting sqref="J7:BM42">
     <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(Fecha_incio&lt;=J$5,ROUNDDOWN((Fecha_final-Fecha_incio+1)*Progresos,0)+Fecha_incio-1&gt;=J$5)</formula>
     </cfRule>
@@ -4871,7 +5599,7 @@
       <formula>AND(Fecha_final&gt;=J$5,Fecha_incio&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Mostrar semana" prompt="Al cambiar este número, se desplazará la vista del diagrama de Gantt." sqref="F4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
     </dataValidation>
@@ -4882,9 +5610,6 @@
   <headerFooter differentFirst="1" scaleWithDoc="0">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
-  <ignoredErrors>
-    <ignoredError sqref="G19" formula="1"/>
-  </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -4901,7 +5626,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E7:E34</xm:sqref>
+          <xm:sqref>E7:E42</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Update Anotacion CRUD, File AnnotationsModel.php se añadio lineas y codigo, tambien se elimino codigo innecesario o repetitivo
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BDCB7E-91D5-4704-A7D1-C7264655AFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206DFF13-FCB9-4645-8756-AA2C46E93FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="82">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -296,9 +296,6 @@
     <t>Eliminar Datos Est</t>
   </si>
   <si>
-    <t>Trigger Est</t>
-  </si>
-  <si>
     <t>Trigger Prof</t>
   </si>
   <si>
@@ -362,10 +359,28 @@
     <t>models/AnnotationsModel.php</t>
   </si>
   <si>
-    <t>Bien pero falta el Trigger</t>
-  </si>
-  <si>
     <t>Se crea bien y funciona trigger</t>
+  </si>
+  <si>
+    <t>ManageStudent.php</t>
+  </si>
+  <si>
+    <t>Funciona Cambiar Archivo</t>
+  </si>
+  <si>
+    <t>teacher/AnnotationsHistory.php</t>
+  </si>
+  <si>
+    <t>Eliminar y actualiza tabla historial ope</t>
+  </si>
+  <si>
+    <t>Trigger Anotaciones</t>
+  </si>
+  <si>
+    <t>Funciona bien el trigger</t>
+  </si>
+  <si>
+    <t>Permitir dejar campos vacios</t>
   </si>
 </sst>
 </file>
@@ -1389,6 +1404,15 @@
     <xf numFmtId="169" fontId="5" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="7" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1408,15 +1432,6 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="7" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="55">
     <cellStyle name="20% - Énfasis1" xfId="31" builtinId="30" customBuiltin="1"/>
@@ -2059,7 +2074,7 @@
     <col min="1" max="1" width="2.7109375" style="32" customWidth="1"/>
     <col min="2" max="2" width="30.5703125" customWidth="1"/>
     <col min="3" max="3" width="34.5703125" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="4" max="4" width="34.85546875" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="10.42578125" style="5" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" customWidth="1"/>
@@ -2075,7 +2090,7 @@
       <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="94" t="s">
+      <c r="B1" s="87" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="1"/>
@@ -2092,7 +2107,7 @@
       <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="92" t="s">
+      <c r="B2" s="85" t="s">
         <v>14</v>
       </c>
       <c r="J2" s="35"/>
@@ -2101,123 +2116,123 @@
       <c r="A3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="93" t="s">
+      <c r="B3" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="92" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="88">
+      <c r="D3" s="92"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="91">
         <v>45822</v>
       </c>
-      <c r="G3" s="88"/>
+      <c r="G3" s="91"/>
     </row>
     <row r="4" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="89" t="s">
+      <c r="C4" s="92" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="89"/>
-      <c r="E4" s="90"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="93"/>
       <c r="F4" s="7">
         <v>1</v>
       </c>
-      <c r="J4" s="85">
+      <c r="J4" s="88">
         <f>J5</f>
         <v>45817</v>
       </c>
-      <c r="K4" s="86"/>
-      <c r="L4" s="86"/>
-      <c r="M4" s="86"/>
-      <c r="N4" s="86"/>
-      <c r="O4" s="86"/>
-      <c r="P4" s="87"/>
-      <c r="Q4" s="85">
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="M4" s="89"/>
+      <c r="N4" s="89"/>
+      <c r="O4" s="89"/>
+      <c r="P4" s="90"/>
+      <c r="Q4" s="88">
         <f>Q5</f>
         <v>45824</v>
       </c>
-      <c r="R4" s="86"/>
-      <c r="S4" s="86"/>
-      <c r="T4" s="86"/>
-      <c r="U4" s="86"/>
-      <c r="V4" s="86"/>
-      <c r="W4" s="87"/>
-      <c r="X4" s="85">
+      <c r="R4" s="89"/>
+      <c r="S4" s="89"/>
+      <c r="T4" s="89"/>
+      <c r="U4" s="89"/>
+      <c r="V4" s="89"/>
+      <c r="W4" s="90"/>
+      <c r="X4" s="88">
         <f>X5</f>
         <v>45831</v>
       </c>
-      <c r="Y4" s="86"/>
-      <c r="Z4" s="86"/>
-      <c r="AA4" s="86"/>
-      <c r="AB4" s="86"/>
-      <c r="AC4" s="86"/>
-      <c r="AD4" s="87"/>
-      <c r="AE4" s="85">
+      <c r="Y4" s="89"/>
+      <c r="Z4" s="89"/>
+      <c r="AA4" s="89"/>
+      <c r="AB4" s="89"/>
+      <c r="AC4" s="89"/>
+      <c r="AD4" s="90"/>
+      <c r="AE4" s="88">
         <f>AE5</f>
         <v>45838</v>
       </c>
-      <c r="AF4" s="86"/>
-      <c r="AG4" s="86"/>
-      <c r="AH4" s="86"/>
-      <c r="AI4" s="86"/>
-      <c r="AJ4" s="86"/>
-      <c r="AK4" s="87"/>
-      <c r="AL4" s="85">
+      <c r="AF4" s="89"/>
+      <c r="AG4" s="89"/>
+      <c r="AH4" s="89"/>
+      <c r="AI4" s="89"/>
+      <c r="AJ4" s="89"/>
+      <c r="AK4" s="90"/>
+      <c r="AL4" s="88">
         <f>AL5</f>
         <v>45845</v>
       </c>
-      <c r="AM4" s="86"/>
-      <c r="AN4" s="86"/>
-      <c r="AO4" s="86"/>
-      <c r="AP4" s="86"/>
-      <c r="AQ4" s="86"/>
-      <c r="AR4" s="87"/>
-      <c r="AS4" s="85">
+      <c r="AM4" s="89"/>
+      <c r="AN4" s="89"/>
+      <c r="AO4" s="89"/>
+      <c r="AP4" s="89"/>
+      <c r="AQ4" s="89"/>
+      <c r="AR4" s="90"/>
+      <c r="AS4" s="88">
         <f>AS5</f>
         <v>45852</v>
       </c>
-      <c r="AT4" s="86"/>
-      <c r="AU4" s="86"/>
-      <c r="AV4" s="86"/>
-      <c r="AW4" s="86"/>
-      <c r="AX4" s="86"/>
-      <c r="AY4" s="87"/>
-      <c r="AZ4" s="85">
+      <c r="AT4" s="89"/>
+      <c r="AU4" s="89"/>
+      <c r="AV4" s="89"/>
+      <c r="AW4" s="89"/>
+      <c r="AX4" s="89"/>
+      <c r="AY4" s="90"/>
+      <c r="AZ4" s="88">
         <f>AZ5</f>
         <v>45859</v>
       </c>
-      <c r="BA4" s="86"/>
-      <c r="BB4" s="86"/>
-      <c r="BC4" s="86"/>
-      <c r="BD4" s="86"/>
-      <c r="BE4" s="86"/>
-      <c r="BF4" s="87"/>
-      <c r="BG4" s="85">
+      <c r="BA4" s="89"/>
+      <c r="BB4" s="89"/>
+      <c r="BC4" s="89"/>
+      <c r="BD4" s="89"/>
+      <c r="BE4" s="89"/>
+      <c r="BF4" s="90"/>
+      <c r="BG4" s="88">
         <f>BG5</f>
         <v>45866</v>
       </c>
-      <c r="BH4" s="86"/>
-      <c r="BI4" s="86"/>
-      <c r="BJ4" s="86"/>
-      <c r="BK4" s="86"/>
-      <c r="BL4" s="86"/>
-      <c r="BM4" s="87"/>
+      <c r="BH4" s="89"/>
+      <c r="BI4" s="89"/>
+      <c r="BJ4" s="89"/>
+      <c r="BK4" s="89"/>
+      <c r="BL4" s="89"/>
+      <c r="BM4" s="90"/>
     </row>
     <row r="5" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="91"/>
-      <c r="C5" s="91"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="91"/>
-      <c r="F5" s="91"/>
-      <c r="G5" s="91"/>
-      <c r="H5" s="91"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="94"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="94"/>
+      <c r="F5" s="94"/>
+      <c r="G5" s="94"/>
+      <c r="H5" s="94"/>
       <c r="J5" s="70">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -2846,7 +2861,7 @@
       </c>
       <c r="D9" s="40"/>
       <c r="E9" s="17">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="F9" s="56">
         <f>F23+1</f>
@@ -3325,7 +3340,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C15" s="38" t="s">
         <v>27</v>
@@ -3407,13 +3422,13 @@
     <row r="16" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
       <c r="B16" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="C16" s="38" t="s">
+      <c r="D16" s="38" t="s">
         <v>68</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>69</v>
       </c>
       <c r="E16" s="14">
         <v>0</v>
@@ -3487,13 +3502,13 @@
     <row r="17" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33"/>
       <c r="B17" s="46" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="38" t="s">
         <v>65</v>
-      </c>
-      <c r="C17" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="D17" s="38" t="s">
-        <v>66</v>
       </c>
       <c r="E17" s="14">
         <v>0.2</v>
@@ -3564,10 +3579,10 @@
     <row r="18" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33"/>
       <c r="B18" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="38" t="s">
         <v>61</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>62</v>
       </c>
       <c r="D18" s="38"/>
       <c r="E18" s="14">
@@ -4052,7 +4067,7 @@
         <v>11</v>
       </c>
       <c r="B24" s="80" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C24" s="81"/>
       <c r="D24" s="81"/>
@@ -4124,19 +4139,23 @@
     <row r="25" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="32"/>
       <c r="B25" s="76" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="77" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="77"/>
-      <c r="D25" s="77"/>
+      <c r="D25" s="77" t="s">
+        <v>76</v>
+      </c>
       <c r="E25" s="78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="79">
-        <v>45851</v>
+        <v>45858</v>
       </c>
       <c r="G25" s="79">
         <f>F25+4</f>
-        <v>45855</v>
+        <v>45862</v>
       </c>
       <c r="H25" s="11"/>
       <c r="I25" s="11">
@@ -4203,14 +4222,16 @@
     <row r="26" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32"/>
       <c r="B26" s="76" t="s">
-        <v>72</v>
-      </c>
-      <c r="C26" s="77"/>
+        <v>71</v>
+      </c>
+      <c r="C26" s="77" t="s">
+        <v>77</v>
+      </c>
       <c r="D26" s="77" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E26" s="78">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F26" s="79">
         <v>45829</v>
@@ -4283,13 +4304,13 @@
     <row r="27" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32"/>
       <c r="B27" s="76" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" s="77" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" s="77" t="s">
         <v>74</v>
-      </c>
-      <c r="D27" s="77" t="s">
-        <v>76</v>
       </c>
       <c r="E27" s="78">
         <v>1</v>
@@ -4367,20 +4388,22 @@
     <row r="28" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32"/>
       <c r="B28" s="76" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="C28" s="77" t="s">
         <v>45</v>
       </c>
-      <c r="D28" s="77"/>
+      <c r="D28" s="77" t="s">
+        <v>80</v>
+      </c>
       <c r="E28" s="78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="79">
-        <v>45829</v>
+        <v>45858</v>
       </c>
       <c r="G28" s="79">
-        <v>45829</v>
+        <v>45858</v>
       </c>
       <c r="H28" s="11"/>
       <c r="I28" s="11">
@@ -4526,7 +4549,9 @@
       <c r="C30" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="42"/>
+      <c r="D30" s="42" t="s">
+        <v>81</v>
+      </c>
       <c r="E30" s="20">
         <v>0.5</v>
       </c>
@@ -4608,22 +4633,22 @@
       <c r="C31" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="D31" s="42"/>
+      <c r="D31" s="42" t="s">
+        <v>75</v>
+      </c>
       <c r="E31" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" s="59">
-        <f>G30+1</f>
-        <v>45843</v>
+        <v>45858</v>
       </c>
       <c r="G31" s="59">
-        <f>F31+4</f>
-        <v>45847</v>
+        <v>45858</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="11">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
@@ -4773,7 +4798,7 @@
         <v>27</v>
       </c>
       <c r="D33" s="42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E33" s="20">
         <v>1</v>
@@ -4854,7 +4879,7 @@
         <v>47</v>
       </c>
       <c r="C34" s="74" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D34" s="43"/>
       <c r="E34" s="22"/>
@@ -4928,10 +4953,10 @@
         <v>49</v>
       </c>
       <c r="C35" s="44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D35" s="44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" s="23">
         <v>1</v>
@@ -5007,10 +5032,10 @@
     <row r="36" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="32"/>
       <c r="B36" s="49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C36" s="44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D36" s="44"/>
       <c r="E36" s="23">
@@ -5087,7 +5112,7 @@
         <v>48</v>
       </c>
       <c r="C37" s="44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D37" s="44"/>
       <c r="E37" s="23">
@@ -5167,7 +5192,7 @@
         <v>50</v>
       </c>
       <c r="C38" s="44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D38" s="44"/>
       <c r="E38" s="23">
@@ -5247,7 +5272,7 @@
         <v>51</v>
       </c>
       <c r="C39" s="44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D39" s="44"/>
       <c r="E39" s="23">
@@ -5324,13 +5349,13 @@
     <row r="40" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32"/>
       <c r="B40" s="49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C40" s="44" t="s">
         <v>27</v>
       </c>
       <c r="D40" s="44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E40" s="23">
         <v>0</v>
@@ -5599,7 +5624,7 @@
       <formula>AND(Fecha_final&gt;=J$5,Fecha_incio&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Mostrar semana" prompt="Al cambiar este número, se desplazará la vista del diagrama de Gantt." sqref="F4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Actualizacion Diseño BD IMPORTANTE, creacion permisos usuarios, validacion del funcionamiento, crea Profesor,Añade campos ManageTeacher,Cambia logica de la pagina, se valido el CRUD para profesor, Admins
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206DFF13-FCB9-4645-8756-AA2C46E93FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2CE3F5-3EA5-4536-902D-46457A749DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="86">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -381,6 +381,18 @@
   </si>
   <si>
     <t>Permitir dejar campos vacios</t>
+  </si>
+  <si>
+    <t>Juddy</t>
+  </si>
+  <si>
+    <t>Asignacion de Permisos</t>
+  </si>
+  <si>
+    <t>Crear en SQL la logica de otorgar permisos</t>
+  </si>
+  <si>
+    <t>Esto es X Usuario</t>
   </si>
 </sst>
 </file>
@@ -1413,6 +1425,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1425,13 +1444,6 @@
     <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="55">
     <cellStyle name="20% - Énfasis1" xfId="31" builtinId="30" customBuiltin="1"/>
@@ -2068,7 +2080,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BM45"/>
+  <dimension ref="A1:BM46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="32" customWidth="1"/>
@@ -2119,120 +2131,120 @@
       <c r="B3" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="92" t="s">
+      <c r="C3" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="92"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="91">
+      <c r="D3" s="88"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="94">
         <v>45822</v>
       </c>
-      <c r="G3" s="91"/>
+      <c r="G3" s="94"/>
     </row>
     <row r="4" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="92" t="s">
+      <c r="C4" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="92"/>
-      <c r="E4" s="93"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="89"/>
       <c r="F4" s="7">
         <v>1</v>
       </c>
-      <c r="J4" s="88">
+      <c r="J4" s="91">
         <f>J5</f>
         <v>45817</v>
       </c>
-      <c r="K4" s="89"/>
-      <c r="L4" s="89"/>
-      <c r="M4" s="89"/>
-      <c r="N4" s="89"/>
-      <c r="O4" s="89"/>
-      <c r="P4" s="90"/>
-      <c r="Q4" s="88">
+      <c r="K4" s="92"/>
+      <c r="L4" s="92"/>
+      <c r="M4" s="92"/>
+      <c r="N4" s="92"/>
+      <c r="O4" s="92"/>
+      <c r="P4" s="93"/>
+      <c r="Q4" s="91">
         <f>Q5</f>
         <v>45824</v>
       </c>
-      <c r="R4" s="89"/>
-      <c r="S4" s="89"/>
-      <c r="T4" s="89"/>
-      <c r="U4" s="89"/>
-      <c r="V4" s="89"/>
-      <c r="W4" s="90"/>
-      <c r="X4" s="88">
+      <c r="R4" s="92"/>
+      <c r="S4" s="92"/>
+      <c r="T4" s="92"/>
+      <c r="U4" s="92"/>
+      <c r="V4" s="92"/>
+      <c r="W4" s="93"/>
+      <c r="X4" s="91">
         <f>X5</f>
         <v>45831</v>
       </c>
-      <c r="Y4" s="89"/>
-      <c r="Z4" s="89"/>
-      <c r="AA4" s="89"/>
-      <c r="AB4" s="89"/>
-      <c r="AC4" s="89"/>
-      <c r="AD4" s="90"/>
-      <c r="AE4" s="88">
+      <c r="Y4" s="92"/>
+      <c r="Z4" s="92"/>
+      <c r="AA4" s="92"/>
+      <c r="AB4" s="92"/>
+      <c r="AC4" s="92"/>
+      <c r="AD4" s="93"/>
+      <c r="AE4" s="91">
         <f>AE5</f>
         <v>45838</v>
       </c>
-      <c r="AF4" s="89"/>
-      <c r="AG4" s="89"/>
-      <c r="AH4" s="89"/>
-      <c r="AI4" s="89"/>
-      <c r="AJ4" s="89"/>
-      <c r="AK4" s="90"/>
-      <c r="AL4" s="88">
+      <c r="AF4" s="92"/>
+      <c r="AG4" s="92"/>
+      <c r="AH4" s="92"/>
+      <c r="AI4" s="92"/>
+      <c r="AJ4" s="92"/>
+      <c r="AK4" s="93"/>
+      <c r="AL4" s="91">
         <f>AL5</f>
         <v>45845</v>
       </c>
-      <c r="AM4" s="89"/>
-      <c r="AN4" s="89"/>
-      <c r="AO4" s="89"/>
-      <c r="AP4" s="89"/>
-      <c r="AQ4" s="89"/>
-      <c r="AR4" s="90"/>
-      <c r="AS4" s="88">
+      <c r="AM4" s="92"/>
+      <c r="AN4" s="92"/>
+      <c r="AO4" s="92"/>
+      <c r="AP4" s="92"/>
+      <c r="AQ4" s="92"/>
+      <c r="AR4" s="93"/>
+      <c r="AS4" s="91">
         <f>AS5</f>
         <v>45852</v>
       </c>
-      <c r="AT4" s="89"/>
-      <c r="AU4" s="89"/>
-      <c r="AV4" s="89"/>
-      <c r="AW4" s="89"/>
-      <c r="AX4" s="89"/>
-      <c r="AY4" s="90"/>
-      <c r="AZ4" s="88">
+      <c r="AT4" s="92"/>
+      <c r="AU4" s="92"/>
+      <c r="AV4" s="92"/>
+      <c r="AW4" s="92"/>
+      <c r="AX4" s="92"/>
+      <c r="AY4" s="93"/>
+      <c r="AZ4" s="91">
         <f>AZ5</f>
         <v>45859</v>
       </c>
-      <c r="BA4" s="89"/>
-      <c r="BB4" s="89"/>
-      <c r="BC4" s="89"/>
-      <c r="BD4" s="89"/>
-      <c r="BE4" s="89"/>
-      <c r="BF4" s="90"/>
-      <c r="BG4" s="88">
+      <c r="BA4" s="92"/>
+      <c r="BB4" s="92"/>
+      <c r="BC4" s="92"/>
+      <c r="BD4" s="92"/>
+      <c r="BE4" s="92"/>
+      <c r="BF4" s="93"/>
+      <c r="BG4" s="91">
         <f>BG5</f>
         <v>45866</v>
       </c>
-      <c r="BH4" s="89"/>
-      <c r="BI4" s="89"/>
-      <c r="BJ4" s="89"/>
-      <c r="BK4" s="89"/>
-      <c r="BL4" s="89"/>
-      <c r="BM4" s="90"/>
+      <c r="BH4" s="92"/>
+      <c r="BI4" s="92"/>
+      <c r="BJ4" s="92"/>
+      <c r="BK4" s="92"/>
+      <c r="BL4" s="92"/>
+      <c r="BM4" s="93"/>
     </row>
     <row r="5" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="94"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="94"/>
-      <c r="F5" s="94"/>
-      <c r="G5" s="94"/>
-      <c r="H5" s="94"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
       <c r="J5" s="70">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -2791,7 +2803,7 @@
       <c r="G8" s="55"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11" t="str">
-        <f t="shared" ref="I8:I42" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
+        <f t="shared" ref="I8:I43" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
         <v/>
       </c>
       <c r="J8" s="28"/>
@@ -2857,14 +2869,14 @@
         <v>33</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="D9" s="40"/>
       <c r="E9" s="17">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="F9" s="56">
-        <f>F23+1</f>
+        <f>F24+1</f>
         <v>45830</v>
       </c>
       <c r="G9" s="56">
@@ -3422,24 +3434,17 @@
     <row r="16" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
       <c r="B16" s="46" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="14">
-        <v>0</v>
-      </c>
-      <c r="F16" s="53">
-        <v>45851</v>
-      </c>
-      <c r="G16" s="53">
-        <f>F16+6</f>
-        <v>45857</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="E16" s="14"/>
+      <c r="F16" s="53"/>
+      <c r="G16" s="53"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
       <c r="J16" s="28"/>
@@ -3502,21 +3507,24 @@
     <row r="17" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33"/>
       <c r="B17" s="46" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E17" s="14">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F17" s="53">
-        <v>45837</v>
-      </c>
-      <c r="G17" s="53"/>
+        <v>45851</v>
+      </c>
+      <c r="G17" s="53">
+        <f>F17+6</f>
+        <v>45857</v>
+      </c>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
       <c r="J17" s="28"/>
@@ -3579,21 +3587,21 @@
     <row r="18" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33"/>
       <c r="B18" s="46" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C18" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" s="38"/>
+        <v>63</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>65</v>
+      </c>
       <c r="E18" s="14">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="F18" s="53">
         <v>45837</v>
       </c>
-      <c r="G18" s="53">
-        <v>45837</v>
-      </c>
+      <c r="G18" s="53"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
       <c r="J18" s="28"/>
@@ -3654,32 +3662,25 @@
       <c r="BM18" s="28"/>
     </row>
     <row r="19" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="33" t="s">
-        <v>9</v>
-      </c>
+      <c r="A19" s="33"/>
       <c r="B19" s="46" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C19" s="38" t="s">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="D19" s="38"/>
       <c r="E19" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="53">
-        <f>G15</f>
-        <v>45828</v>
+        <v>45837</v>
       </c>
       <c r="G19" s="53">
-        <f>F19+2</f>
-        <v>45830</v>
+        <v>45837</v>
       </c>
       <c r="H19" s="11"/>
-      <c r="I19" s="11">
-        <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
+      <c r="I19" s="11"/>
       <c r="J19" s="28"/>
       <c r="K19" s="28"/>
       <c r="L19" s="28"/>
@@ -3692,8 +3693,8 @@
       <c r="S19" s="28"/>
       <c r="T19" s="28"/>
       <c r="U19" s="28"/>
-      <c r="V19" s="29"/>
-      <c r="W19" s="29"/>
+      <c r="V19" s="28"/>
+      <c r="W19" s="28"/>
       <c r="X19" s="28"/>
       <c r="Y19" s="28"/>
       <c r="Z19" s="28"/>
@@ -3738,9 +3739,11 @@
       <c r="BM19" s="28"/>
     </row>
     <row r="20" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="32"/>
+      <c r="A20" s="33" t="s">
+        <v>9</v>
+      </c>
       <c r="B20" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" s="38" t="s">
         <v>27</v>
@@ -3750,17 +3753,17 @@
         <v>0</v>
       </c>
       <c r="F20" s="53">
-        <f>G19</f>
+        <f>G15</f>
+        <v>45828</v>
+      </c>
+      <c r="G20" s="53">
+        <f>F20+2</f>
         <v>45830</v>
-      </c>
-      <c r="G20" s="53">
-        <f>F20+4</f>
-        <v>45834</v>
       </c>
       <c r="H20" s="11"/>
       <c r="I20" s="11">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J20" s="28"/>
       <c r="K20" s="28"/>
@@ -3774,8 +3777,8 @@
       <c r="S20" s="28"/>
       <c r="T20" s="28"/>
       <c r="U20" s="28"/>
-      <c r="V20" s="28"/>
-      <c r="W20" s="28"/>
+      <c r="V20" s="29"/>
+      <c r="W20" s="29"/>
       <c r="X20" s="28"/>
       <c r="Y20" s="28"/>
       <c r="Z20" s="28"/>
@@ -3789,7 +3792,7 @@
       <c r="AH20" s="28"/>
       <c r="AI20" s="28"/>
       <c r="AJ20" s="28"/>
-      <c r="AK20" s="73"/>
+      <c r="AK20" s="28"/>
       <c r="AL20" s="28"/>
       <c r="AM20" s="28"/>
       <c r="AN20" s="28"/>
@@ -3822,25 +3825,28 @@
     <row r="21" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="32"/>
       <c r="B21" s="46" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C21" s="38" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D21" s="38"/>
       <c r="E21" s="14">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F21" s="53">
         <f>G20</f>
-        <v>45834</v>
+        <v>45830</v>
       </c>
       <c r="G21" s="53">
         <f>F21+4</f>
-        <v>45838</v>
+        <v>45834</v>
       </c>
       <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
+      <c r="I21" s="11">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
       <c r="J21" s="28"/>
       <c r="K21" s="28"/>
       <c r="L21" s="28"/>
@@ -3901,28 +3907,25 @@
     <row r="22" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="32"/>
       <c r="B22" s="46" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D22" s="38"/>
       <c r="E22" s="14">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F22" s="53">
-        <f>G20</f>
+        <f>G21</f>
         <v>45834</v>
       </c>
       <c r="G22" s="53">
-        <f>F22+5</f>
-        <v>45839</v>
+        <f>F22+4</f>
+        <v>45838</v>
       </c>
       <c r="H22" s="11"/>
-      <c r="I22" s="11">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
+      <c r="I22" s="11"/>
       <c r="J22" s="28"/>
       <c r="K22" s="28"/>
       <c r="L22" s="28"/>
@@ -3939,7 +3942,7 @@
       <c r="W22" s="28"/>
       <c r="X22" s="28"/>
       <c r="Y22" s="28"/>
-      <c r="Z22" s="29"/>
+      <c r="Z22" s="28"/>
       <c r="AA22" s="28"/>
       <c r="AB22" s="28"/>
       <c r="AC22" s="28"/>
@@ -3950,7 +3953,7 @@
       <c r="AH22" s="28"/>
       <c r="AI22" s="28"/>
       <c r="AJ22" s="28"/>
-      <c r="AK22" s="28"/>
+      <c r="AK22" s="73"/>
       <c r="AL22" s="28"/>
       <c r="AM22" s="28"/>
       <c r="AN22" s="28"/>
@@ -3983,7 +3986,7 @@
     <row r="23" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="32"/>
       <c r="B23" s="46" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C23" s="38" t="s">
         <v>27</v>
@@ -3993,17 +3996,17 @@
         <v>0</v>
       </c>
       <c r="F23" s="53">
-        <f>F19+1</f>
-        <v>45829</v>
+        <f>G21</f>
+        <v>45834</v>
       </c>
       <c r="G23" s="53">
-        <f>F23+2</f>
-        <v>45831</v>
+        <f>F23+5</f>
+        <v>45839</v>
       </c>
       <c r="H23" s="11"/>
       <c r="I23" s="11">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J23" s="28"/>
       <c r="K23" s="28"/>
@@ -4021,7 +4024,7 @@
       <c r="W23" s="28"/>
       <c r="X23" s="28"/>
       <c r="Y23" s="28"/>
-      <c r="Z23" s="28"/>
+      <c r="Z23" s="29"/>
       <c r="AA23" s="28"/>
       <c r="AB23" s="28"/>
       <c r="AC23" s="28"/>
@@ -4063,21 +4066,29 @@
       <c r="BM23" s="28"/>
     </row>
     <row r="24" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B24" s="80" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" s="81"/>
-      <c r="D24" s="81"/>
-      <c r="E24" s="82"/>
-      <c r="F24" s="83"/>
-      <c r="G24" s="84"/>
+      <c r="A24" s="32"/>
+      <c r="B24" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="38"/>
+      <c r="E24" s="14">
+        <v>0</v>
+      </c>
+      <c r="F24" s="53">
+        <f>F20+1</f>
+        <v>45829</v>
+      </c>
+      <c r="G24" s="53">
+        <f>F24+2</f>
+        <v>45831</v>
+      </c>
       <c r="H24" s="11"/>
-      <c r="I24" s="11" t="str">
+      <c r="I24" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="J24" s="28"/>
       <c r="K24" s="28"/>
@@ -4137,30 +4148,21 @@
       <c r="BM24" s="28"/>
     </row>
     <row r="25" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="32"/>
-      <c r="B25" s="76" t="s">
-        <v>72</v>
-      </c>
-      <c r="C25" s="77" t="s">
-        <v>73</v>
-      </c>
-      <c r="D25" s="77" t="s">
-        <v>76</v>
-      </c>
-      <c r="E25" s="78">
-        <v>1</v>
-      </c>
-      <c r="F25" s="79">
-        <v>45858</v>
-      </c>
-      <c r="G25" s="79">
-        <f>F25+4</f>
-        <v>45862</v>
-      </c>
+      <c r="A25" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="80" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="81"/>
+      <c r="D25" s="81"/>
+      <c r="E25" s="82"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="84"/>
       <c r="H25" s="11"/>
-      <c r="I25" s="11">
+      <c r="I25" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v/>
       </c>
       <c r="J25" s="28"/>
       <c r="K25" s="28"/>
@@ -4222,27 +4224,28 @@
     <row r="26" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32"/>
       <c r="B26" s="76" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C26" s="77" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D26" s="77" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E26" s="78">
         <v>1</v>
       </c>
       <c r="F26" s="79">
-        <v>45829</v>
+        <v>45858</v>
       </c>
       <c r="G26" s="79">
-        <v>45829</v>
+        <f>F26+4</f>
+        <v>45862</v>
       </c>
       <c r="H26" s="11"/>
       <c r="I26" s="11">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J26" s="28"/>
       <c r="K26" s="28"/>
@@ -4304,29 +4307,27 @@
     <row r="27" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32"/>
       <c r="B27" s="76" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C27" s="77" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D27" s="77" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E27" s="78">
         <v>1</v>
       </c>
       <c r="F27" s="79">
-        <f>G26+1</f>
-        <v>45830</v>
+        <v>45829</v>
       </c>
       <c r="G27" s="79">
-        <f>F27+4</f>
-        <v>45834</v>
+        <v>45829</v>
       </c>
       <c r="H27" s="11"/>
       <c r="I27" s="11">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J27" s="28"/>
       <c r="K27" s="28"/>
@@ -4388,27 +4389,29 @@
     <row r="28" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32"/>
       <c r="B28" s="76" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C28" s="77" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="D28" s="77" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E28" s="78">
         <v>1</v>
       </c>
       <c r="F28" s="79">
-        <v>45858</v>
+        <f>G27+1</f>
+        <v>45830</v>
       </c>
       <c r="G28" s="79">
-        <v>45858</v>
+        <f>F28+4</f>
+        <v>45834</v>
       </c>
       <c r="H28" s="11"/>
       <c r="I28" s="11">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J28" s="28"/>
       <c r="K28" s="28"/>
@@ -4468,21 +4471,29 @@
       <c r="BM28" s="28"/>
     </row>
     <row r="29" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C29" s="41"/>
-      <c r="D29" s="41"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="58"/>
+      <c r="A29" s="32"/>
+      <c r="B29" s="76" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="E29" s="78">
+        <v>1</v>
+      </c>
+      <c r="F29" s="79">
+        <v>45858</v>
+      </c>
+      <c r="G29" s="79">
+        <v>45858</v>
+      </c>
       <c r="H29" s="11"/>
-      <c r="I29" s="11" t="str">
+      <c r="I29" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J29" s="28"/>
       <c r="K29" s="28"/>
@@ -4542,31 +4553,21 @@
       <c r="BM29" s="28"/>
     </row>
     <row r="30" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="32"/>
-      <c r="B30" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="42" t="s">
-        <v>39</v>
-      </c>
-      <c r="D30" s="42" t="s">
-        <v>81</v>
-      </c>
-      <c r="E30" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="F30" s="59">
-        <f>F15+15</f>
-        <v>45837</v>
-      </c>
-      <c r="G30" s="59">
-        <f>F30+5</f>
-        <v>45842</v>
-      </c>
+      <c r="A30" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="57"/>
+      <c r="G30" s="58"/>
       <c r="H30" s="11"/>
-      <c r="I30" s="11">
+      <c r="I30" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v/>
       </c>
       <c r="J30" s="28"/>
       <c r="K30" s="28"/>
@@ -4628,27 +4629,29 @@
     <row r="31" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32"/>
       <c r="B31" s="48" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C31" s="42" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D31" s="42" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E31" s="20">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F31" s="59">
-        <v>45858</v>
+        <f>F15+15</f>
+        <v>45837</v>
       </c>
       <c r="G31" s="59">
-        <v>45858</v>
+        <f>F31+5</f>
+        <v>45842</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="11">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
@@ -4710,22 +4713,22 @@
     <row r="32" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32"/>
       <c r="B32" s="48" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C32" s="42" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D32" s="42" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="E32" s="20">
         <v>1</v>
       </c>
       <c r="F32" s="59">
-        <v>45829</v>
+        <v>45858</v>
       </c>
       <c r="G32" s="59">
-        <v>45829</v>
+        <v>45858</v>
       </c>
       <c r="H32" s="11"/>
       <c r="I32" s="11">
@@ -4792,27 +4795,27 @@
     <row r="33" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="32"/>
       <c r="B33" s="48" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="C33" s="42" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D33" s="42" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="E33" s="20">
         <v>1</v>
       </c>
       <c r="F33" s="59">
-        <v>45837</v>
+        <v>45829</v>
       </c>
       <c r="G33" s="59">
-        <v>45851</v>
+        <v>45829</v>
       </c>
       <c r="H33" s="11"/>
       <c r="I33" s="11">
         <f t="shared" si="6"/>
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="J33" s="28"/>
       <c r="K33" s="28"/>
@@ -4872,23 +4875,29 @@
       <c r="BM33" s="28"/>
     </row>
     <row r="34" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="74" t="s">
-        <v>55</v>
-      </c>
-      <c r="D34" s="43"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="60"/>
-      <c r="G34" s="61"/>
+      <c r="A34" s="32"/>
+      <c r="B34" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D34" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="E34" s="20">
+        <v>1</v>
+      </c>
+      <c r="F34" s="59">
+        <v>45837</v>
+      </c>
+      <c r="G34" s="59">
+        <v>45851</v>
+      </c>
       <c r="H34" s="11"/>
-      <c r="I34" s="11" t="str">
+      <c r="I34" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>15</v>
       </c>
       <c r="J34" s="28"/>
       <c r="K34" s="28"/>
@@ -4948,29 +4957,23 @@
       <c r="BM34" s="28"/>
     </row>
     <row r="35" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="32"/>
-      <c r="B35" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="C35" s="44" t="s">
-        <v>54</v>
-      </c>
-      <c r="D35" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="E35" s="23">
-        <v>1</v>
-      </c>
-      <c r="F35" s="62">
-        <v>45837</v>
-      </c>
-      <c r="G35" s="62">
-        <v>45837</v>
-      </c>
+      <c r="A35" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" s="74" t="s">
+        <v>55</v>
+      </c>
+      <c r="D35" s="43"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="60"/>
+      <c r="G35" s="61"/>
       <c r="H35" s="11"/>
-      <c r="I35" s="11">
+      <c r="I35" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
       <c r="J35" s="28"/>
       <c r="K35" s="28"/>
@@ -5032,12 +5035,14 @@
     <row r="36" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="32"/>
       <c r="B36" s="49" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C36" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="D36" s="44"/>
+      <c r="D36" s="44" t="s">
+        <v>58</v>
+      </c>
       <c r="E36" s="23">
         <v>1</v>
       </c>
@@ -5048,7 +5053,10 @@
         <v>45837</v>
       </c>
       <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
+      <c r="I36" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
       <c r="J36" s="28"/>
       <c r="K36" s="28"/>
       <c r="L36" s="28"/>
@@ -5109,7 +5117,7 @@
     <row r="37" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="32"/>
       <c r="B37" s="49" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C37" s="44" t="s">
         <v>54</v>
@@ -5125,10 +5133,7 @@
         <v>45837</v>
       </c>
       <c r="H37" s="11"/>
-      <c r="I37" s="11">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
+      <c r="I37" s="11"/>
       <c r="J37" s="28"/>
       <c r="K37" s="28"/>
       <c r="L37" s="28"/>
@@ -5189,7 +5194,7 @@
     <row r="38" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="32"/>
       <c r="B38" s="49" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C38" s="44" t="s">
         <v>54</v>
@@ -5269,7 +5274,7 @@
     <row r="39" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="32"/>
       <c r="B39" s="49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C39" s="44" t="s">
         <v>54</v>
@@ -5349,23 +5354,25 @@
     <row r="40" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32"/>
       <c r="B40" s="49" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C40" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="44" t="s">
-        <v>59</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="D40" s="44"/>
       <c r="E40" s="23">
-        <v>0</v>
-      </c>
-      <c r="F40" s="62"/>
-      <c r="G40" s="62"/>
+        <v>1</v>
+      </c>
+      <c r="F40" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G40" s="62">
+        <v>45837</v>
+      </c>
       <c r="H40" s="11"/>
-      <c r="I40" s="11" t="str">
+      <c r="I40" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J40" s="28"/>
       <c r="K40" s="28"/>
@@ -5425,15 +5432,21 @@
       <c r="BM40" s="28"/>
     </row>
     <row r="41" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B41" s="50"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="63"/>
-      <c r="G41" s="63"/>
+      <c r="A41" s="32"/>
+      <c r="B41" s="49" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D41" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="E41" s="23">
+        <v>0</v>
+      </c>
+      <c r="F41" s="62"/>
+      <c r="G41" s="62"/>
       <c r="H41" s="11"/>
       <c r="I41" s="11" t="str">
         <f t="shared" si="6"/>
@@ -5497,98 +5510,165 @@
       <c r="BM41" s="28"/>
     </row>
     <row r="42" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B42" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C42" s="25"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="64"/>
-      <c r="G42" s="65"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="27" t="str">
+      <c r="A42" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="50"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="63"/>
+      <c r="G42" s="63"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="J42" s="30"/>
-      <c r="K42" s="30"/>
-      <c r="L42" s="30"/>
-      <c r="M42" s="30"/>
-      <c r="N42" s="30"/>
-      <c r="O42" s="30"/>
-      <c r="P42" s="30"/>
-      <c r="Q42" s="30"/>
-      <c r="R42" s="30"/>
-      <c r="S42" s="30"/>
-      <c r="T42" s="30"/>
-      <c r="U42" s="30"/>
-      <c r="V42" s="30"/>
-      <c r="W42" s="30"/>
-      <c r="X42" s="30"/>
-      <c r="Y42" s="30"/>
-      <c r="Z42" s="30"/>
-      <c r="AA42" s="30"/>
-      <c r="AB42" s="30"/>
-      <c r="AC42" s="30"/>
-      <c r="AD42" s="30"/>
-      <c r="AE42" s="30"/>
-      <c r="AF42" s="30"/>
-      <c r="AG42" s="30"/>
-      <c r="AH42" s="30"/>
-      <c r="AI42" s="30"/>
-      <c r="AJ42" s="30"/>
-      <c r="AK42" s="30"/>
-      <c r="AL42" s="30"/>
-      <c r="AM42" s="30"/>
-      <c r="AN42" s="30"/>
-      <c r="AO42" s="30"/>
-      <c r="AP42" s="30"/>
-      <c r="AQ42" s="30"/>
-      <c r="AR42" s="30"/>
-      <c r="AS42" s="30"/>
-      <c r="AT42" s="30"/>
-      <c r="AU42" s="30"/>
-      <c r="AV42" s="30"/>
-      <c r="AW42" s="30"/>
-      <c r="AX42" s="30"/>
-      <c r="AY42" s="30"/>
-      <c r="AZ42" s="30"/>
-      <c r="BA42" s="30"/>
-      <c r="BB42" s="30"/>
-      <c r="BC42" s="30"/>
-      <c r="BD42" s="30"/>
-      <c r="BE42" s="30"/>
-      <c r="BF42" s="30"/>
-      <c r="BG42" s="30"/>
-      <c r="BH42" s="30"/>
-      <c r="BI42" s="30"/>
-      <c r="BJ42" s="30"/>
-      <c r="BK42" s="30"/>
-      <c r="BL42" s="30"/>
-      <c r="BM42" s="30"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="28"/>
+      <c r="L42" s="28"/>
+      <c r="M42" s="28"/>
+      <c r="N42" s="28"/>
+      <c r="O42" s="28"/>
+      <c r="P42" s="28"/>
+      <c r="Q42" s="28"/>
+      <c r="R42" s="28"/>
+      <c r="S42" s="28"/>
+      <c r="T42" s="28"/>
+      <c r="U42" s="28"/>
+      <c r="V42" s="28"/>
+      <c r="W42" s="28"/>
+      <c r="X42" s="28"/>
+      <c r="Y42" s="28"/>
+      <c r="Z42" s="28"/>
+      <c r="AA42" s="28"/>
+      <c r="AB42" s="28"/>
+      <c r="AC42" s="28"/>
+      <c r="AD42" s="28"/>
+      <c r="AE42" s="28"/>
+      <c r="AF42" s="28"/>
+      <c r="AG42" s="28"/>
+      <c r="AH42" s="28"/>
+      <c r="AI42" s="28"/>
+      <c r="AJ42" s="28"/>
+      <c r="AK42" s="28"/>
+      <c r="AL42" s="28"/>
+      <c r="AM42" s="28"/>
+      <c r="AN42" s="28"/>
+      <c r="AO42" s="28"/>
+      <c r="AP42" s="28"/>
+      <c r="AQ42" s="28"/>
+      <c r="AR42" s="28"/>
+      <c r="AS42" s="28"/>
+      <c r="AT42" s="28"/>
+      <c r="AU42" s="28"/>
+      <c r="AV42" s="28"/>
+      <c r="AW42" s="28"/>
+      <c r="AX42" s="28"/>
+      <c r="AY42" s="28"/>
+      <c r="AZ42" s="28"/>
+      <c r="BA42" s="28"/>
+      <c r="BB42" s="28"/>
+      <c r="BC42" s="28"/>
+      <c r="BD42" s="28"/>
+      <c r="BE42" s="28"/>
+      <c r="BF42" s="28"/>
+      <c r="BG42" s="28"/>
+      <c r="BH42" s="28"/>
+      <c r="BI42" s="28"/>
+      <c r="BJ42" s="28"/>
+      <c r="BK42" s="28"/>
+      <c r="BL42" s="28"/>
+      <c r="BM42" s="28"/>
     </row>
-    <row r="43" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H43" s="6"/>
+    <row r="43" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="25"/>
+      <c r="D43" s="25"/>
+      <c r="E43" s="26"/>
+      <c r="F43" s="64"/>
+      <c r="G43" s="65"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J43" s="30"/>
+      <c r="K43" s="30"/>
+      <c r="L43" s="30"/>
+      <c r="M43" s="30"/>
+      <c r="N43" s="30"/>
+      <c r="O43" s="30"/>
+      <c r="P43" s="30"/>
+      <c r="Q43" s="30"/>
+      <c r="R43" s="30"/>
+      <c r="S43" s="30"/>
+      <c r="T43" s="30"/>
+      <c r="U43" s="30"/>
+      <c r="V43" s="30"/>
+      <c r="W43" s="30"/>
+      <c r="X43" s="30"/>
+      <c r="Y43" s="30"/>
+      <c r="Z43" s="30"/>
+      <c r="AA43" s="30"/>
+      <c r="AB43" s="30"/>
+      <c r="AC43" s="30"/>
+      <c r="AD43" s="30"/>
+      <c r="AE43" s="30"/>
+      <c r="AF43" s="30"/>
+      <c r="AG43" s="30"/>
+      <c r="AH43" s="30"/>
+      <c r="AI43" s="30"/>
+      <c r="AJ43" s="30"/>
+      <c r="AK43" s="30"/>
+      <c r="AL43" s="30"/>
+      <c r="AM43" s="30"/>
+      <c r="AN43" s="30"/>
+      <c r="AO43" s="30"/>
+      <c r="AP43" s="30"/>
+      <c r="AQ43" s="30"/>
+      <c r="AR43" s="30"/>
+      <c r="AS43" s="30"/>
+      <c r="AT43" s="30"/>
+      <c r="AU43" s="30"/>
+      <c r="AV43" s="30"/>
+      <c r="AW43" s="30"/>
+      <c r="AX43" s="30"/>
+      <c r="AY43" s="30"/>
+      <c r="AZ43" s="30"/>
+      <c r="BA43" s="30"/>
+      <c r="BB43" s="30"/>
+      <c r="BC43" s="30"/>
+      <c r="BD43" s="30"/>
+      <c r="BE43" s="30"/>
+      <c r="BF43" s="30"/>
+      <c r="BG43" s="30"/>
+      <c r="BH43" s="30"/>
+      <c r="BI43" s="30"/>
+      <c r="BJ43" s="30"/>
+      <c r="BK43" s="30"/>
+      <c r="BL43" s="30"/>
+      <c r="BM43" s="30"/>
     </row>
     <row r="44" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="G44" s="34"/>
+      <c r="H44" s="6"/>
     </row>
     <row r="45" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="G45" s="34"/>
+    </row>
+    <row r="46" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="AL4:AR4"/>
-    <mergeCell ref="AS4:AY4"/>
     <mergeCell ref="AZ4:BF4"/>
     <mergeCell ref="BG4:BM4"/>
     <mergeCell ref="F3:G3"/>
@@ -5596,8 +5676,13 @@
     <mergeCell ref="Q4:W4"/>
     <mergeCell ref="X4:AD4"/>
     <mergeCell ref="AE4:AK4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="AL4:AR4"/>
+    <mergeCell ref="AS4:AY4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E42">
+  <conditionalFormatting sqref="E7:E43">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5611,12 +5696,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:BM42">
+  <conditionalFormatting sqref="J5:BM43">
     <cfRule type="expression" dxfId="2" priority="33">
       <formula>AND(TODAY()&gt;=J$5,TODAY()&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:BM42">
+  <conditionalFormatting sqref="J7:BM43">
     <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(Fecha_incio&lt;=J$5,ROUNDDOWN((Fecha_final-Fecha_incio+1)*Progresos,0)+Fecha_incio-1&gt;=J$5)</formula>
     </cfRule>
@@ -5651,7 +5736,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E7:E42</xm:sqref>
+          <xm:sqref>E7:E43</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
CRUD completo corregido para Estudiante, consultas como insertar se hicieron con la funcion bind param,validacion de los datos, variables, optimizo tabs, space between line to line
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2CE3F5-3EA5-4536-902D-46457A749DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD45B30-003F-4114-B814-FC86A2E406CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,12 +76,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="89">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -257,9 +260,6 @@
     <t>forms/ManageStudent.php</t>
   </si>
   <si>
-    <t>Editar Datos Est</t>
-  </si>
-  <si>
     <t>Crear Datos Est</t>
   </si>
   <si>
@@ -362,9 +362,6 @@
     <t>Se crea bien y funciona trigger</t>
   </si>
   <si>
-    <t>ManageStudent.php</t>
-  </si>
-  <si>
     <t>Funciona Cambiar Archivo</t>
   </si>
   <si>
@@ -393,6 +390,21 @@
   </si>
   <si>
     <t>Esto es X Usuario</t>
+  </si>
+  <si>
+    <t>Leer Datos Est</t>
+  </si>
+  <si>
+    <t>Se leen correctamente</t>
+  </si>
+  <si>
+    <t>Posible Error Cambio imagen</t>
+  </si>
+  <si>
+    <t>StudentModel.php</t>
+  </si>
+  <si>
+    <t>Cuando modificamos cedula no cambia imagen</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1184,7 @@
     <xf numFmtId="0" fontId="9" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1424,6 +1436,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
       <alignment horizontal="right" indent="1"/>
@@ -2080,7 +2095,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BM46"/>
+  <dimension ref="A1:BM47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="32" customWidth="1"/>
@@ -2131,120 +2146,120 @@
       <c r="B3" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="88" t="s">
+      <c r="C3" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="88"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="94">
+      <c r="D3" s="89"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="95">
         <v>45822</v>
       </c>
-      <c r="G3" s="94"/>
+      <c r="G3" s="95"/>
     </row>
     <row r="4" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="88" t="s">
+      <c r="C4" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="88"/>
-      <c r="E4" s="89"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="90"/>
       <c r="F4" s="7">
         <v>1</v>
       </c>
-      <c r="J4" s="91">
+      <c r="J4" s="92">
         <f>J5</f>
         <v>45817</v>
       </c>
-      <c r="K4" s="92"/>
-      <c r="L4" s="92"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="93"/>
-      <c r="Q4" s="91">
+      <c r="K4" s="93"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="93"/>
+      <c r="O4" s="93"/>
+      <c r="P4" s="94"/>
+      <c r="Q4" s="92">
         <f>Q5</f>
         <v>45824</v>
       </c>
-      <c r="R4" s="92"/>
-      <c r="S4" s="92"/>
-      <c r="T4" s="92"/>
-      <c r="U4" s="92"/>
-      <c r="V4" s="92"/>
-      <c r="W4" s="93"/>
-      <c r="X4" s="91">
+      <c r="R4" s="93"/>
+      <c r="S4" s="93"/>
+      <c r="T4" s="93"/>
+      <c r="U4" s="93"/>
+      <c r="V4" s="93"/>
+      <c r="W4" s="94"/>
+      <c r="X4" s="92">
         <f>X5</f>
         <v>45831</v>
       </c>
-      <c r="Y4" s="92"/>
-      <c r="Z4" s="92"/>
-      <c r="AA4" s="92"/>
-      <c r="AB4" s="92"/>
-      <c r="AC4" s="92"/>
-      <c r="AD4" s="93"/>
-      <c r="AE4" s="91">
+      <c r="Y4" s="93"/>
+      <c r="Z4" s="93"/>
+      <c r="AA4" s="93"/>
+      <c r="AB4" s="93"/>
+      <c r="AC4" s="93"/>
+      <c r="AD4" s="94"/>
+      <c r="AE4" s="92">
         <f>AE5</f>
         <v>45838</v>
       </c>
-      <c r="AF4" s="92"/>
-      <c r="AG4" s="92"/>
-      <c r="AH4" s="92"/>
-      <c r="AI4" s="92"/>
-      <c r="AJ4" s="92"/>
-      <c r="AK4" s="93"/>
-      <c r="AL4" s="91">
+      <c r="AF4" s="93"/>
+      <c r="AG4" s="93"/>
+      <c r="AH4" s="93"/>
+      <c r="AI4" s="93"/>
+      <c r="AJ4" s="93"/>
+      <c r="AK4" s="94"/>
+      <c r="AL4" s="92">
         <f>AL5</f>
         <v>45845</v>
       </c>
-      <c r="AM4" s="92"/>
-      <c r="AN4" s="92"/>
-      <c r="AO4" s="92"/>
-      <c r="AP4" s="92"/>
-      <c r="AQ4" s="92"/>
-      <c r="AR4" s="93"/>
-      <c r="AS4" s="91">
+      <c r="AM4" s="93"/>
+      <c r="AN4" s="93"/>
+      <c r="AO4" s="93"/>
+      <c r="AP4" s="93"/>
+      <c r="AQ4" s="93"/>
+      <c r="AR4" s="94"/>
+      <c r="AS4" s="92">
         <f>AS5</f>
         <v>45852</v>
       </c>
-      <c r="AT4" s="92"/>
-      <c r="AU4" s="92"/>
-      <c r="AV4" s="92"/>
-      <c r="AW4" s="92"/>
-      <c r="AX4" s="92"/>
-      <c r="AY4" s="93"/>
-      <c r="AZ4" s="91">
+      <c r="AT4" s="93"/>
+      <c r="AU4" s="93"/>
+      <c r="AV4" s="93"/>
+      <c r="AW4" s="93"/>
+      <c r="AX4" s="93"/>
+      <c r="AY4" s="94"/>
+      <c r="AZ4" s="92">
         <f>AZ5</f>
         <v>45859</v>
       </c>
-      <c r="BA4" s="92"/>
-      <c r="BB4" s="92"/>
-      <c r="BC4" s="92"/>
-      <c r="BD4" s="92"/>
-      <c r="BE4" s="92"/>
-      <c r="BF4" s="93"/>
-      <c r="BG4" s="91">
+      <c r="BA4" s="93"/>
+      <c r="BB4" s="93"/>
+      <c r="BC4" s="93"/>
+      <c r="BD4" s="93"/>
+      <c r="BE4" s="93"/>
+      <c r="BF4" s="94"/>
+      <c r="BG4" s="92">
         <f>BG5</f>
         <v>45866</v>
       </c>
-      <c r="BH4" s="92"/>
-      <c r="BI4" s="92"/>
-      <c r="BJ4" s="92"/>
-      <c r="BK4" s="92"/>
-      <c r="BL4" s="92"/>
-      <c r="BM4" s="93"/>
+      <c r="BH4" s="93"/>
+      <c r="BI4" s="93"/>
+      <c r="BJ4" s="93"/>
+      <c r="BK4" s="93"/>
+      <c r="BL4" s="93"/>
+      <c r="BM4" s="94"/>
     </row>
     <row r="5" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="90"/>
-      <c r="C5" s="90"/>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="90"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="91"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
       <c r="J5" s="70">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -2478,10 +2493,10 @@
         <v>15</v>
       </c>
       <c r="C6" s="68" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="68" t="s">
         <v>42</v>
-      </c>
-      <c r="D6" s="68" t="s">
-        <v>43</v>
       </c>
       <c r="E6" s="68" t="s">
         <v>20</v>
@@ -2803,7 +2818,7 @@
       <c r="G8" s="55"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11" t="str">
-        <f t="shared" ref="I8:I43" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
+        <f t="shared" ref="I8:I44" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
         <v/>
       </c>
       <c r="J8" s="28"/>
@@ -2869,7 +2884,7 @@
         <v>33</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D9" s="40"/>
       <c r="E9" s="17">
@@ -3352,7 +3367,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="46" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" s="38" t="s">
         <v>27</v>
@@ -3434,13 +3449,13 @@
     <row r="16" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33"/>
       <c r="B16" s="46" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="C16" s="38" t="s">
-        <v>85</v>
-      </c>
       <c r="D16" s="38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E16" s="14"/>
       <c r="F16" s="53"/>
@@ -3507,13 +3522,13 @@
     <row r="17" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33"/>
       <c r="B17" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="D17" s="38" t="s">
         <v>67</v>
-      </c>
-      <c r="D17" s="38" t="s">
-        <v>68</v>
       </c>
       <c r="E17" s="14">
         <v>0</v>
@@ -3587,13 +3602,13 @@
     <row r="18" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33"/>
       <c r="B18" s="46" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="38" t="s">
         <v>64</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="38" t="s">
-        <v>65</v>
       </c>
       <c r="E18" s="14">
         <v>0.2</v>
@@ -3664,10 +3679,10 @@
     <row r="19" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33"/>
       <c r="B19" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="38" t="s">
         <v>60</v>
-      </c>
-      <c r="C19" s="38" t="s">
-        <v>61</v>
       </c>
       <c r="D19" s="38"/>
       <c r="E19" s="14">
@@ -4152,7 +4167,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="80" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C25" s="81"/>
       <c r="D25" s="81"/>
@@ -4224,13 +4239,13 @@
     <row r="26" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32"/>
       <c r="B26" s="76" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="77" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="77" t="s">
-        <v>73</v>
-      </c>
       <c r="D26" s="77" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E26" s="78">
         <v>1</v>
@@ -4307,13 +4322,13 @@
     <row r="27" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32"/>
       <c r="B27" s="76" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" s="77" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D27" s="77" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E27" s="78">
         <v>1</v>
@@ -4389,13 +4404,13 @@
     <row r="28" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32"/>
       <c r="B28" s="76" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C28" s="77" t="s">
+        <v>72</v>
+      </c>
+      <c r="D28" s="77" t="s">
         <v>73</v>
-      </c>
-      <c r="D28" s="77" t="s">
-        <v>74</v>
       </c>
       <c r="E28" s="78">
         <v>1</v>
@@ -4473,13 +4488,13 @@
     <row r="29" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="32"/>
       <c r="B29" s="76" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D29" s="77" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E29" s="78">
         <v>1</v>
@@ -4557,7 +4572,7 @@
         <v>11</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C30" s="41"/>
       <c r="D30" s="41"/>
@@ -4628,17 +4643,17 @@
     </row>
     <row r="31" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32"/>
-      <c r="B31" s="48" t="s">
+      <c r="B31" s="88" t="s">
         <v>38</v>
       </c>
       <c r="C31" s="42" t="s">
         <v>39</v>
       </c>
       <c r="D31" s="42" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E31" s="20">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F31" s="59">
         <f>F15+15</f>
@@ -4713,28 +4728,19 @@
     <row r="32" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32"/>
       <c r="B32" s="48" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="C32" s="42" t="s">
-        <v>27</v>
+        <v>87</v>
       </c>
       <c r="D32" s="42" t="s">
-        <v>75</v>
-      </c>
-      <c r="E32" s="20">
-        <v>1</v>
-      </c>
-      <c r="F32" s="59">
-        <v>45858</v>
-      </c>
-      <c r="G32" s="59">
-        <v>45858</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="E32" s="20"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
       <c r="H32" s="11"/>
-      <c r="I32" s="11">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
+      <c r="I32" s="11"/>
       <c r="J32" s="28"/>
       <c r="K32" s="28"/>
       <c r="L32" s="28"/>
@@ -4794,14 +4800,14 @@
     </row>
     <row r="33" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="32"/>
-      <c r="B33" s="48" t="s">
-        <v>52</v>
+      <c r="B33" s="88" t="s">
+        <v>51</v>
       </c>
       <c r="C33" s="42" t="s">
         <v>39</v>
       </c>
       <c r="D33" s="42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E33" s="20">
         <v>1</v>
@@ -4876,29 +4882,26 @@
     </row>
     <row r="34" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="32"/>
-      <c r="B34" s="48" t="s">
-        <v>41</v>
+      <c r="B34" s="88" t="s">
+        <v>84</v>
       </c>
       <c r="C34" s="42" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D34" s="42" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="E34" s="20">
         <v>1</v>
       </c>
       <c r="F34" s="59">
-        <v>45837</v>
+        <v>45829</v>
       </c>
       <c r="G34" s="59">
-        <v>45851</v>
+        <v>45829</v>
       </c>
       <c r="H34" s="11"/>
-      <c r="I34" s="11">
-        <f t="shared" si="6"/>
-        <v>15</v>
-      </c>
+      <c r="I34" s="11"/>
       <c r="J34" s="28"/>
       <c r="K34" s="28"/>
       <c r="L34" s="28"/>
@@ -4957,23 +4960,29 @@
       <c r="BM34" s="28"/>
     </row>
     <row r="35" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C35" s="74" t="s">
-        <v>55</v>
-      </c>
-      <c r="D35" s="43"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="60"/>
-      <c r="G35" s="61"/>
+      <c r="A35" s="32"/>
+      <c r="B35" s="88" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="E35" s="20">
+        <v>1</v>
+      </c>
+      <c r="F35" s="59">
+        <v>45837</v>
+      </c>
+      <c r="G35" s="59">
+        <v>45851</v>
+      </c>
       <c r="H35" s="11"/>
-      <c r="I35" s="11" t="str">
+      <c r="I35" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>15</v>
       </c>
       <c r="J35" s="28"/>
       <c r="K35" s="28"/>
@@ -5033,29 +5042,23 @@
       <c r="BM35" s="28"/>
     </row>
     <row r="36" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="32"/>
-      <c r="B36" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36" s="44" t="s">
+      <c r="A36" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="74" t="s">
         <v>54</v>
       </c>
-      <c r="D36" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="E36" s="23">
-        <v>1</v>
-      </c>
-      <c r="F36" s="62">
-        <v>45837</v>
-      </c>
-      <c r="G36" s="62">
-        <v>45837</v>
-      </c>
+      <c r="D36" s="43"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="60"/>
+      <c r="G36" s="61"/>
       <c r="H36" s="11"/>
-      <c r="I36" s="11">
+      <c r="I36" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
       <c r="J36" s="28"/>
       <c r="K36" s="28"/>
@@ -5117,12 +5120,14 @@
     <row r="37" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="32"/>
       <c r="B37" s="49" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C37" s="44" t="s">
-        <v>54</v>
-      </c>
-      <c r="D37" s="44"/>
+        <v>53</v>
+      </c>
+      <c r="D37" s="44" t="s">
+        <v>57</v>
+      </c>
       <c r="E37" s="23">
         <v>1</v>
       </c>
@@ -5133,7 +5138,10 @@
         <v>45837</v>
       </c>
       <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
+      <c r="I37" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
       <c r="J37" s="28"/>
       <c r="K37" s="28"/>
       <c r="L37" s="28"/>
@@ -5194,10 +5202,10 @@
     <row r="38" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="32"/>
       <c r="B38" s="49" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C38" s="44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D38" s="44"/>
       <c r="E38" s="23">
@@ -5210,10 +5218,7 @@
         <v>45837</v>
       </c>
       <c r="H38" s="11"/>
-      <c r="I38" s="11">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
+      <c r="I38" s="11"/>
       <c r="J38" s="28"/>
       <c r="K38" s="28"/>
       <c r="L38" s="28"/>
@@ -5274,10 +5279,10 @@
     <row r="39" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="32"/>
       <c r="B39" s="49" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C39" s="44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D39" s="44"/>
       <c r="E39" s="23">
@@ -5354,10 +5359,10 @@
     <row r="40" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32"/>
       <c r="B40" s="49" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C40" s="44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D40" s="44"/>
       <c r="E40" s="23">
@@ -5434,23 +5439,25 @@
     <row r="41" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="32"/>
       <c r="B41" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D41" s="44" t="s">
-        <v>59</v>
-      </c>
+      <c r="D41" s="44"/>
       <c r="E41" s="23">
-        <v>0</v>
-      </c>
-      <c r="F41" s="62"/>
-      <c r="G41" s="62"/>
+        <v>1</v>
+      </c>
+      <c r="F41" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G41" s="62">
+        <v>45837</v>
+      </c>
       <c r="H41" s="11"/>
-      <c r="I41" s="11" t="str">
+      <c r="I41" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J41" s="28"/>
       <c r="K41" s="28"/>
@@ -5510,15 +5517,21 @@
       <c r="BM41" s="28"/>
     </row>
     <row r="42" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B42" s="50"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="45"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="63"/>
-      <c r="G42" s="63"/>
+      <c r="A42" s="32"/>
+      <c r="B42" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D42" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="E42" s="23">
+        <v>0</v>
+      </c>
+      <c r="F42" s="62"/>
+      <c r="G42" s="62"/>
       <c r="H42" s="11"/>
       <c r="I42" s="11" t="str">
         <f t="shared" si="6"/>
@@ -5582,90 +5595,162 @@
       <c r="BM42" s="28"/>
     </row>
     <row r="43" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C43" s="25"/>
-      <c r="D43" s="25"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="64"/>
-      <c r="G43" s="65"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27" t="str">
+      <c r="A43" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="50"/>
+      <c r="C43" s="45"/>
+      <c r="D43" s="45"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="63"/>
+      <c r="G43" s="63"/>
+      <c r="H43" s="11"/>
+      <c r="I43" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="J43" s="30"/>
-      <c r="K43" s="30"/>
-      <c r="L43" s="30"/>
-      <c r="M43" s="30"/>
-      <c r="N43" s="30"/>
-      <c r="O43" s="30"/>
-      <c r="P43" s="30"/>
-      <c r="Q43" s="30"/>
-      <c r="R43" s="30"/>
-      <c r="S43" s="30"/>
-      <c r="T43" s="30"/>
-      <c r="U43" s="30"/>
-      <c r="V43" s="30"/>
-      <c r="W43" s="30"/>
-      <c r="X43" s="30"/>
-      <c r="Y43" s="30"/>
-      <c r="Z43" s="30"/>
-      <c r="AA43" s="30"/>
-      <c r="AB43" s="30"/>
-      <c r="AC43" s="30"/>
-      <c r="AD43" s="30"/>
-      <c r="AE43" s="30"/>
-      <c r="AF43" s="30"/>
-      <c r="AG43" s="30"/>
-      <c r="AH43" s="30"/>
-      <c r="AI43" s="30"/>
-      <c r="AJ43" s="30"/>
-      <c r="AK43" s="30"/>
-      <c r="AL43" s="30"/>
-      <c r="AM43" s="30"/>
-      <c r="AN43" s="30"/>
-      <c r="AO43" s="30"/>
-      <c r="AP43" s="30"/>
-      <c r="AQ43" s="30"/>
-      <c r="AR43" s="30"/>
-      <c r="AS43" s="30"/>
-      <c r="AT43" s="30"/>
-      <c r="AU43" s="30"/>
-      <c r="AV43" s="30"/>
-      <c r="AW43" s="30"/>
-      <c r="AX43" s="30"/>
-      <c r="AY43" s="30"/>
-      <c r="AZ43" s="30"/>
-      <c r="BA43" s="30"/>
-      <c r="BB43" s="30"/>
-      <c r="BC43" s="30"/>
-      <c r="BD43" s="30"/>
-      <c r="BE43" s="30"/>
-      <c r="BF43" s="30"/>
-      <c r="BG43" s="30"/>
-      <c r="BH43" s="30"/>
-      <c r="BI43" s="30"/>
-      <c r="BJ43" s="30"/>
-      <c r="BK43" s="30"/>
-      <c r="BL43" s="30"/>
-      <c r="BM43" s="30"/>
+      <c r="J43" s="28"/>
+      <c r="K43" s="28"/>
+      <c r="L43" s="28"/>
+      <c r="M43" s="28"/>
+      <c r="N43" s="28"/>
+      <c r="O43" s="28"/>
+      <c r="P43" s="28"/>
+      <c r="Q43" s="28"/>
+      <c r="R43" s="28"/>
+      <c r="S43" s="28"/>
+      <c r="T43" s="28"/>
+      <c r="U43" s="28"/>
+      <c r="V43" s="28"/>
+      <c r="W43" s="28"/>
+      <c r="X43" s="28"/>
+      <c r="Y43" s="28"/>
+      <c r="Z43" s="28"/>
+      <c r="AA43" s="28"/>
+      <c r="AB43" s="28"/>
+      <c r="AC43" s="28"/>
+      <c r="AD43" s="28"/>
+      <c r="AE43" s="28"/>
+      <c r="AF43" s="28"/>
+      <c r="AG43" s="28"/>
+      <c r="AH43" s="28"/>
+      <c r="AI43" s="28"/>
+      <c r="AJ43" s="28"/>
+      <c r="AK43" s="28"/>
+      <c r="AL43" s="28"/>
+      <c r="AM43" s="28"/>
+      <c r="AN43" s="28"/>
+      <c r="AO43" s="28"/>
+      <c r="AP43" s="28"/>
+      <c r="AQ43" s="28"/>
+      <c r="AR43" s="28"/>
+      <c r="AS43" s="28"/>
+      <c r="AT43" s="28"/>
+      <c r="AU43" s="28"/>
+      <c r="AV43" s="28"/>
+      <c r="AW43" s="28"/>
+      <c r="AX43" s="28"/>
+      <c r="AY43" s="28"/>
+      <c r="AZ43" s="28"/>
+      <c r="BA43" s="28"/>
+      <c r="BB43" s="28"/>
+      <c r="BC43" s="28"/>
+      <c r="BD43" s="28"/>
+      <c r="BE43" s="28"/>
+      <c r="BF43" s="28"/>
+      <c r="BG43" s="28"/>
+      <c r="BH43" s="28"/>
+      <c r="BI43" s="28"/>
+      <c r="BJ43" s="28"/>
+      <c r="BK43" s="28"/>
+      <c r="BL43" s="28"/>
+      <c r="BM43" s="28"/>
     </row>
-    <row r="44" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H44" s="6"/>
+    <row r="44" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="25"/>
+      <c r="D44" s="25"/>
+      <c r="E44" s="26"/>
+      <c r="F44" s="64"/>
+      <c r="G44" s="65"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J44" s="30"/>
+      <c r="K44" s="30"/>
+      <c r="L44" s="30"/>
+      <c r="M44" s="30"/>
+      <c r="N44" s="30"/>
+      <c r="O44" s="30"/>
+      <c r="P44" s="30"/>
+      <c r="Q44" s="30"/>
+      <c r="R44" s="30"/>
+      <c r="S44" s="30"/>
+      <c r="T44" s="30"/>
+      <c r="U44" s="30"/>
+      <c r="V44" s="30"/>
+      <c r="W44" s="30"/>
+      <c r="X44" s="30"/>
+      <c r="Y44" s="30"/>
+      <c r="Z44" s="30"/>
+      <c r="AA44" s="30"/>
+      <c r="AB44" s="30"/>
+      <c r="AC44" s="30"/>
+      <c r="AD44" s="30"/>
+      <c r="AE44" s="30"/>
+      <c r="AF44" s="30"/>
+      <c r="AG44" s="30"/>
+      <c r="AH44" s="30"/>
+      <c r="AI44" s="30"/>
+      <c r="AJ44" s="30"/>
+      <c r="AK44" s="30"/>
+      <c r="AL44" s="30"/>
+      <c r="AM44" s="30"/>
+      <c r="AN44" s="30"/>
+      <c r="AO44" s="30"/>
+      <c r="AP44" s="30"/>
+      <c r="AQ44" s="30"/>
+      <c r="AR44" s="30"/>
+      <c r="AS44" s="30"/>
+      <c r="AT44" s="30"/>
+      <c r="AU44" s="30"/>
+      <c r="AV44" s="30"/>
+      <c r="AW44" s="30"/>
+      <c r="AX44" s="30"/>
+      <c r="AY44" s="30"/>
+      <c r="AZ44" s="30"/>
+      <c r="BA44" s="30"/>
+      <c r="BB44" s="30"/>
+      <c r="BC44" s="30"/>
+      <c r="BD44" s="30"/>
+      <c r="BE44" s="30"/>
+      <c r="BF44" s="30"/>
+      <c r="BG44" s="30"/>
+      <c r="BH44" s="30"/>
+      <c r="BI44" s="30"/>
+      <c r="BJ44" s="30"/>
+      <c r="BK44" s="30"/>
+      <c r="BL44" s="30"/>
+      <c r="BM44" s="30"/>
     </row>
     <row r="45" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="G45" s="34"/>
+      <c r="H45" s="6"/>
     </row>
     <row r="46" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="G46" s="34"/>
+    </row>
+    <row r="47" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -5682,7 +5767,7 @@
     <mergeCell ref="AL4:AR4"/>
     <mergeCell ref="AS4:AY4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E43">
+  <conditionalFormatting sqref="E7:E44">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5696,12 +5781,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:BM43">
+  <conditionalFormatting sqref="J5:BM44">
     <cfRule type="expression" dxfId="2" priority="33">
       <formula>AND(TODAY()&gt;=J$5,TODAY()&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:BM43">
+  <conditionalFormatting sqref="J7:BM44">
     <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(Fecha_incio&lt;=J$5,ROUNDDOWN((Fecha_final-Fecha_incio+1)*Progresos,0)+Fecha_incio-1&gt;=J$5)</formula>
     </cfRule>
@@ -5736,7 +5821,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E7:E43</xm:sqref>
+          <xm:sqref>E7:E44</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Modificamos profesor, permitiendo asignar curso como director, tipodcto reparado para teacher cambio de nombres de las variables,modificacion de Manage para teacher student, implementacion de nuevos input para almacenar mas datos
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD45B30-003F-4114-B814-FC86A2E406CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E0D9CBB-8E5A-4819-BD87-FD4D0FBADC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="94">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -405,6 +405,21 @@
   </si>
   <si>
     <t>Cuando modificamos cedula no cambia imagen</t>
+  </si>
+  <si>
+    <t>La idea es enviarlo al correo registrado</t>
+  </si>
+  <si>
+    <t>Firma del estudiante</t>
+  </si>
+  <si>
+    <t>La idea es que tenga un checkbox de confirmacion de la anotacion</t>
+  </si>
+  <si>
+    <t>Acudiente enviar Anotacion Notificacion</t>
+  </si>
+  <si>
+    <t>FILTRAR ANOTACION y ESTUDIANTE</t>
   </si>
 </sst>
 </file>
@@ -1440,6 +1455,18 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
       <alignment horizontal="right" indent="1"/>
     </xf>
@@ -1447,18 +1474,6 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="55">
     <cellStyle name="20% - Énfasis1" xfId="31" builtinId="30" customBuiltin="1"/>
@@ -2095,7 +2110,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BM47"/>
+  <dimension ref="A1:BM50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="32" customWidth="1"/>
@@ -2146,120 +2161,120 @@
       <c r="B3" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="95">
+      <c r="D3" s="93"/>
+      <c r="E3" s="94"/>
+      <c r="F3" s="92">
         <v>45822</v>
       </c>
-      <c r="G3" s="95"/>
+      <c r="G3" s="92"/>
     </row>
     <row r="4" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="89" t="s">
+      <c r="C4" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="89"/>
-      <c r="E4" s="90"/>
+      <c r="D4" s="93"/>
+      <c r="E4" s="94"/>
       <c r="F4" s="7">
         <v>1</v>
       </c>
-      <c r="J4" s="92">
+      <c r="J4" s="89">
         <f>J5</f>
         <v>45817</v>
       </c>
-      <c r="K4" s="93"/>
-      <c r="L4" s="93"/>
-      <c r="M4" s="93"/>
-      <c r="N4" s="93"/>
-      <c r="O4" s="93"/>
-      <c r="P4" s="94"/>
-      <c r="Q4" s="92">
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
+      <c r="P4" s="91"/>
+      <c r="Q4" s="89">
         <f>Q5</f>
         <v>45824</v>
       </c>
-      <c r="R4" s="93"/>
-      <c r="S4" s="93"/>
-      <c r="T4" s="93"/>
-      <c r="U4" s="93"/>
-      <c r="V4" s="93"/>
-      <c r="W4" s="94"/>
-      <c r="X4" s="92">
+      <c r="R4" s="90"/>
+      <c r="S4" s="90"/>
+      <c r="T4" s="90"/>
+      <c r="U4" s="90"/>
+      <c r="V4" s="90"/>
+      <c r="W4" s="91"/>
+      <c r="X4" s="89">
         <f>X5</f>
         <v>45831</v>
       </c>
-      <c r="Y4" s="93"/>
-      <c r="Z4" s="93"/>
-      <c r="AA4" s="93"/>
-      <c r="AB4" s="93"/>
-      <c r="AC4" s="93"/>
-      <c r="AD4" s="94"/>
-      <c r="AE4" s="92">
+      <c r="Y4" s="90"/>
+      <c r="Z4" s="90"/>
+      <c r="AA4" s="90"/>
+      <c r="AB4" s="90"/>
+      <c r="AC4" s="90"/>
+      <c r="AD4" s="91"/>
+      <c r="AE4" s="89">
         <f>AE5</f>
         <v>45838</v>
       </c>
-      <c r="AF4" s="93"/>
-      <c r="AG4" s="93"/>
-      <c r="AH4" s="93"/>
-      <c r="AI4" s="93"/>
-      <c r="AJ4" s="93"/>
-      <c r="AK4" s="94"/>
-      <c r="AL4" s="92">
+      <c r="AF4" s="90"/>
+      <c r="AG4" s="90"/>
+      <c r="AH4" s="90"/>
+      <c r="AI4" s="90"/>
+      <c r="AJ4" s="90"/>
+      <c r="AK4" s="91"/>
+      <c r="AL4" s="89">
         <f>AL5</f>
         <v>45845</v>
       </c>
-      <c r="AM4" s="93"/>
-      <c r="AN4" s="93"/>
-      <c r="AO4" s="93"/>
-      <c r="AP4" s="93"/>
-      <c r="AQ4" s="93"/>
-      <c r="AR4" s="94"/>
-      <c r="AS4" s="92">
+      <c r="AM4" s="90"/>
+      <c r="AN4" s="90"/>
+      <c r="AO4" s="90"/>
+      <c r="AP4" s="90"/>
+      <c r="AQ4" s="90"/>
+      <c r="AR4" s="91"/>
+      <c r="AS4" s="89">
         <f>AS5</f>
         <v>45852</v>
       </c>
-      <c r="AT4" s="93"/>
-      <c r="AU4" s="93"/>
-      <c r="AV4" s="93"/>
-      <c r="AW4" s="93"/>
-      <c r="AX4" s="93"/>
-      <c r="AY4" s="94"/>
-      <c r="AZ4" s="92">
+      <c r="AT4" s="90"/>
+      <c r="AU4" s="90"/>
+      <c r="AV4" s="90"/>
+      <c r="AW4" s="90"/>
+      <c r="AX4" s="90"/>
+      <c r="AY4" s="91"/>
+      <c r="AZ4" s="89">
         <f>AZ5</f>
         <v>45859</v>
       </c>
-      <c r="BA4" s="93"/>
-      <c r="BB4" s="93"/>
-      <c r="BC4" s="93"/>
-      <c r="BD4" s="93"/>
-      <c r="BE4" s="93"/>
-      <c r="BF4" s="94"/>
-      <c r="BG4" s="92">
+      <c r="BA4" s="90"/>
+      <c r="BB4" s="90"/>
+      <c r="BC4" s="90"/>
+      <c r="BD4" s="90"/>
+      <c r="BE4" s="90"/>
+      <c r="BF4" s="91"/>
+      <c r="BG4" s="89">
         <f>BG5</f>
         <v>45866</v>
       </c>
-      <c r="BH4" s="93"/>
-      <c r="BI4" s="93"/>
-      <c r="BJ4" s="93"/>
-      <c r="BK4" s="93"/>
-      <c r="BL4" s="93"/>
-      <c r="BM4" s="94"/>
+      <c r="BH4" s="90"/>
+      <c r="BI4" s="90"/>
+      <c r="BJ4" s="90"/>
+      <c r="BK4" s="90"/>
+      <c r="BL4" s="90"/>
+      <c r="BM4" s="91"/>
     </row>
     <row r="5" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="91"/>
-      <c r="C5" s="91"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="91"/>
-      <c r="F5" s="91"/>
-      <c r="G5" s="91"/>
-      <c r="H5" s="91"/>
+      <c r="B5" s="95"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="95"/>
+      <c r="E5" s="95"/>
+      <c r="F5" s="95"/>
+      <c r="G5" s="95"/>
+      <c r="H5" s="95"/>
       <c r="J5" s="70">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -2818,7 +2833,7 @@
       <c r="G8" s="55"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11" t="str">
-        <f t="shared" ref="I8:I44" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
+        <f t="shared" ref="I8:I47" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
         <v/>
       </c>
       <c r="J8" s="28"/>
@@ -4568,22 +4583,25 @@
       <c r="BM29" s="28"/>
     </row>
     <row r="30" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B30" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="58"/>
+      <c r="A30" s="32"/>
+      <c r="B30" s="76" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="77"/>
+      <c r="D30" s="77" t="s">
+        <v>91</v>
+      </c>
+      <c r="E30" s="78">
+        <v>0</v>
+      </c>
+      <c r="F30" s="79">
+        <v>0</v>
+      </c>
+      <c r="G30" s="79">
+        <v>0</v>
+      </c>
       <c r="H30" s="11"/>
-      <c r="I30" s="11" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
+      <c r="I30" s="11"/>
       <c r="J30" s="28"/>
       <c r="K30" s="28"/>
       <c r="L30" s="28"/>
@@ -4643,31 +4661,16 @@
     </row>
     <row r="31" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="32"/>
-      <c r="B31" s="88" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" s="42" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31" s="42" t="s">
-        <v>79</v>
-      </c>
-      <c r="E31" s="20">
-        <v>1</v>
-      </c>
-      <c r="F31" s="59">
-        <f>F15+15</f>
-        <v>45837</v>
-      </c>
-      <c r="G31" s="59">
-        <f>F31+5</f>
-        <v>45842</v>
-      </c>
+      <c r="B31" s="76" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="77"/>
+      <c r="D31" s="77"/>
+      <c r="E31" s="78"/>
+      <c r="F31" s="79"/>
+      <c r="G31" s="79"/>
       <c r="H31" s="11"/>
-      <c r="I31" s="11">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
+      <c r="I31" s="11"/>
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
       <c r="L31" s="28"/>
@@ -4727,18 +4730,22 @@
     </row>
     <row r="32" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="32"/>
-      <c r="B32" s="48" t="s">
-        <v>86</v>
-      </c>
-      <c r="C32" s="42" t="s">
-        <v>87</v>
-      </c>
-      <c r="D32" s="42" t="s">
-        <v>88</v>
-      </c>
-      <c r="E32" s="20"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
+      <c r="B32" s="76" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" s="77"/>
+      <c r="D32" s="77" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" s="78">
+        <v>0</v>
+      </c>
+      <c r="F32" s="79">
+        <v>0</v>
+      </c>
+      <c r="G32" s="79">
+        <v>0</v>
+      </c>
       <c r="H32" s="11"/>
       <c r="I32" s="11"/>
       <c r="J32" s="28"/>
@@ -4799,29 +4806,21 @@
       <c r="BM32" s="28"/>
     </row>
     <row r="33" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="32"/>
-      <c r="B33" s="88" t="s">
-        <v>51</v>
-      </c>
-      <c r="C33" s="42" t="s">
-        <v>39</v>
-      </c>
-      <c r="D33" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="E33" s="20">
-        <v>1</v>
-      </c>
-      <c r="F33" s="59">
-        <v>45829</v>
-      </c>
-      <c r="G33" s="59">
-        <v>45829</v>
-      </c>
+      <c r="A33" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="58"/>
       <c r="H33" s="11"/>
-      <c r="I33" s="11">
+      <c r="I33" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
       <c r="J33" s="28"/>
       <c r="K33" s="28"/>
@@ -4883,25 +4882,30 @@
     <row r="34" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="32"/>
       <c r="B34" s="88" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="C34" s="42" t="s">
         <v>39</v>
       </c>
       <c r="D34" s="42" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E34" s="20">
         <v>1</v>
       </c>
       <c r="F34" s="59">
-        <v>45829</v>
+        <f>F15+15</f>
+        <v>45837</v>
       </c>
       <c r="G34" s="59">
-        <v>45829</v>
+        <f>F34+5</f>
+        <v>45842</v>
       </c>
       <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
+      <c r="I34" s="11">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
       <c r="J34" s="28"/>
       <c r="K34" s="28"/>
       <c r="L34" s="28"/>
@@ -4961,29 +4965,20 @@
     </row>
     <row r="35" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="32"/>
-      <c r="B35" s="88" t="s">
-        <v>40</v>
+      <c r="B35" s="48" t="s">
+        <v>86</v>
       </c>
       <c r="C35" s="42" t="s">
-        <v>27</v>
+        <v>87</v>
       </c>
       <c r="D35" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" s="20">
-        <v>1</v>
-      </c>
-      <c r="F35" s="59">
-        <v>45837</v>
-      </c>
-      <c r="G35" s="59">
-        <v>45851</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="E35" s="20"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="59"/>
       <c r="H35" s="11"/>
-      <c r="I35" s="11">
-        <f t="shared" si="6"/>
-        <v>15</v>
-      </c>
+      <c r="I35" s="11"/>
       <c r="J35" s="28"/>
       <c r="K35" s="28"/>
       <c r="L35" s="28"/>
@@ -5042,23 +5037,29 @@
       <c r="BM35" s="28"/>
     </row>
     <row r="36" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="74" t="s">
-        <v>54</v>
-      </c>
-      <c r="D36" s="43"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="60"/>
-      <c r="G36" s="61"/>
+      <c r="A36" s="32"/>
+      <c r="B36" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="C36" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="E36" s="20">
+        <v>1</v>
+      </c>
+      <c r="F36" s="59">
+        <v>45829</v>
+      </c>
+      <c r="G36" s="59">
+        <v>45829</v>
+      </c>
       <c r="H36" s="11"/>
-      <c r="I36" s="11" t="str">
+      <c r="I36" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J36" s="28"/>
       <c r="K36" s="28"/>
@@ -5119,29 +5120,26 @@
     </row>
     <row r="37" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="32"/>
-      <c r="B37" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="C37" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="D37" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="E37" s="23">
+      <c r="B37" s="88" t="s">
+        <v>84</v>
+      </c>
+      <c r="C37" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="D37" s="42" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" s="20">
         <v>1</v>
       </c>
-      <c r="F37" s="62">
-        <v>45837</v>
-      </c>
-      <c r="G37" s="62">
-        <v>45837</v>
+      <c r="F37" s="59">
+        <v>45829</v>
+      </c>
+      <c r="G37" s="59">
+        <v>45829</v>
       </c>
       <c r="H37" s="11"/>
-      <c r="I37" s="11">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
+      <c r="I37" s="11"/>
       <c r="J37" s="28"/>
       <c r="K37" s="28"/>
       <c r="L37" s="28"/>
@@ -5201,24 +5199,29 @@
     </row>
     <row r="38" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="32"/>
-      <c r="B38" s="49" t="s">
-        <v>55</v>
-      </c>
-      <c r="C38" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="D38" s="44"/>
-      <c r="E38" s="23">
+      <c r="B38" s="88" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="E38" s="20">
         <v>1</v>
       </c>
-      <c r="F38" s="62">
+      <c r="F38" s="59">
         <v>45837</v>
       </c>
-      <c r="G38" s="62">
-        <v>45837</v>
+      <c r="G38" s="59">
+        <v>45851</v>
       </c>
       <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
+      <c r="I38" s="11">
+        <f t="shared" si="6"/>
+        <v>15</v>
+      </c>
       <c r="J38" s="28"/>
       <c r="K38" s="28"/>
       <c r="L38" s="28"/>
@@ -5277,27 +5280,23 @@
       <c r="BM38" s="28"/>
     </row>
     <row r="39" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="32"/>
-      <c r="B39" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="C39" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="D39" s="44"/>
-      <c r="E39" s="23">
-        <v>1</v>
-      </c>
-      <c r="F39" s="62">
-        <v>45837</v>
-      </c>
-      <c r="G39" s="62">
-        <v>45837</v>
-      </c>
+      <c r="A39" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="74" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39" s="43"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="60"/>
+      <c r="G39" s="61"/>
       <c r="H39" s="11"/>
-      <c r="I39" s="11">
+      <c r="I39" s="11" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
       <c r="J39" s="28"/>
       <c r="K39" s="28"/>
@@ -5359,12 +5358,14 @@
     <row r="40" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="32"/>
       <c r="B40" s="49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C40" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="D40" s="44"/>
+      <c r="D40" s="44" t="s">
+        <v>57</v>
+      </c>
       <c r="E40" s="23">
         <v>1</v>
       </c>
@@ -5439,7 +5440,7 @@
     <row r="41" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="32"/>
       <c r="B41" s="49" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C41" s="44" t="s">
         <v>53</v>
@@ -5455,10 +5456,7 @@
         <v>45837</v>
       </c>
       <c r="H41" s="11"/>
-      <c r="I41" s="11">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
+      <c r="I41" s="11"/>
       <c r="J41" s="28"/>
       <c r="K41" s="28"/>
       <c r="L41" s="28"/>
@@ -5519,23 +5517,25 @@
     <row r="42" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="32"/>
       <c r="B42" s="49" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C42" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D42" s="44" t="s">
-        <v>58</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="D42" s="44"/>
       <c r="E42" s="23">
-        <v>0</v>
-      </c>
-      <c r="F42" s="62"/>
-      <c r="G42" s="62"/>
+        <v>1</v>
+      </c>
+      <c r="F42" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G42" s="62">
+        <v>45837</v>
+      </c>
       <c r="H42" s="11"/>
-      <c r="I42" s="11" t="str">
+      <c r="I42" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J42" s="28"/>
       <c r="K42" s="28"/>
@@ -5595,19 +5595,27 @@
       <c r="BM42" s="28"/>
     </row>
     <row r="43" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B43" s="50"/>
-      <c r="C43" s="45"/>
-      <c r="D43" s="45"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="63"/>
-      <c r="G43" s="63"/>
+      <c r="A43" s="32"/>
+      <c r="B43" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="D43" s="44"/>
+      <c r="E43" s="23">
+        <v>1</v>
+      </c>
+      <c r="F43" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G43" s="62">
+        <v>45837</v>
+      </c>
       <c r="H43" s="11"/>
-      <c r="I43" s="11" t="str">
+      <c r="I43" s="11">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J43" s="28"/>
       <c r="K43" s="28"/>
@@ -5667,93 +5675,328 @@
       <c r="BM43" s="28"/>
     </row>
     <row r="44" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B44" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C44" s="25"/>
-      <c r="D44" s="25"/>
-      <c r="E44" s="26"/>
-      <c r="F44" s="64"/>
-      <c r="G44" s="65"/>
-      <c r="H44" s="27"/>
-      <c r="I44" s="27" t="str">
+      <c r="A44" s="32"/>
+      <c r="B44" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C44" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="D44" s="44"/>
+      <c r="E44" s="23">
+        <v>1</v>
+      </c>
+      <c r="F44" s="62">
+        <v>45837</v>
+      </c>
+      <c r="G44" s="62">
+        <v>45837</v>
+      </c>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="J44" s="28"/>
+      <c r="K44" s="28"/>
+      <c r="L44" s="28"/>
+      <c r="M44" s="28"/>
+      <c r="N44" s="28"/>
+      <c r="O44" s="28"/>
+      <c r="P44" s="28"/>
+      <c r="Q44" s="28"/>
+      <c r="R44" s="28"/>
+      <c r="S44" s="28"/>
+      <c r="T44" s="28"/>
+      <c r="U44" s="28"/>
+      <c r="V44" s="28"/>
+      <c r="W44" s="28"/>
+      <c r="X44" s="28"/>
+      <c r="Y44" s="28"/>
+      <c r="Z44" s="28"/>
+      <c r="AA44" s="28"/>
+      <c r="AB44" s="28"/>
+      <c r="AC44" s="28"/>
+      <c r="AD44" s="28"/>
+      <c r="AE44" s="28"/>
+      <c r="AF44" s="28"/>
+      <c r="AG44" s="28"/>
+      <c r="AH44" s="28"/>
+      <c r="AI44" s="28"/>
+      <c r="AJ44" s="28"/>
+      <c r="AK44" s="28"/>
+      <c r="AL44" s="28"/>
+      <c r="AM44" s="28"/>
+      <c r="AN44" s="28"/>
+      <c r="AO44" s="28"/>
+      <c r="AP44" s="28"/>
+      <c r="AQ44" s="28"/>
+      <c r="AR44" s="28"/>
+      <c r="AS44" s="28"/>
+      <c r="AT44" s="28"/>
+      <c r="AU44" s="28"/>
+      <c r="AV44" s="28"/>
+      <c r="AW44" s="28"/>
+      <c r="AX44" s="28"/>
+      <c r="AY44" s="28"/>
+      <c r="AZ44" s="28"/>
+      <c r="BA44" s="28"/>
+      <c r="BB44" s="28"/>
+      <c r="BC44" s="28"/>
+      <c r="BD44" s="28"/>
+      <c r="BE44" s="28"/>
+      <c r="BF44" s="28"/>
+      <c r="BG44" s="28"/>
+      <c r="BH44" s="28"/>
+      <c r="BI44" s="28"/>
+      <c r="BJ44" s="28"/>
+      <c r="BK44" s="28"/>
+      <c r="BL44" s="28"/>
+      <c r="BM44" s="28"/>
+    </row>
+    <row r="45" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="32"/>
+      <c r="B45" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D45" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" s="23">
+        <v>0</v>
+      </c>
+      <c r="F45" s="62"/>
+      <c r="G45" s="62"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="J44" s="30"/>
-      <c r="K44" s="30"/>
-      <c r="L44" s="30"/>
-      <c r="M44" s="30"/>
-      <c r="N44" s="30"/>
-      <c r="O44" s="30"/>
-      <c r="P44" s="30"/>
-      <c r="Q44" s="30"/>
-      <c r="R44" s="30"/>
-      <c r="S44" s="30"/>
-      <c r="T44" s="30"/>
-      <c r="U44" s="30"/>
-      <c r="V44" s="30"/>
-      <c r="W44" s="30"/>
-      <c r="X44" s="30"/>
-      <c r="Y44" s="30"/>
-      <c r="Z44" s="30"/>
-      <c r="AA44" s="30"/>
-      <c r="AB44" s="30"/>
-      <c r="AC44" s="30"/>
-      <c r="AD44" s="30"/>
-      <c r="AE44" s="30"/>
-      <c r="AF44" s="30"/>
-      <c r="AG44" s="30"/>
-      <c r="AH44" s="30"/>
-      <c r="AI44" s="30"/>
-      <c r="AJ44" s="30"/>
-      <c r="AK44" s="30"/>
-      <c r="AL44" s="30"/>
-      <c r="AM44" s="30"/>
-      <c r="AN44" s="30"/>
-      <c r="AO44" s="30"/>
-      <c r="AP44" s="30"/>
-      <c r="AQ44" s="30"/>
-      <c r="AR44" s="30"/>
-      <c r="AS44" s="30"/>
-      <c r="AT44" s="30"/>
-      <c r="AU44" s="30"/>
-      <c r="AV44" s="30"/>
-      <c r="AW44" s="30"/>
-      <c r="AX44" s="30"/>
-      <c r="AY44" s="30"/>
-      <c r="AZ44" s="30"/>
-      <c r="BA44" s="30"/>
-      <c r="BB44" s="30"/>
-      <c r="BC44" s="30"/>
-      <c r="BD44" s="30"/>
-      <c r="BE44" s="30"/>
-      <c r="BF44" s="30"/>
-      <c r="BG44" s="30"/>
-      <c r="BH44" s="30"/>
-      <c r="BI44" s="30"/>
-      <c r="BJ44" s="30"/>
-      <c r="BK44" s="30"/>
-      <c r="BL44" s="30"/>
-      <c r="BM44" s="30"/>
+      <c r="J45" s="28"/>
+      <c r="K45" s="28"/>
+      <c r="L45" s="28"/>
+      <c r="M45" s="28"/>
+      <c r="N45" s="28"/>
+      <c r="O45" s="28"/>
+      <c r="P45" s="28"/>
+      <c r="Q45" s="28"/>
+      <c r="R45" s="28"/>
+      <c r="S45" s="28"/>
+      <c r="T45" s="28"/>
+      <c r="U45" s="28"/>
+      <c r="V45" s="28"/>
+      <c r="W45" s="28"/>
+      <c r="X45" s="28"/>
+      <c r="Y45" s="28"/>
+      <c r="Z45" s="28"/>
+      <c r="AA45" s="28"/>
+      <c r="AB45" s="28"/>
+      <c r="AC45" s="28"/>
+      <c r="AD45" s="28"/>
+      <c r="AE45" s="28"/>
+      <c r="AF45" s="28"/>
+      <c r="AG45" s="28"/>
+      <c r="AH45" s="28"/>
+      <c r="AI45" s="28"/>
+      <c r="AJ45" s="28"/>
+      <c r="AK45" s="28"/>
+      <c r="AL45" s="28"/>
+      <c r="AM45" s="28"/>
+      <c r="AN45" s="28"/>
+      <c r="AO45" s="28"/>
+      <c r="AP45" s="28"/>
+      <c r="AQ45" s="28"/>
+      <c r="AR45" s="28"/>
+      <c r="AS45" s="28"/>
+      <c r="AT45" s="28"/>
+      <c r="AU45" s="28"/>
+      <c r="AV45" s="28"/>
+      <c r="AW45" s="28"/>
+      <c r="AX45" s="28"/>
+      <c r="AY45" s="28"/>
+      <c r="AZ45" s="28"/>
+      <c r="BA45" s="28"/>
+      <c r="BB45" s="28"/>
+      <c r="BC45" s="28"/>
+      <c r="BD45" s="28"/>
+      <c r="BE45" s="28"/>
+      <c r="BF45" s="28"/>
+      <c r="BG45" s="28"/>
+      <c r="BH45" s="28"/>
+      <c r="BI45" s="28"/>
+      <c r="BJ45" s="28"/>
+      <c r="BK45" s="28"/>
+      <c r="BL45" s="28"/>
+      <c r="BM45" s="28"/>
     </row>
-    <row r="45" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H45" s="6"/>
+    <row r="46" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="50"/>
+      <c r="C46" s="45"/>
+      <c r="D46" s="45"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="63"/>
+      <c r="G46" s="63"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J46" s="28"/>
+      <c r="K46" s="28"/>
+      <c r="L46" s="28"/>
+      <c r="M46" s="28"/>
+      <c r="N46" s="28"/>
+      <c r="O46" s="28"/>
+      <c r="P46" s="28"/>
+      <c r="Q46" s="28"/>
+      <c r="R46" s="28"/>
+      <c r="S46" s="28"/>
+      <c r="T46" s="28"/>
+      <c r="U46" s="28"/>
+      <c r="V46" s="28"/>
+      <c r="W46" s="28"/>
+      <c r="X46" s="28"/>
+      <c r="Y46" s="28"/>
+      <c r="Z46" s="28"/>
+      <c r="AA46" s="28"/>
+      <c r="AB46" s="28"/>
+      <c r="AC46" s="28"/>
+      <c r="AD46" s="28"/>
+      <c r="AE46" s="28"/>
+      <c r="AF46" s="28"/>
+      <c r="AG46" s="28"/>
+      <c r="AH46" s="28"/>
+      <c r="AI46" s="28"/>
+      <c r="AJ46" s="28"/>
+      <c r="AK46" s="28"/>
+      <c r="AL46" s="28"/>
+      <c r="AM46" s="28"/>
+      <c r="AN46" s="28"/>
+      <c r="AO46" s="28"/>
+      <c r="AP46" s="28"/>
+      <c r="AQ46" s="28"/>
+      <c r="AR46" s="28"/>
+      <c r="AS46" s="28"/>
+      <c r="AT46" s="28"/>
+      <c r="AU46" s="28"/>
+      <c r="AV46" s="28"/>
+      <c r="AW46" s="28"/>
+      <c r="AX46" s="28"/>
+      <c r="AY46" s="28"/>
+      <c r="AZ46" s="28"/>
+      <c r="BA46" s="28"/>
+      <c r="BB46" s="28"/>
+      <c r="BC46" s="28"/>
+      <c r="BD46" s="28"/>
+      <c r="BE46" s="28"/>
+      <c r="BF46" s="28"/>
+      <c r="BG46" s="28"/>
+      <c r="BH46" s="28"/>
+      <c r="BI46" s="28"/>
+      <c r="BJ46" s="28"/>
+      <c r="BK46" s="28"/>
+      <c r="BL46" s="28"/>
+      <c r="BM46" s="28"/>
     </row>
-    <row r="46" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="G46" s="34"/>
+    <row r="47" spans="1:65" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
+      <c r="E47" s="26"/>
+      <c r="F47" s="64"/>
+      <c r="G47" s="65"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J47" s="30"/>
+      <c r="K47" s="30"/>
+      <c r="L47" s="30"/>
+      <c r="M47" s="30"/>
+      <c r="N47" s="30"/>
+      <c r="O47" s="30"/>
+      <c r="P47" s="30"/>
+      <c r="Q47" s="30"/>
+      <c r="R47" s="30"/>
+      <c r="S47" s="30"/>
+      <c r="T47" s="30"/>
+      <c r="U47" s="30"/>
+      <c r="V47" s="30"/>
+      <c r="W47" s="30"/>
+      <c r="X47" s="30"/>
+      <c r="Y47" s="30"/>
+      <c r="Z47" s="30"/>
+      <c r="AA47" s="30"/>
+      <c r="AB47" s="30"/>
+      <c r="AC47" s="30"/>
+      <c r="AD47" s="30"/>
+      <c r="AE47" s="30"/>
+      <c r="AF47" s="30"/>
+      <c r="AG47" s="30"/>
+      <c r="AH47" s="30"/>
+      <c r="AI47" s="30"/>
+      <c r="AJ47" s="30"/>
+      <c r="AK47" s="30"/>
+      <c r="AL47" s="30"/>
+      <c r="AM47" s="30"/>
+      <c r="AN47" s="30"/>
+      <c r="AO47" s="30"/>
+      <c r="AP47" s="30"/>
+      <c r="AQ47" s="30"/>
+      <c r="AR47" s="30"/>
+      <c r="AS47" s="30"/>
+      <c r="AT47" s="30"/>
+      <c r="AU47" s="30"/>
+      <c r="AV47" s="30"/>
+      <c r="AW47" s="30"/>
+      <c r="AX47" s="30"/>
+      <c r="AY47" s="30"/>
+      <c r="AZ47" s="30"/>
+      <c r="BA47" s="30"/>
+      <c r="BB47" s="30"/>
+      <c r="BC47" s="30"/>
+      <c r="BD47" s="30"/>
+      <c r="BE47" s="30"/>
+      <c r="BF47" s="30"/>
+      <c r="BG47" s="30"/>
+      <c r="BH47" s="30"/>
+      <c r="BI47" s="30"/>
+      <c r="BJ47" s="30"/>
+      <c r="BK47" s="30"/>
+      <c r="BL47" s="30"/>
+      <c r="BM47" s="30"/>
     </row>
-    <row r="47" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
+    <row r="48" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H48" s="6"/>
+    </row>
+    <row r="49" spans="3:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="G49" s="34"/>
+    </row>
+    <row r="50" spans="3:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="AL4:AR4"/>
+    <mergeCell ref="AS4:AY4"/>
     <mergeCell ref="AZ4:BF4"/>
     <mergeCell ref="BG4:BM4"/>
     <mergeCell ref="F3:G3"/>
@@ -5761,13 +6004,8 @@
     <mergeCell ref="Q4:W4"/>
     <mergeCell ref="X4:AD4"/>
     <mergeCell ref="AE4:AK4"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="AL4:AR4"/>
-    <mergeCell ref="AS4:AY4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E44">
+  <conditionalFormatting sqref="E7:E47">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5781,12 +6019,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:BM44">
+  <conditionalFormatting sqref="J5:BM47">
     <cfRule type="expression" dxfId="2" priority="33">
       <formula>AND(TODAY()&gt;=J$5,TODAY()&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:BM44">
+  <conditionalFormatting sqref="J7:BM47">
     <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(Fecha_incio&lt;=J$5,ROUNDDOWN((Fecha_final-Fecha_incio+1)*Progresos,0)+Fecha_incio-1&gt;=J$5)</formula>
     </cfRule>
@@ -5821,7 +6059,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E7:E44</xm:sqref>
+          <xm:sqref>E7:E47</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Update Icons Web, Linked with favicon, put icons all the page, IMPORTANT!! Created Filters to Teacher DNI,Name,Last Name, GRADE its Works
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB27929-2DF5-4355-9CE0-FD0D0AFD00EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FADECF-D3F2-49A8-8608-46701CD2A9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="94">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -350,9 +350,6 @@
     <t>StudentModel.php</t>
   </si>
   <si>
-    <t>Cuando modificamos cedula no cambia imagen</t>
-  </si>
-  <si>
     <t>La idea es enviarlo al correo registrado</t>
   </si>
   <si>
@@ -420,6 +417,9 @@
   </si>
   <si>
     <t>Acudiente enviar Anot Notificacion</t>
+  </si>
+  <si>
+    <t>Cuando solo admite 1 GB como maximo</t>
   </si>
 </sst>
 </file>
@@ -1333,179 +1333,179 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="44" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="44" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="44" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="10" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="9" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="12" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="11" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="2" xfId="10" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="2" xfId="30" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="38" borderId="2" xfId="50" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="8" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="45" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="45" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="45" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="4" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="3" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="44" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="44" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="44" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="10" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="9" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="12" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="11" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="2" xfId="10" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="2" xfId="30" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="38" borderId="2" xfId="50" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="8" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="45" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="45" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="45" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="45" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="55">
@@ -1565,74 +1565,7 @@
     <cellStyle name="Total" xfId="29" builtinId="25" customBuiltin="1"/>
     <cellStyle name="zTextoOculto" xfId="3" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
   </cellStyles>
-  <dxfs count="19">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill>
@@ -1759,15 +1692,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ListaTareasPendientes" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="18"/>
-      <tableStyleElement type="headerRow" dxfId="17"/>
-      <tableStyleElement type="totalRow" dxfId="16"/>
-      <tableStyleElement type="firstColumn" dxfId="15"/>
-      <tableStyleElement type="lastColumn" dxfId="14"/>
-      <tableStyleElement type="firstRowStripe" dxfId="13"/>
-      <tableStyleElement type="secondRowStripe" dxfId="12"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="11"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="10"/>
+      <tableStyleElement type="wholeTable" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="totalRow" dxfId="9"/>
+      <tableStyleElement type="firstColumn" dxfId="8"/>
+      <tableStyleElement type="lastColumn" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" dxfId="6"/>
+      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="4"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="3"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2265,121 +2198,121 @@
       <c r="C3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="47">
+      <c r="E3" s="100"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="99">
         <v>45822</v>
       </c>
-      <c r="H3" s="47"/>
+      <c r="H3" s="99"/>
     </row>
     <row r="4" spans="1:66" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="101"/>
       <c r="G4" s="3">
         <v>1</v>
       </c>
-      <c r="K4" s="48">
+      <c r="K4" s="96">
         <f>K5</f>
         <v>45817</v>
       </c>
-      <c r="L4" s="49"/>
-      <c r="M4" s="49"/>
-      <c r="N4" s="49"/>
-      <c r="O4" s="49"/>
-      <c r="P4" s="49"/>
-      <c r="Q4" s="50"/>
-      <c r="R4" s="48">
+      <c r="L4" s="97"/>
+      <c r="M4" s="97"/>
+      <c r="N4" s="97"/>
+      <c r="O4" s="97"/>
+      <c r="P4" s="97"/>
+      <c r="Q4" s="98"/>
+      <c r="R4" s="96">
         <f>R5</f>
         <v>45824</v>
       </c>
-      <c r="S4" s="49"/>
-      <c r="T4" s="49"/>
-      <c r="U4" s="49"/>
-      <c r="V4" s="49"/>
-      <c r="W4" s="49"/>
-      <c r="X4" s="50"/>
-      <c r="Y4" s="48">
+      <c r="S4" s="97"/>
+      <c r="T4" s="97"/>
+      <c r="U4" s="97"/>
+      <c r="V4" s="97"/>
+      <c r="W4" s="97"/>
+      <c r="X4" s="98"/>
+      <c r="Y4" s="96">
         <f>Y5</f>
         <v>45831</v>
       </c>
-      <c r="Z4" s="49"/>
-      <c r="AA4" s="49"/>
-      <c r="AB4" s="49"/>
-      <c r="AC4" s="49"/>
-      <c r="AD4" s="49"/>
-      <c r="AE4" s="50"/>
-      <c r="AF4" s="48">
+      <c r="Z4" s="97"/>
+      <c r="AA4" s="97"/>
+      <c r="AB4" s="97"/>
+      <c r="AC4" s="97"/>
+      <c r="AD4" s="97"/>
+      <c r="AE4" s="98"/>
+      <c r="AF4" s="96">
         <f>AF5</f>
         <v>45838</v>
       </c>
-      <c r="AG4" s="49"/>
-      <c r="AH4" s="49"/>
-      <c r="AI4" s="49"/>
-      <c r="AJ4" s="49"/>
-      <c r="AK4" s="49"/>
-      <c r="AL4" s="50"/>
-      <c r="AM4" s="48">
+      <c r="AG4" s="97"/>
+      <c r="AH4" s="97"/>
+      <c r="AI4" s="97"/>
+      <c r="AJ4" s="97"/>
+      <c r="AK4" s="97"/>
+      <c r="AL4" s="98"/>
+      <c r="AM4" s="96">
         <f>AM5</f>
         <v>45845</v>
       </c>
-      <c r="AN4" s="49"/>
-      <c r="AO4" s="49"/>
-      <c r="AP4" s="49"/>
-      <c r="AQ4" s="49"/>
-      <c r="AR4" s="49"/>
-      <c r="AS4" s="50"/>
-      <c r="AT4" s="48">
+      <c r="AN4" s="97"/>
+      <c r="AO4" s="97"/>
+      <c r="AP4" s="97"/>
+      <c r="AQ4" s="97"/>
+      <c r="AR4" s="97"/>
+      <c r="AS4" s="98"/>
+      <c r="AT4" s="96">
         <f>AT5</f>
         <v>45852</v>
       </c>
-      <c r="AU4" s="49"/>
-      <c r="AV4" s="49"/>
-      <c r="AW4" s="49"/>
-      <c r="AX4" s="49"/>
-      <c r="AY4" s="49"/>
-      <c r="AZ4" s="50"/>
-      <c r="BA4" s="48">
+      <c r="AU4" s="97"/>
+      <c r="AV4" s="97"/>
+      <c r="AW4" s="97"/>
+      <c r="AX4" s="97"/>
+      <c r="AY4" s="97"/>
+      <c r="AZ4" s="98"/>
+      <c r="BA4" s="96">
         <f>BA5</f>
         <v>45859</v>
       </c>
-      <c r="BB4" s="49"/>
-      <c r="BC4" s="49"/>
-      <c r="BD4" s="49"/>
-      <c r="BE4" s="49"/>
-      <c r="BF4" s="49"/>
-      <c r="BG4" s="50"/>
-      <c r="BH4" s="48">
+      <c r="BB4" s="97"/>
+      <c r="BC4" s="97"/>
+      <c r="BD4" s="97"/>
+      <c r="BE4" s="97"/>
+      <c r="BF4" s="97"/>
+      <c r="BG4" s="98"/>
+      <c r="BH4" s="96">
         <f>BH5</f>
         <v>45866</v>
       </c>
-      <c r="BI4" s="49"/>
-      <c r="BJ4" s="49"/>
-      <c r="BK4" s="49"/>
-      <c r="BL4" s="49"/>
-      <c r="BM4" s="49"/>
-      <c r="BN4" s="50"/>
+      <c r="BI4" s="97"/>
+      <c r="BJ4" s="97"/>
+      <c r="BK4" s="97"/>
+      <c r="BL4" s="97"/>
+      <c r="BM4" s="97"/>
+      <c r="BN4" s="98"/>
     </row>
     <row r="5" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="102"/>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
       <c r="K5" s="21">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -2610,13 +2543,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C6" s="33" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>34</v>
@@ -2863,8 +2796,8 @@
       <c r="A7" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
       <c r="G7" s="1"/>
       <c r="J7" s="1" t="str">
         <f>IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
@@ -2931,15 +2864,15 @@
       <c r="A8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="77" t="s">
+      <c r="B8" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="77"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="78"/>
-      <c r="F8" s="79"/>
-      <c r="G8" s="80"/>
-      <c r="H8" s="81"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="74"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5" t="str">
         <f t="shared" ref="J8:J46" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
@@ -3005,23 +2938,23 @@
     <row r="9" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="38"/>
       <c r="B9" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="54" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="55" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="47" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="55"/>
+      <c r="E9" s="48"/>
       <c r="F9" s="7">
         <v>0.3</v>
       </c>
-      <c r="G9" s="56">
+      <c r="G9" s="49">
         <f>G22+1</f>
         <v>45830</v>
       </c>
-      <c r="H9" s="56">
+      <c r="H9" s="49">
         <f>G9+4</f>
         <v>45834</v>
       </c>
@@ -3088,24 +3021,24 @@
       <c r="BN9" s="13"/>
     </row>
     <row r="10" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="76" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" s="54" t="s">
+      <c r="B10" s="69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="55" t="s">
+      <c r="D10" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="55"/>
+      <c r="E10" s="48"/>
       <c r="F10" s="7">
         <v>0.1</v>
       </c>
-      <c r="G10" s="56">
+      <c r="G10" s="49">
         <f>G9+2</f>
         <v>45832</v>
       </c>
-      <c r="H10" s="56">
+      <c r="H10" s="49">
         <f>G10+5</f>
         <v>45837</v>
       </c>
@@ -3172,24 +3105,24 @@
       <c r="BN10" s="13"/>
     </row>
     <row r="11" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="75" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="54" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="55" t="s">
+      <c r="B11" s="68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="55"/>
+      <c r="E11" s="48"/>
       <c r="F11" s="7">
         <v>0.5</v>
       </c>
-      <c r="G11" s="56">
+      <c r="G11" s="49">
         <f>H10</f>
         <v>45837</v>
       </c>
-      <c r="H11" s="56">
+      <c r="H11" s="49">
         <f>G11+3</f>
         <v>45840</v>
       </c>
@@ -3256,24 +3189,24 @@
       <c r="BN11" s="13"/>
     </row>
     <row r="12" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="75" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="54" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="55" t="s">
+      <c r="B12" s="68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="55"/>
+      <c r="E12" s="48"/>
       <c r="F12" s="7">
         <v>0.8</v>
       </c>
-      <c r="G12" s="56">
+      <c r="G12" s="49">
         <f>G11</f>
         <v>45837</v>
       </c>
-      <c r="H12" s="56">
+      <c r="H12" s="49">
         <f>G12+2</f>
         <v>45839</v>
       </c>
@@ -3343,15 +3276,15 @@
       <c r="A13" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="82" t="s">
+      <c r="B13" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="82"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="84"/>
-      <c r="G13" s="85"/>
-      <c r="H13" s="86"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="76"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="78"/>
+      <c r="H13" s="79"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5" t="str">
         <f t="shared" si="6"/>
@@ -3419,23 +3352,23 @@
         <v>8</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="57" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" s="58" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="58"/>
+      <c r="E14" s="51"/>
       <c r="F14" s="6">
         <v>0.8</v>
       </c>
-      <c r="G14" s="59">
+      <c r="G14" s="52">
         <f>InicioDelProyecto</f>
         <v>45822</v>
       </c>
-      <c r="H14" s="59">
+      <c r="H14" s="52">
         <f>G14+6</f>
         <v>45828</v>
       </c>
@@ -3503,23 +3436,23 @@
     </row>
     <row r="15" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="38"/>
-      <c r="B15" s="76" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="57" t="s">
+      <c r="B15" s="69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="58" t="s">
+      <c r="D15" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="58"/>
+      <c r="E15" s="51"/>
       <c r="F15" s="6">
         <v>0.8</v>
       </c>
-      <c r="G15" s="59">
+      <c r="G15" s="52">
         <v>45837</v>
       </c>
-      <c r="H15" s="59">
+      <c r="H15" s="52">
         <v>45837</v>
       </c>
       <c r="I15" s="5"/>
@@ -3583,25 +3516,25 @@
     </row>
     <row r="16" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="38"/>
-      <c r="B16" s="75" t="s">
-        <v>84</v>
-      </c>
-      <c r="C16" s="57" t="s">
+      <c r="B16" s="68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="58" t="s">
+      <c r="D16" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="58" t="s">
+      <c r="E16" s="51" t="s">
         <v>53</v>
       </c>
       <c r="F16" s="6">
         <v>0.1</v>
       </c>
-      <c r="G16" s="59">
+      <c r="G16" s="52">
         <v>45851</v>
       </c>
-      <c r="H16" s="59">
+      <c r="H16" s="52">
         <f>G16+6</f>
         <v>45857</v>
       </c>
@@ -3666,25 +3599,25 @@
     </row>
     <row r="17" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="38"/>
-      <c r="B17" s="75" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="57" t="s">
+      <c r="B17" s="68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="58" t="s">
+      <c r="D17" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="58" t="s">
+      <c r="E17" s="51" t="s">
         <v>50</v>
       </c>
       <c r="F17" s="6">
         <v>0.2</v>
       </c>
-      <c r="G17" s="59">
+      <c r="G17" s="52">
         <v>45837</v>
       </c>
-      <c r="H17" s="59"/>
+      <c r="H17" s="52"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="13"/>
@@ -3747,21 +3680,21 @@
     <row r="18" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="38"/>
       <c r="B18" s="34"/>
-      <c r="C18" s="57" t="s">
+      <c r="C18" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="58" t="s">
+      <c r="D18" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="58"/>
+      <c r="E18" s="51"/>
       <c r="F18" s="6">
         <v>0</v>
       </c>
-      <c r="G18" s="59">
+      <c r="G18" s="52">
         <f>H14</f>
         <v>45828</v>
       </c>
-      <c r="H18" s="59">
+      <c r="H18" s="52">
         <f>G18+2</f>
         <v>45830</v>
       </c>
@@ -3829,21 +3762,21 @@
         <v>9</v>
       </c>
       <c r="B19" s="34"/>
-      <c r="C19" s="57" t="s">
+      <c r="C19" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="58" t="s">
+      <c r="D19" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="58"/>
+      <c r="E19" s="51"/>
       <c r="F19" s="6">
         <v>0</v>
       </c>
-      <c r="G19" s="59">
+      <c r="G19" s="52">
         <f>H18</f>
         <v>45830</v>
       </c>
-      <c r="H19" s="59">
+      <c r="H19" s="52">
         <f>G19+4</f>
         <v>45834</v>
       </c>
@@ -3911,21 +3844,21 @@
     </row>
     <row r="20" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="34"/>
-      <c r="C20" s="57" t="s">
+      <c r="C20" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="58" t="s">
+      <c r="D20" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="58"/>
+      <c r="E20" s="51"/>
       <c r="F20" s="6">
         <v>0.5</v>
       </c>
-      <c r="G20" s="59">
+      <c r="G20" s="52">
         <f>H19</f>
         <v>45834</v>
       </c>
-      <c r="H20" s="59">
+      <c r="H20" s="52">
         <f>G20+4</f>
         <v>45838</v>
       </c>
@@ -3992,24 +3925,24 @@
       <c r="BN20" s="13"/>
     </row>
     <row r="21" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="76" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="57" t="s">
+      <c r="B21" s="69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="58" t="s">
+      <c r="D21" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="58"/>
+      <c r="E21" s="51"/>
       <c r="F21" s="6">
         <v>0.3</v>
       </c>
-      <c r="G21" s="59">
+      <c r="G21" s="52">
         <f>H19</f>
         <v>45834</v>
       </c>
-      <c r="H21" s="59">
+      <c r="H21" s="52">
         <f>G21+5</f>
         <v>45839</v>
       </c>
@@ -4074,23 +4007,23 @@
     </row>
     <row r="22" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C22" s="57" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="58" t="s">
+      <c r="D22" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="58"/>
+      <c r="E22" s="51"/>
       <c r="F22" s="6">
         <v>0</v>
       </c>
-      <c r="G22" s="59">
+      <c r="G22" s="52">
         <f>G18+1</f>
         <v>45829</v>
       </c>
-      <c r="H22" s="59">
+      <c r="H22" s="52">
         <f>G22+2</f>
         <v>45831</v>
       </c>
@@ -4157,21 +4090,21 @@
       <c r="BN22" s="13"/>
     </row>
     <row r="23" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="76" t="s">
-        <v>83</v>
-      </c>
-      <c r="C23" s="57" t="s">
+      <c r="B23" s="69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="58" t="s">
+      <c r="D23" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="E23" s="58" t="s">
+      <c r="E23" s="51" t="s">
         <v>64</v>
       </c>
       <c r="F23" s="6"/>
-      <c r="G23" s="59"/>
-      <c r="H23" s="59"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5" t="str">
         <f t="shared" si="6"/>
@@ -4235,15 +4168,15 @@
       <c r="BN23" s="13"/>
     </row>
     <row r="24" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="87" t="s">
-        <v>78</v>
-      </c>
-      <c r="C24" s="87"/>
-      <c r="D24" s="88"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="89"/>
-      <c r="G24" s="90"/>
-      <c r="H24" s="91"/>
+      <c r="B24" s="80" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="80"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="83"/>
+      <c r="H24" s="84"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5" t="str">
         <f t="shared" si="6"/>
@@ -4308,24 +4241,24 @@
     </row>
     <row r="25" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C25" s="60" t="s">
-        <v>86</v>
-      </c>
-      <c r="D25" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="61" t="s">
+      <c r="E25" s="54" t="s">
         <v>57</v>
       </c>
       <c r="F25" s="25">
         <v>1</v>
       </c>
-      <c r="G25" s="62">
+      <c r="G25" s="55">
         <v>45858</v>
       </c>
-      <c r="H25" s="62">
+      <c r="H25" s="55">
         <f>G25+4</f>
         <v>45862</v>
       </c>
@@ -4393,24 +4326,24 @@
     </row>
     <row r="26" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C26" s="60" t="s">
-        <v>87</v>
-      </c>
-      <c r="D26" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="E26" s="61" t="s">
+      <c r="E26" s="54" t="s">
         <v>57</v>
       </c>
       <c r="F26" s="25">
         <v>1</v>
       </c>
-      <c r="G26" s="62">
+      <c r="G26" s="55">
         <v>45858</v>
       </c>
-      <c r="H26" s="62">
+      <c r="H26" s="55">
         <f>G26+4</f>
         <v>45862</v>
       </c>
@@ -4478,24 +4411,24 @@
     </row>
     <row r="27" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C27" s="60" t="s">
-        <v>89</v>
-      </c>
-      <c r="D27" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="53" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="E27" s="61" t="s">
+      <c r="E27" s="54" t="s">
         <v>59</v>
       </c>
       <c r="F27" s="25">
         <v>1</v>
       </c>
-      <c r="G27" s="62">
+      <c r="G27" s="55">
         <v>45829</v>
       </c>
-      <c r="H27" s="62">
+      <c r="H27" s="55">
         <v>45829</v>
       </c>
       <c r="I27" s="5"/>
@@ -4562,25 +4495,25 @@
     </row>
     <row r="28" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28" s="60" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="53" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="E28" s="61" t="s">
+      <c r="E28" s="54" t="s">
         <v>56</v>
       </c>
       <c r="F28" s="25">
         <v>1</v>
       </c>
-      <c r="G28" s="62">
+      <c r="G28" s="55">
         <f>H27+1</f>
         <v>45830</v>
       </c>
-      <c r="H28" s="62">
+      <c r="H28" s="55">
         <f>G28+4</f>
         <v>45834</v>
       </c>
@@ -4647,23 +4580,25 @@
       <c r="BN28" s="13"/>
     </row>
     <row r="29" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="35"/>
-      <c r="C29" s="60" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="61" t="s">
+      <c r="B29" s="68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="54" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="61" t="s">
+      <c r="E29" s="54" t="s">
         <v>60</v>
       </c>
       <c r="F29" s="25">
         <v>1</v>
       </c>
-      <c r="G29" s="62">
+      <c r="G29" s="55">
         <v>45858</v>
       </c>
-      <c r="H29" s="62">
+      <c r="H29" s="55">
         <v>45858</v>
       </c>
       <c r="I29" s="5"/>
@@ -4727,20 +4662,20 @@
     </row>
     <row r="30" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="35"/>
-      <c r="C30" s="60" t="s">
-        <v>88</v>
-      </c>
-      <c r="D30" s="61"/>
-      <c r="E30" s="61" t="s">
-        <v>72</v>
+      <c r="C30" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" s="54"/>
+      <c r="E30" s="54" t="s">
+        <v>71</v>
       </c>
       <c r="F30" s="25">
         <v>0</v>
       </c>
-      <c r="G30" s="62">
+      <c r="G30" s="55">
         <v>0</v>
       </c>
-      <c r="H30" s="62">
+      <c r="H30" s="55">
         <v>0</v>
       </c>
       <c r="I30" s="5"/>
@@ -4804,14 +4739,14 @@
     </row>
     <row r="31" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="35"/>
-      <c r="C31" s="60" t="s">
-        <v>92</v>
-      </c>
-      <c r="D31" s="61"/>
-      <c r="E31" s="61"/>
+      <c r="C31" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="D31" s="54"/>
+      <c r="E31" s="54"/>
       <c r="F31" s="25"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="62"/>
+      <c r="G31" s="55"/>
+      <c r="H31" s="55"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="13"/>
@@ -4872,23 +4807,23 @@
       <c r="BN31" s="13"/>
     </row>
     <row r="32" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="76" t="s">
-        <v>83</v>
-      </c>
-      <c r="C32" s="60" t="s">
-        <v>93</v>
-      </c>
-      <c r="D32" s="61"/>
-      <c r="E32" s="61" t="s">
-        <v>71</v>
+      <c r="B32" s="69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" s="54"/>
+      <c r="E32" s="54" t="s">
+        <v>70</v>
       </c>
       <c r="F32" s="25">
         <v>0</v>
       </c>
-      <c r="G32" s="62">
+      <c r="G32" s="55">
         <v>0</v>
       </c>
-      <c r="H32" s="62">
+      <c r="H32" s="55">
         <v>0</v>
       </c>
       <c r="I32" s="5"/>
@@ -4954,15 +4889,15 @@
       <c r="BN32" s="13"/>
     </row>
     <row r="33" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="92" t="s">
-        <v>79</v>
-      </c>
-      <c r="C33" s="92"/>
-      <c r="D33" s="93"/>
-      <c r="E33" s="93"/>
-      <c r="F33" s="94"/>
-      <c r="G33" s="95"/>
-      <c r="H33" s="96"/>
+      <c r="B33" s="85" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="85"/>
+      <c r="D33" s="86"/>
+      <c r="E33" s="86"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="88"/>
+      <c r="H33" s="89"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5" t="str">
         <f t="shared" si="6"/>
@@ -5027,24 +4962,24 @@
     </row>
     <row r="34" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="102" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="95" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="63" t="s">
+      <c r="D34" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="E34" s="63" t="s">
+      <c r="E34" s="56" t="s">
         <v>67</v>
       </c>
       <c r="F34" s="8">
         <v>1</v>
       </c>
-      <c r="G34" s="64">
+      <c r="G34" s="57">
         <v>45829</v>
       </c>
-      <c r="H34" s="64">
+      <c r="H34" s="57">
         <v>45829</v>
       </c>
       <c r="I34" s="5"/>
@@ -5108,25 +5043,25 @@
     </row>
     <row r="35" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C35" s="102" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="95" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="63" t="s">
+      <c r="D35" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="E35" s="63" t="s">
+      <c r="E35" s="56" t="s">
         <v>61</v>
       </c>
       <c r="F35" s="8">
         <v>1</v>
       </c>
-      <c r="G35" s="64">
+      <c r="G35" s="57">
         <f>G14+15</f>
         <v>45837</v>
       </c>
-      <c r="H35" s="64">
+      <c r="H35" s="57">
         <f>G35+5</f>
         <v>45842</v>
       </c>
@@ -5194,24 +5129,24 @@
     </row>
     <row r="36" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C36" s="102" t="s">
+        <v>80</v>
+      </c>
+      <c r="C36" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="63" t="s">
+      <c r="D36" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="63" t="s">
+      <c r="E36" s="56" t="s">
         <v>35</v>
       </c>
       <c r="F36" s="8">
         <v>1</v>
       </c>
-      <c r="G36" s="64">
+      <c r="G36" s="57">
         <v>45829</v>
       </c>
-      <c r="H36" s="64">
+      <c r="H36" s="57">
         <v>45829</v>
       </c>
       <c r="I36" s="5"/>
@@ -5275,24 +5210,24 @@
     </row>
     <row r="37" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C37" s="102" t="s">
+        <v>80</v>
+      </c>
+      <c r="C37" s="95" t="s">
         <v>33</v>
       </c>
-      <c r="D37" s="63" t="s">
+      <c r="D37" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="E37" s="63" t="s">
+      <c r="E37" s="56" t="s">
         <v>54</v>
       </c>
       <c r="F37" s="8">
         <v>1</v>
       </c>
-      <c r="G37" s="64">
+      <c r="G37" s="57">
         <v>45837</v>
       </c>
-      <c r="H37" s="64">
+      <c r="H37" s="57">
         <v>45851</v>
       </c>
       <c r="I37" s="5"/>
@@ -5358,21 +5293,21 @@
       <c r="BN37" s="13"/>
     </row>
     <row r="38" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="76" t="s">
-        <v>83</v>
-      </c>
-      <c r="C38" s="65" t="s">
+      <c r="B38" s="69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="63" t="s">
+      <c r="D38" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="E38" s="63" t="s">
-        <v>70</v>
+      <c r="E38" s="56" t="s">
+        <v>93</v>
       </c>
       <c r="F38" s="8"/>
-      <c r="G38" s="64"/>
-      <c r="H38" s="64"/>
+      <c r="G38" s="57"/>
+      <c r="H38" s="57"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5" t="str">
         <f t="shared" si="6"/>
@@ -5436,15 +5371,15 @@
       <c r="BN38" s="13"/>
     </row>
     <row r="39" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="97" t="s">
-        <v>80</v>
-      </c>
-      <c r="C39" s="97"/>
-      <c r="D39" s="98"/>
-      <c r="E39" s="98"/>
-      <c r="F39" s="99"/>
-      <c r="G39" s="100"/>
-      <c r="H39" s="101"/>
+      <c r="B39" s="90" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" s="90"/>
+      <c r="D39" s="91"/>
+      <c r="E39" s="91"/>
+      <c r="F39" s="92"/>
+      <c r="G39" s="93"/>
+      <c r="H39" s="94"/>
       <c r="I39" s="5"/>
       <c r="J39" s="5" t="str">
         <f t="shared" si="6"/>
@@ -5509,22 +5444,22 @@
     </row>
     <row r="40" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C40" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="D40" s="67" t="s">
+        <v>80</v>
+      </c>
+      <c r="C40" s="59" t="s">
+        <v>84</v>
+      </c>
+      <c r="D40" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="E40" s="67"/>
+      <c r="E40" s="60"/>
       <c r="F40" s="9">
         <v>1</v>
       </c>
-      <c r="G40" s="68">
+      <c r="G40" s="61">
         <v>45837</v>
       </c>
-      <c r="H40" s="68">
+      <c r="H40" s="61">
         <v>45837</v>
       </c>
       <c r="I40" s="5"/>
@@ -5588,24 +5523,24 @@
     </row>
     <row r="41" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C41" s="66" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="59" t="s">
         <v>37</v>
       </c>
-      <c r="D41" s="67" t="s">
+      <c r="D41" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="E41" s="67" t="s">
+      <c r="E41" s="60" t="s">
         <v>44</v>
       </c>
       <c r="F41" s="9">
         <v>1</v>
       </c>
-      <c r="G41" s="68">
+      <c r="G41" s="61">
         <v>45837</v>
       </c>
-      <c r="H41" s="68">
+      <c r="H41" s="61">
         <v>45837</v>
       </c>
       <c r="I41" s="5"/>
@@ -5672,22 +5607,22 @@
     </row>
     <row r="42" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="66" t="s">
+        <v>80</v>
+      </c>
+      <c r="C42" s="59" t="s">
         <v>38</v>
       </c>
-      <c r="D42" s="67" t="s">
+      <c r="D42" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="E42" s="67"/>
+      <c r="E42" s="60"/>
       <c r="F42" s="9">
         <v>1</v>
       </c>
-      <c r="G42" s="68">
+      <c r="G42" s="61">
         <v>45837</v>
       </c>
-      <c r="H42" s="68">
+      <c r="H42" s="61">
         <v>45837</v>
       </c>
       <c r="I42" s="5"/>
@@ -5754,22 +5689,22 @@
     </row>
     <row r="43" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C43" s="66" t="s">
+        <v>80</v>
+      </c>
+      <c r="C43" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="D43" s="67" t="s">
+      <c r="D43" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="E43" s="67"/>
+      <c r="E43" s="60"/>
       <c r="F43" s="9">
         <v>1</v>
       </c>
-      <c r="G43" s="68">
+      <c r="G43" s="61">
         <v>45837</v>
       </c>
-      <c r="H43" s="68">
+      <c r="H43" s="61">
         <v>45837</v>
       </c>
       <c r="I43" s="5"/>
@@ -5836,20 +5771,20 @@
     </row>
     <row r="44" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="36"/>
-      <c r="C44" s="66" t="s">
+      <c r="C44" s="59" t="s">
         <v>43</v>
       </c>
-      <c r="D44" s="67" t="s">
+      <c r="D44" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="E44" s="67"/>
+      <c r="E44" s="60"/>
       <c r="F44" s="9">
         <v>1</v>
       </c>
-      <c r="G44" s="68">
+      <c r="G44" s="61">
         <v>45837</v>
       </c>
-      <c r="H44" s="68">
+      <c r="H44" s="61">
         <v>45837</v>
       </c>
       <c r="I44" s="5"/>
@@ -5916,20 +5851,20 @@
     </row>
     <row r="45" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B45" s="36"/>
-      <c r="C45" s="66" t="s">
+      <c r="C45" s="59" t="s">
         <v>41</v>
       </c>
-      <c r="D45" s="67" t="s">
+      <c r="D45" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="E45" s="67" t="s">
+      <c r="E45" s="60" t="s">
         <v>45</v>
       </c>
       <c r="F45" s="9">
         <v>0</v>
       </c>
-      <c r="G45" s="68"/>
-      <c r="H45" s="68"/>
+      <c r="G45" s="61"/>
+      <c r="H45" s="61"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5" t="str">
         <f t="shared" si="6"/>
@@ -5997,12 +5932,12 @@
         <v>11</v>
       </c>
       <c r="B46" s="37"/>
-      <c r="C46" s="69"/>
-      <c r="D46" s="70"/>
-      <c r="E46" s="70"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="63"/>
       <c r="F46" s="4"/>
-      <c r="G46" s="71"/>
-      <c r="H46" s="71"/>
+      <c r="G46" s="64"/>
+      <c r="H46" s="64"/>
       <c r="I46" s="12"/>
       <c r="J46" s="12" t="str">
         <f t="shared" si="6"/>
@@ -6067,7 +6002,7 @@
     </row>
     <row r="47" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="10"/>
-      <c r="C47" s="72" t="s">
+      <c r="C47" s="65" t="s">
         <v>13</v>
       </c>
       <c r="D47" s="10"/>
@@ -6078,9 +6013,9 @@
       <c r="I47" s="2"/>
     </row>
     <row r="49" spans="4:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D49" s="73"/>
-      <c r="E49" s="73"/>
-      <c r="H49" s="74"/>
+      <c r="D49" s="66"/>
+      <c r="E49" s="66"/>
+      <c r="H49" s="67"/>
     </row>
     <row r="50" spans="4:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D50" s="44"/>
@@ -6088,6 +6023,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="AM4:AS4"/>
+    <mergeCell ref="AT4:AZ4"/>
     <mergeCell ref="BA4:BG4"/>
     <mergeCell ref="BH4:BN4"/>
     <mergeCell ref="G3:H3"/>
@@ -6095,11 +6035,6 @@
     <mergeCell ref="R4:X4"/>
     <mergeCell ref="Y4:AE4"/>
     <mergeCell ref="AF4:AL4"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="AM4:AS4"/>
-    <mergeCell ref="AT4:AZ4"/>
   </mergeCells>
   <conditionalFormatting sqref="F7:F47">
     <cfRule type="dataBar" priority="16">

</xml_diff>

<commit_message>
IMPORTANT!!, Users Student Cand login in the page to watch all annotations he has created, UI images, Font Awesome .Icons change, Filters to Student Implemented, Search for Last name, First name, Grade,DNI,Change Rol Users Permisos, for Delete and Update, Student,Disable Option to update Inputs Obligatorio
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,17 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FADECF-D3F2-49A8-8608-46701CD2A9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8AF2DD9-62C5-49C9-8744-284E21B32FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="calendarioproyecto" sheetId="11" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="12" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="CIQWBGuid" hidden="1">"2cd8126d-26c3-430c-b7fa-a069e3a1fc62"</definedName>
@@ -84,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="133">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -209,9 +210,6 @@
     <t>Jose Miguel Alvarez Fagua</t>
   </si>
   <si>
-    <t>Jose Miguel Alvarez</t>
-  </si>
-  <si>
     <t>Backend</t>
   </si>
   <si>
@@ -326,9 +324,6 @@
     <t>Permitir dejar campos vacios</t>
   </si>
   <si>
-    <t>Juddy</t>
-  </si>
-  <si>
     <t>Asignacion de Permisos</t>
   </si>
   <si>
@@ -420,6 +415,129 @@
   </si>
   <si>
     <t>Cuando solo admite 1 GB como maximo</t>
+  </si>
+  <si>
+    <t>Prioridad</t>
+  </si>
+  <si>
+    <t>Tarea</t>
+  </si>
+  <si>
+    <t>Progreso</t>
+  </si>
+  <si>
+    <t>Inicio</t>
+  </si>
+  <si>
+    <t>Fin</t>
+  </si>
+  <si>
+    <t>Reasignar fotos de usuarios</t>
+  </si>
+  <si>
+    <t>Diseño de estructura de página web</t>
+  </si>
+  <si>
+    <t>Optimización de código CSS/HTML</t>
+  </si>
+  <si>
+    <t>Fin del proyecto:</t>
+  </si>
+  <si>
+    <t>Validación de redireccionamiento (href)</t>
+  </si>
+  <si>
+    <t>Revisión de permisos</t>
+  </si>
+  <si>
+    <t>Guardado con campos vacíos (Insert User)</t>
+  </si>
+  <si>
+    <t>Permisos en header (Profesor)</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Error en modificar</t>
+  </si>
+  <si>
+    <t>Validación general del backend</t>
+  </si>
+  <si>
+    <t>Actualización de datos estudiantiles</t>
+  </si>
+  <si>
+    <t>Revisión de consultas SQL</t>
+  </si>
+  <si>
+    <t>Organización de estructura MVC</t>
+  </si>
+  <si>
+    <t>Asignación de permisos por usuario</t>
+  </si>
+  <si>
+    <t>Leer datos de anotaciones</t>
+  </si>
+  <si>
+    <t>Actualizar datos de anotaciones</t>
+  </si>
+  <si>
+    <t>Eliminar anotaciones</t>
+  </si>
+  <si>
+    <t>Crear anotaciones con trigger</t>
+  </si>
+  <si>
+    <t>Trigger de anotaciones</t>
+  </si>
+  <si>
+    <t>Firma del estudiante (checkbox)</t>
+  </si>
+  <si>
+    <t>Notificación a acudiente por correo</t>
+  </si>
+  <si>
+    <t>Anotaciones</t>
+  </si>
+  <si>
+    <t>Estudiantes</t>
+  </si>
+  <si>
+    <t>Leer datos de estudiantes</t>
+  </si>
+  <si>
+    <t>Actualizar datos (permitir campos vacíos)</t>
+  </si>
+  <si>
+    <t>Eliminar datos de estudiantes</t>
+  </si>
+  <si>
+    <t>Crear datos con claves foráneas</t>
+  </si>
+  <si>
+    <t>Docentes</t>
+  </si>
+  <si>
+    <t>Leer datos de profesores</t>
+  </si>
+  <si>
+    <t>Actualizar datos (procedure)</t>
+  </si>
+  <si>
+    <t>Eliminar datos de profesores</t>
+  </si>
+  <si>
+    <t>Crear datos de profesores</t>
+  </si>
+  <si>
+    <t>Guardado de imágenes de profesores</t>
+  </si>
+  <si>
+    <t>Trigger para profesores</t>
+  </si>
+  <si>
+    <t>Guardado de imágenes de estudiantes</t>
   </si>
 </sst>
 </file>
@@ -667,7 +785,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="46">
+  <fills count="47">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -925,8 +1043,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -1126,6 +1250,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1199,7 +1347,7 @@
     <xf numFmtId="0" fontId="9" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1486,6 +1634,15 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1498,14 +1655,23 @@
     <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="46" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="55">
@@ -2147,10 +2313,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="42" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="43" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="34.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="43" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="60.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" style="1" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" style="43" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" style="1" customWidth="1"/>
@@ -2188,6 +2354,15 @@
       </c>
       <c r="B2" s="31"/>
       <c r="C2" s="26"/>
+      <c r="D2" s="96" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="96"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="102">
+        <v>45822</v>
+      </c>
+      <c r="H2" s="102"/>
       <c r="K2" s="44"/>
     </row>
     <row r="3" spans="1:66" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2198,121 +2373,121 @@
       <c r="C3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="100" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="100"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="99">
-        <v>45822</v>
-      </c>
-      <c r="H3" s="99"/>
+      <c r="D3" s="96" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="96"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="102">
+        <v>45931</v>
+      </c>
+      <c r="H3" s="102"/>
     </row>
     <row r="4" spans="1:66" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="100" t="s">
+      <c r="D4" s="96" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="100"/>
-      <c r="F4" s="101"/>
+      <c r="E4" s="96"/>
+      <c r="F4" s="97"/>
       <c r="G4" s="3">
-        <v>1</v>
-      </c>
-      <c r="K4" s="96">
+        <v>-15</v>
+      </c>
+      <c r="K4" s="99">
         <f>K5</f>
         <v>45817</v>
       </c>
-      <c r="L4" s="97"/>
-      <c r="M4" s="97"/>
-      <c r="N4" s="97"/>
-      <c r="O4" s="97"/>
-      <c r="P4" s="97"/>
-      <c r="Q4" s="98"/>
-      <c r="R4" s="96">
+      <c r="L4" s="100"/>
+      <c r="M4" s="100"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="100"/>
+      <c r="P4" s="100"/>
+      <c r="Q4" s="101"/>
+      <c r="R4" s="99">
         <f>R5</f>
         <v>45824</v>
       </c>
-      <c r="S4" s="97"/>
-      <c r="T4" s="97"/>
-      <c r="U4" s="97"/>
-      <c r="V4" s="97"/>
-      <c r="W4" s="97"/>
-      <c r="X4" s="98"/>
-      <c r="Y4" s="96">
+      <c r="S4" s="100"/>
+      <c r="T4" s="100"/>
+      <c r="U4" s="100"/>
+      <c r="V4" s="100"/>
+      <c r="W4" s="100"/>
+      <c r="X4" s="101"/>
+      <c r="Y4" s="99">
         <f>Y5</f>
         <v>45831</v>
       </c>
-      <c r="Z4" s="97"/>
-      <c r="AA4" s="97"/>
-      <c r="AB4" s="97"/>
-      <c r="AC4" s="97"/>
-      <c r="AD4" s="97"/>
-      <c r="AE4" s="98"/>
-      <c r="AF4" s="96">
+      <c r="Z4" s="100"/>
+      <c r="AA4" s="100"/>
+      <c r="AB4" s="100"/>
+      <c r="AC4" s="100"/>
+      <c r="AD4" s="100"/>
+      <c r="AE4" s="101"/>
+      <c r="AF4" s="99">
         <f>AF5</f>
         <v>45838</v>
       </c>
-      <c r="AG4" s="97"/>
-      <c r="AH4" s="97"/>
-      <c r="AI4" s="97"/>
-      <c r="AJ4" s="97"/>
-      <c r="AK4" s="97"/>
-      <c r="AL4" s="98"/>
-      <c r="AM4" s="96">
+      <c r="AG4" s="100"/>
+      <c r="AH4" s="100"/>
+      <c r="AI4" s="100"/>
+      <c r="AJ4" s="100"/>
+      <c r="AK4" s="100"/>
+      <c r="AL4" s="101"/>
+      <c r="AM4" s="99">
         <f>AM5</f>
         <v>45845</v>
       </c>
-      <c r="AN4" s="97"/>
-      <c r="AO4" s="97"/>
-      <c r="AP4" s="97"/>
-      <c r="AQ4" s="97"/>
-      <c r="AR4" s="97"/>
-      <c r="AS4" s="98"/>
-      <c r="AT4" s="96">
+      <c r="AN4" s="100"/>
+      <c r="AO4" s="100"/>
+      <c r="AP4" s="100"/>
+      <c r="AQ4" s="100"/>
+      <c r="AR4" s="100"/>
+      <c r="AS4" s="101"/>
+      <c r="AT4" s="99">
         <f>AT5</f>
         <v>45852</v>
       </c>
-      <c r="AU4" s="97"/>
-      <c r="AV4" s="97"/>
-      <c r="AW4" s="97"/>
-      <c r="AX4" s="97"/>
-      <c r="AY4" s="97"/>
-      <c r="AZ4" s="98"/>
-      <c r="BA4" s="96">
+      <c r="AU4" s="100"/>
+      <c r="AV4" s="100"/>
+      <c r="AW4" s="100"/>
+      <c r="AX4" s="100"/>
+      <c r="AY4" s="100"/>
+      <c r="AZ4" s="101"/>
+      <c r="BA4" s="99">
         <f>BA5</f>
         <v>45859</v>
       </c>
-      <c r="BB4" s="97"/>
-      <c r="BC4" s="97"/>
-      <c r="BD4" s="97"/>
-      <c r="BE4" s="97"/>
-      <c r="BF4" s="97"/>
-      <c r="BG4" s="98"/>
-      <c r="BH4" s="96">
+      <c r="BB4" s="100"/>
+      <c r="BC4" s="100"/>
+      <c r="BD4" s="100"/>
+      <c r="BE4" s="100"/>
+      <c r="BF4" s="100"/>
+      <c r="BG4" s="101"/>
+      <c r="BH4" s="99">
         <f>BH5</f>
         <v>45866</v>
       </c>
-      <c r="BI4" s="97"/>
-      <c r="BJ4" s="97"/>
-      <c r="BK4" s="97"/>
-      <c r="BL4" s="97"/>
-      <c r="BM4" s="97"/>
-      <c r="BN4" s="98"/>
+      <c r="BI4" s="100"/>
+      <c r="BJ4" s="100"/>
+      <c r="BK4" s="100"/>
+      <c r="BL4" s="100"/>
+      <c r="BM4" s="100"/>
+      <c r="BN4" s="101"/>
     </row>
     <row r="5" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="45"/>
-      <c r="C5" s="102"/>
-      <c r="D5" s="102"/>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102"/>
-      <c r="G5" s="102"/>
-      <c r="H5" s="102"/>
-      <c r="I5" s="102"/>
+      <c r="C5" s="98"/>
+      <c r="D5" s="98"/>
+      <c r="E5" s="98"/>
+      <c r="F5" s="98"/>
+      <c r="G5" s="98"/>
+      <c r="H5" s="98"/>
+      <c r="I5" s="98"/>
       <c r="K5" s="21">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -2543,16 +2718,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C6" s="33" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>16</v>
@@ -2865,7 +3040,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="70" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="70"/>
       <c r="D8" s="71"/>
@@ -2938,25 +3113,23 @@
     <row r="9" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="38"/>
       <c r="B9" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="48" t="s">
-        <v>62</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="D9" s="48"/>
       <c r="E9" s="48"/>
       <c r="F9" s="7">
         <v>0.3</v>
       </c>
       <c r="G9" s="49">
-        <f>G22+1</f>
-        <v>45830</v>
+        <f>G2+1</f>
+        <v>45823</v>
       </c>
       <c r="H9" s="49">
         <f>G9+4</f>
-        <v>45834</v>
+        <v>45827</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5">
@@ -3022,25 +3195,23 @@
     </row>
     <row r="10" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C10" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="48" t="s">
-        <v>23</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D10" s="48"/>
       <c r="E10" s="48"/>
       <c r="F10" s="7">
         <v>0.1</v>
       </c>
       <c r="G10" s="49">
         <f>G9+2</f>
-        <v>45832</v>
+        <v>45825</v>
       </c>
       <c r="H10" s="49">
         <f>G10+5</f>
-        <v>45837</v>
+        <v>45830</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5">
@@ -3106,25 +3277,23 @@
     </row>
     <row r="11" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="68" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C11" s="47" t="s">
-        <v>73</v>
-      </c>
-      <c r="D11" s="48" t="s">
-        <v>23</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="D11" s="48"/>
       <c r="E11" s="48"/>
       <c r="F11" s="7">
         <v>0.5</v>
       </c>
       <c r="G11" s="49">
         <f>H10</f>
-        <v>45837</v>
+        <v>45830</v>
       </c>
       <c r="H11" s="49">
         <f>G11+3</f>
-        <v>45840</v>
+        <v>45833</v>
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="5">
@@ -3190,25 +3359,23 @@
     </row>
     <row r="12" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="68" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C12" s="47" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="48" t="s">
-        <v>23</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="D12" s="48"/>
       <c r="E12" s="48"/>
       <c r="F12" s="7">
         <v>0.8</v>
       </c>
       <c r="G12" s="49">
         <f>G11</f>
-        <v>45837</v>
+        <v>45830</v>
       </c>
       <c r="H12" s="49">
         <f>G12+2</f>
-        <v>45839</v>
+        <v>45832</v>
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5">
@@ -3277,7 +3444,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="75" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="75"/>
       <c r="D13" s="76"/>
@@ -3352,25 +3519,23 @@
         <v>8</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="51" t="s">
-        <v>23</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="D14" s="51"/>
       <c r="E14" s="51"/>
       <c r="F14" s="6">
         <v>0.8</v>
       </c>
       <c r="G14" s="52">
         <f>InicioDelProyecto</f>
-        <v>45822</v>
+        <v>45931</v>
       </c>
       <c r="H14" s="52">
         <f>G14+6</f>
-        <v>45828</v>
+        <v>45937</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5">
@@ -3437,13 +3602,13 @@
     <row r="15" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="38"/>
       <c r="B15" s="69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C15" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="51" t="s">
         <v>46</v>
-      </c>
-      <c r="D15" s="51" t="s">
-        <v>47</v>
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="6">
@@ -3517,16 +3682,16 @@
     <row r="16" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="38"/>
       <c r="B16" s="68" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C16" s="50" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="51" t="s">
+      <c r="E16" s="51" t="s">
         <v>52</v>
-      </c>
-      <c r="E16" s="51" t="s">
-        <v>53</v>
       </c>
       <c r="F16" s="6">
         <v>0.1</v>
@@ -3600,16 +3765,16 @@
     <row r="17" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="38"/>
       <c r="B17" s="68" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C17" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="51" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="51" t="s">
         <v>49</v>
-      </c>
-      <c r="D17" s="51" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="51" t="s">
-        <v>50</v>
       </c>
       <c r="F17" s="6">
         <v>0.2</v>
@@ -3681,22 +3846,20 @@
       <c r="A18" s="38"/>
       <c r="B18" s="34"/>
       <c r="C18" s="50" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="51" t="s">
-        <v>23</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="D18" s="51"/>
       <c r="E18" s="51"/>
       <c r="F18" s="6">
         <v>0</v>
       </c>
       <c r="G18" s="52">
         <f>H14</f>
-        <v>45828</v>
+        <v>45937</v>
       </c>
       <c r="H18" s="52">
         <f>G18+2</f>
-        <v>45830</v>
+        <v>45939</v>
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
@@ -3763,22 +3926,20 @@
       </c>
       <c r="B19" s="34"/>
       <c r="C19" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="51" t="s">
-        <v>23</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D19" s="51"/>
       <c r="E19" s="51"/>
       <c r="F19" s="6">
         <v>0</v>
       </c>
       <c r="G19" s="52">
         <f>H18</f>
-        <v>45830</v>
+        <v>45939</v>
       </c>
       <c r="H19" s="52">
         <f>G19+4</f>
-        <v>45834</v>
+        <v>45943</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5">
@@ -3845,10 +4006,10 @@
     <row r="20" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="34"/>
       <c r="C20" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="51" t="s">
         <v>31</v>
-      </c>
-      <c r="D20" s="51" t="s">
-        <v>32</v>
       </c>
       <c r="E20" s="51"/>
       <c r="F20" s="6">
@@ -3856,11 +4017,11 @@
       </c>
       <c r="G20" s="52">
         <f>H19</f>
-        <v>45834</v>
+        <v>45943</v>
       </c>
       <c r="H20" s="52">
         <f>G20+4</f>
-        <v>45838</v>
+        <v>45947</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5">
@@ -3926,25 +4087,23 @@
     </row>
     <row r="21" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C21" s="50" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="51" t="s">
-        <v>23</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D21" s="51"/>
       <c r="E21" s="51"/>
       <c r="F21" s="6">
         <v>0.3</v>
       </c>
       <c r="G21" s="52">
         <f>H19</f>
-        <v>45834</v>
+        <v>45943</v>
       </c>
       <c r="H21" s="52">
         <f>G21+5</f>
-        <v>45839</v>
+        <v>45948</v>
       </c>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
@@ -4007,25 +4166,23 @@
     </row>
     <row r="22" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C22" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="D22" s="51" t="s">
-        <v>23</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="D22" s="51"/>
       <c r="E22" s="51"/>
       <c r="F22" s="6">
         <v>0</v>
       </c>
       <c r="G22" s="52">
         <f>G18+1</f>
-        <v>45829</v>
+        <v>45938</v>
       </c>
       <c r="H22" s="52">
         <f>G22+2</f>
-        <v>45831</v>
+        <v>45940</v>
       </c>
       <c r="I22" s="5"/>
       <c r="J22" s="5">
@@ -4091,16 +4248,16 @@
     </row>
     <row r="23" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C23" s="50" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="51" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="51" t="s">
-        <v>65</v>
-      </c>
       <c r="E23" s="51" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="52"/>
@@ -4169,7 +4326,7 @@
     </row>
     <row r="24" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="80" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C24" s="80"/>
       <c r="D24" s="81"/>
@@ -4241,16 +4398,16 @@
     </row>
     <row r="25" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C25" s="53" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D25" s="54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E25" s="54" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F25" s="25">
         <v>1</v>
@@ -4326,16 +4483,16 @@
     </row>
     <row r="26" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C26" s="53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D26" s="54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E26" s="54" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F26" s="25">
         <v>1</v>
@@ -4411,16 +4568,16 @@
     </row>
     <row r="27" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C27" s="53" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D27" s="54" t="s">
+        <v>57</v>
+      </c>
+      <c r="E27" s="54" t="s">
         <v>58</v>
-      </c>
-      <c r="E27" s="54" t="s">
-        <v>59</v>
       </c>
       <c r="F27" s="25">
         <v>1</v>
@@ -4495,16 +4652,16 @@
     </row>
     <row r="28" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C28" s="53" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D28" s="54" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" s="54" t="s">
         <v>55</v>
-      </c>
-      <c r="E28" s="54" t="s">
-        <v>56</v>
       </c>
       <c r="F28" s="25">
         <v>1</v>
@@ -4581,16 +4738,16 @@
     </row>
     <row r="29" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="68" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C29" s="53" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D29" s="54" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E29" s="54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F29" s="25">
         <v>1</v>
@@ -4663,11 +4820,11 @@
     <row r="30" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="35"/>
       <c r="C30" s="53" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D30" s="54"/>
       <c r="E30" s="54" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F30" s="25">
         <v>0</v>
@@ -4740,7 +4897,7 @@
     <row r="31" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="35"/>
       <c r="C31" s="53" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D31" s="54"/>
       <c r="E31" s="54"/>
@@ -4808,14 +4965,14 @@
     </row>
     <row r="32" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C32" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D32" s="54"/>
       <c r="E32" s="54" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F32" s="25">
         <v>0</v>
@@ -4890,7 +5047,7 @@
     </row>
     <row r="33" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="85" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C33" s="85"/>
       <c r="D33" s="86"/>
@@ -4962,16 +5119,16 @@
     </row>
     <row r="34" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C34" s="95" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D34" s="56" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E34" s="56" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F34" s="8">
         <v>1</v>
@@ -5043,27 +5200,27 @@
     </row>
     <row r="35" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C35" s="95" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="56" t="s">
-        <v>32</v>
-      </c>
       <c r="E35" s="56" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F35" s="8">
         <v>1</v>
       </c>
       <c r="G35" s="57">
         <f>G14+15</f>
-        <v>45837</v>
+        <v>45946</v>
       </c>
       <c r="H35" s="57">
         <f>G35+5</f>
-        <v>45842</v>
+        <v>45951</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5">
@@ -5129,16 +5286,16 @@
     </row>
     <row r="36" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C36" s="95" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D36" s="56" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E36" s="56" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F36" s="8">
         <v>1</v>
@@ -5210,16 +5367,14 @@
     </row>
     <row r="37" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C37" s="95" t="s">
-        <v>33</v>
-      </c>
-      <c r="D37" s="56" t="s">
-        <v>23</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="D37" s="56"/>
       <c r="E37" s="56" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F37" s="8">
         <v>1</v>
@@ -5294,16 +5449,16 @@
     </row>
     <row r="38" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C38" s="58" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D38" s="56" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E38" s="56" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F38" s="8"/>
       <c r="G38" s="57"/>
@@ -5372,7 +5527,7 @@
     </row>
     <row r="39" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="90" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C39" s="90"/>
       <c r="D39" s="91"/>
@@ -5444,13 +5599,13 @@
     </row>
     <row r="40" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C40" s="59" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D40" s="60" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E40" s="60"/>
       <c r="F40" s="9">
@@ -5523,16 +5678,16 @@
     </row>
     <row r="41" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C41" s="59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D41" s="60" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E41" s="60" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F41" s="9">
         <v>1</v>
@@ -5607,13 +5762,13 @@
     </row>
     <row r="42" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C42" s="59" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D42" s="60" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E42" s="60"/>
       <c r="F42" s="9">
@@ -5689,13 +5844,13 @@
     </row>
     <row r="43" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C43" s="59" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D43" s="60" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E43" s="60"/>
       <c r="F43" s="9">
@@ -5772,10 +5927,10 @@
     <row r="44" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="36"/>
       <c r="C44" s="59" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D44" s="60" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E44" s="60"/>
       <c r="F44" s="9">
@@ -5852,13 +6007,11 @@
     <row r="45" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B45" s="36"/>
       <c r="C45" s="59" t="s">
-        <v>41</v>
-      </c>
-      <c r="D45" s="60" t="s">
-        <v>23</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="D45" s="60"/>
       <c r="E45" s="60" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F45" s="9">
         <v>0</v>
@@ -6022,12 +6175,9 @@
       <c r="E50" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="AM4:AS4"/>
-    <mergeCell ref="AT4:AZ4"/>
+  <mergeCells count="14">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="G2:H2"/>
     <mergeCell ref="BA4:BG4"/>
     <mergeCell ref="BH4:BN4"/>
     <mergeCell ref="G3:H3"/>
@@ -6035,6 +6185,11 @@
     <mergeCell ref="R4:X4"/>
     <mergeCell ref="Y4:AE4"/>
     <mergeCell ref="AF4:AL4"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="AM4:AS4"/>
+    <mergeCell ref="AT4:AZ4"/>
   </mergeCells>
   <conditionalFormatting sqref="F7:F47">
     <cfRule type="dataBar" priority="16">
@@ -6063,7 +6218,7 @@
       <formula>AND(Fecha_final&gt;=K$5,Fecha_incio&lt;L$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Mostrar semana" prompt="Al cambiar este número, se desplazará la vista del diagrama de Gantt." sqref="G4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>1</formula1>
     </dataValidation>
@@ -6096,4 +6251,685 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B608EB8-DABD-4C00-A7D4-1124308B6A39}">
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="43" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" style="43" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="43" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.28515625" style="43" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.42578125" style="43"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="107" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="107"/>
+      <c r="C1" s="107"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="107"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="103" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="103" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="103" t="s">
+        <v>95</v>
+      </c>
+      <c r="E2" s="103" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="104" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="105">
+        <v>0.3</v>
+      </c>
+      <c r="D3" s="106">
+        <v>45830</v>
+      </c>
+      <c r="E3" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="104" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="105">
+        <v>0.8</v>
+      </c>
+      <c r="D4" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E4" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="104" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="105">
+        <v>0.8</v>
+      </c>
+      <c r="D5" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E5" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="107" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="107"/>
+      <c r="C7" s="107"/>
+      <c r="D7" s="107"/>
+      <c r="E7" s="107"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="103" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="103" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="103" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="103" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="104" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="105">
+        <v>0.8</v>
+      </c>
+      <c r="D9" s="106">
+        <v>45822</v>
+      </c>
+      <c r="E9" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="104" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="104" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="105">
+        <v>0.8</v>
+      </c>
+      <c r="D10" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E10" s="106">
+        <v>45837</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="104" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="105">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="106">
+        <v>45851</v>
+      </c>
+      <c r="E11" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="104" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="105">
+        <v>0.2</v>
+      </c>
+      <c r="D12" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E12" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="104" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="105">
+        <v>1</v>
+      </c>
+      <c r="D13" s="106">
+        <v>45828</v>
+      </c>
+      <c r="E13" s="106">
+        <v>45830</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="104" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" s="105">
+        <v>0</v>
+      </c>
+      <c r="D14" s="106">
+        <v>45830</v>
+      </c>
+      <c r="E14" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="104" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="105">
+        <v>1</v>
+      </c>
+      <c r="D15" s="106">
+        <v>45834</v>
+      </c>
+      <c r="E15" s="106">
+        <v>45838</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="104" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="104" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="105">
+        <v>0.5</v>
+      </c>
+      <c r="D16" s="106">
+        <v>45834</v>
+      </c>
+      <c r="E16" s="106">
+        <v>45839</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="104" t="s">
+        <v>110</v>
+      </c>
+      <c r="C17" s="105">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="106">
+        <v>45829</v>
+      </c>
+      <c r="E17" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="104" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="104" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="105">
+        <v>0.75</v>
+      </c>
+      <c r="D18" s="106">
+        <v>45829</v>
+      </c>
+      <c r="E18" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="108" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="108"/>
+      <c r="C20" s="108"/>
+      <c r="D20" s="108"/>
+      <c r="E20" s="108"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="103" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="103" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="103" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="103" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="104" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" s="105">
+        <v>1</v>
+      </c>
+      <c r="D22" s="106">
+        <v>45858</v>
+      </c>
+      <c r="E22" s="106">
+        <v>45862</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="104" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" s="105">
+        <v>1</v>
+      </c>
+      <c r="D23" s="106">
+        <v>45858</v>
+      </c>
+      <c r="E23" s="106">
+        <v>45862</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="104" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="105">
+        <v>1</v>
+      </c>
+      <c r="D24" s="106">
+        <v>45829</v>
+      </c>
+      <c r="E24" s="106">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B25" s="104" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="105">
+        <v>1</v>
+      </c>
+      <c r="D25" s="106">
+        <v>45830</v>
+      </c>
+      <c r="E25" s="106">
+        <v>45834</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" s="104" t="s">
+        <v>116</v>
+      </c>
+      <c r="C26" s="105">
+        <v>1</v>
+      </c>
+      <c r="D26" s="106">
+        <v>45858</v>
+      </c>
+      <c r="E26" s="106">
+        <v>45858</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="B27" s="104" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" s="105">
+        <v>0</v>
+      </c>
+      <c r="D27" s="106" t="s">
+        <v>105</v>
+      </c>
+      <c r="E27" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="104" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" s="104" t="s">
+        <v>118</v>
+      </c>
+      <c r="C28" s="105">
+        <v>0</v>
+      </c>
+      <c r="D28" s="106" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="107" t="s">
+        <v>120</v>
+      </c>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="107"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="103" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="103" t="s">
+        <v>94</v>
+      </c>
+      <c r="D31" s="103" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" s="103" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="104" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" s="105">
+        <v>1</v>
+      </c>
+      <c r="D32" s="106">
+        <v>45829</v>
+      </c>
+      <c r="E32" s="106">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="104" t="s">
+        <v>122</v>
+      </c>
+      <c r="C33" s="105">
+        <v>1</v>
+      </c>
+      <c r="D33" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E33" s="106">
+        <v>45842</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="104" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" s="105">
+        <v>1</v>
+      </c>
+      <c r="D34" s="106">
+        <v>45829</v>
+      </c>
+      <c r="E34" s="106">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="104" t="s">
+        <v>124</v>
+      </c>
+      <c r="C35" s="105">
+        <v>1</v>
+      </c>
+      <c r="D35" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E35" s="106">
+        <v>45851</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="104" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" s="104" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36" s="105">
+        <v>1</v>
+      </c>
+      <c r="D36" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E36" s="106">
+        <v>45851</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="107" t="s">
+        <v>125</v>
+      </c>
+      <c r="B38" s="107"/>
+      <c r="C38" s="107"/>
+      <c r="D38" s="107"/>
+      <c r="E38" s="107"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="103" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="103" t="s">
+        <v>94</v>
+      </c>
+      <c r="D39" s="103" t="s">
+        <v>95</v>
+      </c>
+      <c r="E39" s="103" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="104" t="s">
+        <v>126</v>
+      </c>
+      <c r="C40" s="105">
+        <v>1</v>
+      </c>
+      <c r="D40" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E40" s="106">
+        <v>45837</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="104" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" s="105">
+        <v>1</v>
+      </c>
+      <c r="D41" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E41" s="106">
+        <v>45837</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" s="104" t="s">
+        <v>128</v>
+      </c>
+      <c r="C42" s="105">
+        <v>1</v>
+      </c>
+      <c r="D42" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E42" s="106">
+        <v>45837</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="104" t="s">
+        <v>129</v>
+      </c>
+      <c r="C43" s="105">
+        <v>1</v>
+      </c>
+      <c r="D43" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E43" s="106">
+        <v>45837</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="104" t="s">
+        <v>78</v>
+      </c>
+      <c r="B44" s="104" t="s">
+        <v>130</v>
+      </c>
+      <c r="C44" s="105">
+        <v>1</v>
+      </c>
+      <c r="D44" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E44" s="106">
+        <v>45837</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="104" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" s="104" t="s">
+        <v>131</v>
+      </c>
+      <c r="C45" s="105">
+        <v>0</v>
+      </c>
+      <c r="D45" s="106">
+        <v>45837</v>
+      </c>
+      <c r="E45" s="106">
+        <v>45931</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A38:E38"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Create Documentation for the project,Diagram Class,Entity Relationship,Use Case All
</commit_message>
<xml_diff>
--- a/Diagrama Gantt.xlsx
+++ b/Diagrama Gantt.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8AF2DD9-62C5-49C9-8744-284E21B32FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41BA246-43C7-419C-B076-62022A5A6896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="calendarioproyecto" sheetId="11" r:id="rId1"/>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="135">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -538,6 +538,12 @@
   </si>
   <si>
     <t>Guardado de imágenes de estudiantes</t>
+  </si>
+  <si>
+    <t>Descargo del Estudiante</t>
+  </si>
+  <si>
+    <t>Permitir dejar compromisos del estudiante por anotacion</t>
   </si>
 </sst>
 </file>
@@ -1634,38 +1640,38 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="12" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="46" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="42" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="46" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2309,7 +2315,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BN50"/>
+  <dimension ref="A1:BN51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="42" customWidth="1"/>
@@ -2354,11 +2360,11 @@
       </c>
       <c r="B2" s="31"/>
       <c r="C2" s="26"/>
-      <c r="D2" s="96" t="s">
+      <c r="D2" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="96"/>
-      <c r="F2" s="97"/>
+      <c r="E2" s="100"/>
+      <c r="F2" s="101"/>
       <c r="G2" s="102">
         <v>45822</v>
       </c>
@@ -2373,11 +2379,11 @@
       <c r="C3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="96" t="s">
+      <c r="D3" s="100" t="s">
         <v>100</v>
       </c>
-      <c r="E3" s="96"/>
-      <c r="F3" s="97"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="101"/>
       <c r="G3" s="102">
         <v>45931</v>
       </c>
@@ -2387,107 +2393,107 @@
       <c r="A4" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="96" t="s">
+      <c r="D4" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="96"/>
-      <c r="F4" s="97"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="101"/>
       <c r="G4" s="3">
         <v>-15</v>
       </c>
-      <c r="K4" s="99">
+      <c r="K4" s="103">
         <f>K5</f>
         <v>45817</v>
       </c>
-      <c r="L4" s="100"/>
-      <c r="M4" s="100"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="100"/>
-      <c r="P4" s="100"/>
-      <c r="Q4" s="101"/>
-      <c r="R4" s="99">
+      <c r="L4" s="104"/>
+      <c r="M4" s="104"/>
+      <c r="N4" s="104"/>
+      <c r="O4" s="104"/>
+      <c r="P4" s="104"/>
+      <c r="Q4" s="105"/>
+      <c r="R4" s="103">
         <f>R5</f>
         <v>45824</v>
       </c>
-      <c r="S4" s="100"/>
-      <c r="T4" s="100"/>
-      <c r="U4" s="100"/>
-      <c r="V4" s="100"/>
-      <c r="W4" s="100"/>
-      <c r="X4" s="101"/>
-      <c r="Y4" s="99">
+      <c r="S4" s="104"/>
+      <c r="T4" s="104"/>
+      <c r="U4" s="104"/>
+      <c r="V4" s="104"/>
+      <c r="W4" s="104"/>
+      <c r="X4" s="105"/>
+      <c r="Y4" s="103">
         <f>Y5</f>
         <v>45831</v>
       </c>
-      <c r="Z4" s="100"/>
-      <c r="AA4" s="100"/>
-      <c r="AB4" s="100"/>
-      <c r="AC4" s="100"/>
-      <c r="AD4" s="100"/>
-      <c r="AE4" s="101"/>
-      <c r="AF4" s="99">
+      <c r="Z4" s="104"/>
+      <c r="AA4" s="104"/>
+      <c r="AB4" s="104"/>
+      <c r="AC4" s="104"/>
+      <c r="AD4" s="104"/>
+      <c r="AE4" s="105"/>
+      <c r="AF4" s="103">
         <f>AF5</f>
         <v>45838</v>
       </c>
-      <c r="AG4" s="100"/>
-      <c r="AH4" s="100"/>
-      <c r="AI4" s="100"/>
-      <c r="AJ4" s="100"/>
-      <c r="AK4" s="100"/>
-      <c r="AL4" s="101"/>
-      <c r="AM4" s="99">
+      <c r="AG4" s="104"/>
+      <c r="AH4" s="104"/>
+      <c r="AI4" s="104"/>
+      <c r="AJ4" s="104"/>
+      <c r="AK4" s="104"/>
+      <c r="AL4" s="105"/>
+      <c r="AM4" s="103">
         <f>AM5</f>
         <v>45845</v>
       </c>
-      <c r="AN4" s="100"/>
-      <c r="AO4" s="100"/>
-      <c r="AP4" s="100"/>
-      <c r="AQ4" s="100"/>
-      <c r="AR4" s="100"/>
-      <c r="AS4" s="101"/>
-      <c r="AT4" s="99">
+      <c r="AN4" s="104"/>
+      <c r="AO4" s="104"/>
+      <c r="AP4" s="104"/>
+      <c r="AQ4" s="104"/>
+      <c r="AR4" s="104"/>
+      <c r="AS4" s="105"/>
+      <c r="AT4" s="103">
         <f>AT5</f>
         <v>45852</v>
       </c>
-      <c r="AU4" s="100"/>
-      <c r="AV4" s="100"/>
-      <c r="AW4" s="100"/>
-      <c r="AX4" s="100"/>
-      <c r="AY4" s="100"/>
-      <c r="AZ4" s="101"/>
-      <c r="BA4" s="99">
+      <c r="AU4" s="104"/>
+      <c r="AV4" s="104"/>
+      <c r="AW4" s="104"/>
+      <c r="AX4" s="104"/>
+      <c r="AY4" s="104"/>
+      <c r="AZ4" s="105"/>
+      <c r="BA4" s="103">
         <f>BA5</f>
         <v>45859</v>
       </c>
-      <c r="BB4" s="100"/>
-      <c r="BC4" s="100"/>
-      <c r="BD4" s="100"/>
-      <c r="BE4" s="100"/>
-      <c r="BF4" s="100"/>
-      <c r="BG4" s="101"/>
-      <c r="BH4" s="99">
+      <c r="BB4" s="104"/>
+      <c r="BC4" s="104"/>
+      <c r="BD4" s="104"/>
+      <c r="BE4" s="104"/>
+      <c r="BF4" s="104"/>
+      <c r="BG4" s="105"/>
+      <c r="BH4" s="103">
         <f>BH5</f>
         <v>45866</v>
       </c>
-      <c r="BI4" s="100"/>
-      <c r="BJ4" s="100"/>
-      <c r="BK4" s="100"/>
-      <c r="BL4" s="100"/>
-      <c r="BM4" s="100"/>
-      <c r="BN4" s="101"/>
+      <c r="BI4" s="104"/>
+      <c r="BJ4" s="104"/>
+      <c r="BK4" s="104"/>
+      <c r="BL4" s="104"/>
+      <c r="BM4" s="104"/>
+      <c r="BN4" s="105"/>
     </row>
     <row r="5" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="45"/>
-      <c r="C5" s="98"/>
-      <c r="D5" s="98"/>
-      <c r="E5" s="98"/>
-      <c r="F5" s="98"/>
-      <c r="G5" s="98"/>
-      <c r="H5" s="98"/>
-      <c r="I5" s="98"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
       <c r="K5" s="21">
         <f>InicioDelProyecto-WEEKDAY(InicioDelProyecto,1)+2+7*(SemanaParaMostrar-1)</f>
         <v>45817</v>
@@ -3050,7 +3056,7 @@
       <c r="H8" s="74"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5" t="str">
-        <f t="shared" ref="J8:J46" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
+        <f t="shared" ref="J8:J47" si="6">IF(OR(ISBLANK(Fecha_incio),ISBLANK(Fecha_final)),"",Fecha_final-Fecha_incio+1)</f>
         <v/>
       </c>
       <c r="K8" s="13"/>
@@ -5526,20 +5532,25 @@
       <c r="BN38" s="13"/>
     </row>
     <row r="39" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="90" t="s">
-        <v>77</v>
-      </c>
-      <c r="C39" s="90"/>
-      <c r="D39" s="91"/>
-      <c r="E39" s="91"/>
-      <c r="F39" s="92"/>
-      <c r="G39" s="93"/>
-      <c r="H39" s="94"/>
+      <c r="B39" s="69" t="s">
+        <v>81</v>
+      </c>
+      <c r="C39" s="58" t="s">
+        <v>133</v>
+      </c>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56" t="s">
+        <v>134</v>
+      </c>
+      <c r="F39" s="8">
+        <v>0</v>
+      </c>
+      <c r="G39" s="57">
+        <v>45934</v>
+      </c>
+      <c r="H39" s="57"/>
       <c r="I39" s="5"/>
-      <c r="J39" s="5" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
+      <c r="J39" s="5"/>
       <c r="K39" s="13"/>
       <c r="L39" s="13"/>
       <c r="M39" s="13"/>
@@ -5598,27 +5609,20 @@
       <c r="BN39" s="13"/>
     </row>
     <row r="40" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="C40" s="59" t="s">
-        <v>82</v>
-      </c>
-      <c r="D40" s="60" t="s">
-        <v>41</v>
-      </c>
-      <c r="E40" s="60"/>
-      <c r="F40" s="9">
-        <v>1</v>
-      </c>
-      <c r="G40" s="61">
-        <v>45837</v>
-      </c>
-      <c r="H40" s="61">
-        <v>45837</v>
-      </c>
+      <c r="B40" s="90" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="90"/>
+      <c r="D40" s="91"/>
+      <c r="E40" s="91"/>
+      <c r="F40" s="92"/>
+      <c r="G40" s="93"/>
+      <c r="H40" s="94"/>
       <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
+      <c r="J40" s="5" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
       <c r="K40" s="13"/>
       <c r="L40" s="13"/>
       <c r="M40" s="13"/>
@@ -5681,14 +5685,12 @@
         <v>78</v>
       </c>
       <c r="C41" s="59" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="D41" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="E41" s="60" t="s">
-        <v>43</v>
-      </c>
+      <c r="E41" s="60"/>
       <c r="F41" s="9">
         <v>1</v>
       </c>
@@ -5699,10 +5701,7 @@
         <v>45837</v>
       </c>
       <c r="I41" s="5"/>
-      <c r="J41" s="5">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
+      <c r="J41" s="5"/>
       <c r="K41" s="13"/>
       <c r="L41" s="13"/>
       <c r="M41" s="13"/>
@@ -5765,12 +5764,14 @@
         <v>78</v>
       </c>
       <c r="C42" s="59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D42" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="E42" s="60"/>
+      <c r="E42" s="60" t="s">
+        <v>43</v>
+      </c>
       <c r="F42" s="9">
         <v>1</v>
       </c>
@@ -5847,7 +5848,7 @@
         <v>78</v>
       </c>
       <c r="C43" s="59" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D43" s="60" t="s">
         <v>41</v>
@@ -5925,9 +5926,11 @@
       <c r="BN43" s="13"/>
     </row>
     <row r="44" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="36"/>
+      <c r="B44" s="29" t="s">
+        <v>78</v>
+      </c>
       <c r="C44" s="59" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D44" s="60" t="s">
         <v>41</v>
@@ -6007,21 +6010,25 @@
     <row r="45" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B45" s="36"/>
       <c r="C45" s="59" t="s">
-        <v>40</v>
-      </c>
-      <c r="D45" s="60"/>
-      <c r="E45" s="60" t="s">
-        <v>44</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D45" s="60" t="s">
+        <v>41</v>
+      </c>
+      <c r="E45" s="60"/>
       <c r="F45" s="9">
-        <v>0</v>
-      </c>
-      <c r="G45" s="61"/>
-      <c r="H45" s="61"/>
+        <v>1</v>
+      </c>
+      <c r="G45" s="61">
+        <v>45837</v>
+      </c>
+      <c r="H45" s="61">
+        <v>45837</v>
+      </c>
       <c r="I45" s="5"/>
-      <c r="J45" s="5" t="str">
+      <c r="J45" s="5">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K45" s="13"/>
       <c r="L45" s="13"/>
@@ -6081,101 +6088,180 @@
       <c r="BN45" s="13"/>
     </row>
     <row r="46" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="38" t="s">
-        <v>11</v>
-      </c>
-      <c r="B46" s="37"/>
-      <c r="C46" s="62"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="63"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="64"/>
-      <c r="H46" s="64"/>
-      <c r="I46" s="12"/>
-      <c r="J46" s="12" t="str">
+      <c r="B46" s="36"/>
+      <c r="C46" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="D46" s="60"/>
+      <c r="E46" s="60" t="s">
+        <v>44</v>
+      </c>
+      <c r="F46" s="9">
+        <v>0</v>
+      </c>
+      <c r="G46" s="61"/>
+      <c r="H46" s="61"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K46" s="15"/>
-      <c r="L46" s="15"/>
-      <c r="M46" s="15"/>
-      <c r="N46" s="15"/>
-      <c r="O46" s="15"/>
-      <c r="P46" s="15"/>
-      <c r="Q46" s="15"/>
-      <c r="R46" s="15"/>
-      <c r="S46" s="15"/>
-      <c r="T46" s="15"/>
-      <c r="U46" s="15"/>
-      <c r="V46" s="15"/>
-      <c r="W46" s="15"/>
-      <c r="X46" s="15"/>
-      <c r="Y46" s="15"/>
-      <c r="Z46" s="15"/>
-      <c r="AA46" s="15"/>
-      <c r="AB46" s="15"/>
-      <c r="AC46" s="15"/>
-      <c r="AD46" s="15"/>
-      <c r="AE46" s="15"/>
-      <c r="AF46" s="15"/>
-      <c r="AG46" s="15"/>
-      <c r="AH46" s="15"/>
-      <c r="AI46" s="15"/>
-      <c r="AJ46" s="15"/>
-      <c r="AK46" s="15"/>
-      <c r="AL46" s="15"/>
-      <c r="AM46" s="15"/>
-      <c r="AN46" s="15"/>
-      <c r="AO46" s="15"/>
-      <c r="AP46" s="15"/>
-      <c r="AQ46" s="15"/>
-      <c r="AR46" s="15"/>
-      <c r="AS46" s="15"/>
-      <c r="AT46" s="15"/>
-      <c r="AU46" s="15"/>
-      <c r="AV46" s="15"/>
-      <c r="AW46" s="15"/>
-      <c r="AX46" s="15"/>
-      <c r="AY46" s="15"/>
-      <c r="AZ46" s="15"/>
-      <c r="BA46" s="15"/>
-      <c r="BB46" s="15"/>
-      <c r="BC46" s="15"/>
-      <c r="BD46" s="15"/>
-      <c r="BE46" s="15"/>
-      <c r="BF46" s="15"/>
-      <c r="BG46" s="15"/>
-      <c r="BH46" s="15"/>
-      <c r="BI46" s="15"/>
-      <c r="BJ46" s="15"/>
-      <c r="BK46" s="15"/>
-      <c r="BL46" s="15"/>
-      <c r="BM46" s="15"/>
-      <c r="BN46" s="15"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="13"/>
+      <c r="N46" s="13"/>
+      <c r="O46" s="13"/>
+      <c r="P46" s="13"/>
+      <c r="Q46" s="13"/>
+      <c r="R46" s="13"/>
+      <c r="S46" s="13"/>
+      <c r="T46" s="13"/>
+      <c r="U46" s="13"/>
+      <c r="V46" s="13"/>
+      <c r="W46" s="13"/>
+      <c r="X46" s="13"/>
+      <c r="Y46" s="13"/>
+      <c r="Z46" s="13"/>
+      <c r="AA46" s="13"/>
+      <c r="AB46" s="13"/>
+      <c r="AC46" s="13"/>
+      <c r="AD46" s="13"/>
+      <c r="AE46" s="13"/>
+      <c r="AF46" s="13"/>
+      <c r="AG46" s="13"/>
+      <c r="AH46" s="13"/>
+      <c r="AI46" s="13"/>
+      <c r="AJ46" s="13"/>
+      <c r="AK46" s="13"/>
+      <c r="AL46" s="13"/>
+      <c r="AM46" s="13"/>
+      <c r="AN46" s="13"/>
+      <c r="AO46" s="13"/>
+      <c r="AP46" s="13"/>
+      <c r="AQ46" s="13"/>
+      <c r="AR46" s="13"/>
+      <c r="AS46" s="13"/>
+      <c r="AT46" s="13"/>
+      <c r="AU46" s="13"/>
+      <c r="AV46" s="13"/>
+      <c r="AW46" s="13"/>
+      <c r="AX46" s="13"/>
+      <c r="AY46" s="13"/>
+      <c r="AZ46" s="13"/>
+      <c r="BA46" s="13"/>
+      <c r="BB46" s="13"/>
+      <c r="BC46" s="13"/>
+      <c r="BD46" s="13"/>
+      <c r="BE46" s="13"/>
+      <c r="BF46" s="13"/>
+      <c r="BG46" s="13"/>
+      <c r="BH46" s="13"/>
+      <c r="BI46" s="13"/>
+      <c r="BJ46" s="13"/>
+      <c r="BK46" s="13"/>
+      <c r="BL46" s="13"/>
+      <c r="BM46" s="13"/>
+      <c r="BN46" s="13"/>
     </row>
     <row r="47" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="10"/>
-      <c r="C47" s="65" t="s">
+      <c r="A47" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" s="37"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="63"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="64"/>
+      <c r="H47" s="64"/>
+      <c r="I47" s="12"/>
+      <c r="J47" s="12" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="K47" s="15"/>
+      <c r="L47" s="15"/>
+      <c r="M47" s="15"/>
+      <c r="N47" s="15"/>
+      <c r="O47" s="15"/>
+      <c r="P47" s="15"/>
+      <c r="Q47" s="15"/>
+      <c r="R47" s="15"/>
+      <c r="S47" s="15"/>
+      <c r="T47" s="15"/>
+      <c r="U47" s="15"/>
+      <c r="V47" s="15"/>
+      <c r="W47" s="15"/>
+      <c r="X47" s="15"/>
+      <c r="Y47" s="15"/>
+      <c r="Z47" s="15"/>
+      <c r="AA47" s="15"/>
+      <c r="AB47" s="15"/>
+      <c r="AC47" s="15"/>
+      <c r="AD47" s="15"/>
+      <c r="AE47" s="15"/>
+      <c r="AF47" s="15"/>
+      <c r="AG47" s="15"/>
+      <c r="AH47" s="15"/>
+      <c r="AI47" s="15"/>
+      <c r="AJ47" s="15"/>
+      <c r="AK47" s="15"/>
+      <c r="AL47" s="15"/>
+      <c r="AM47" s="15"/>
+      <c r="AN47" s="15"/>
+      <c r="AO47" s="15"/>
+      <c r="AP47" s="15"/>
+      <c r="AQ47" s="15"/>
+      <c r="AR47" s="15"/>
+      <c r="AS47" s="15"/>
+      <c r="AT47" s="15"/>
+      <c r="AU47" s="15"/>
+      <c r="AV47" s="15"/>
+      <c r="AW47" s="15"/>
+      <c r="AX47" s="15"/>
+      <c r="AY47" s="15"/>
+      <c r="AZ47" s="15"/>
+      <c r="BA47" s="15"/>
+      <c r="BB47" s="15"/>
+      <c r="BC47" s="15"/>
+      <c r="BD47" s="15"/>
+      <c r="BE47" s="15"/>
+      <c r="BF47" s="15"/>
+      <c r="BG47" s="15"/>
+      <c r="BH47" s="15"/>
+      <c r="BI47" s="15"/>
+      <c r="BJ47" s="15"/>
+      <c r="BK47" s="15"/>
+      <c r="BL47" s="15"/>
+      <c r="BM47" s="15"/>
+      <c r="BN47" s="15"/>
+    </row>
+    <row r="48" spans="1:66" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="10"/>
+      <c r="C48" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="18"/>
-      <c r="I47" s="2"/>
-    </row>
-    <row r="49" spans="4:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D49" s="66"/>
-      <c r="E49" s="66"/>
-      <c r="H49" s="67"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="17"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="2"/>
     </row>
     <row r="50" spans="4:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D50" s="44"/>
-      <c r="E50" s="44"/>
+      <c r="D50" s="66"/>
+      <c r="E50" s="66"/>
+      <c r="H50" s="67"/>
+    </row>
+    <row r="51" spans="4:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D51" s="44"/>
+      <c r="E51" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="C5:I5"/>
+    <mergeCell ref="AM4:AS4"/>
+    <mergeCell ref="AT4:AZ4"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="BA4:BG4"/>
@@ -6187,11 +6273,8 @@
     <mergeCell ref="AF4:AL4"/>
     <mergeCell ref="D3:F3"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="C5:I5"/>
-    <mergeCell ref="AM4:AS4"/>
-    <mergeCell ref="AT4:AZ4"/>
   </mergeCells>
-  <conditionalFormatting sqref="F7:F47">
+  <conditionalFormatting sqref="F7:F48">
     <cfRule type="dataBar" priority="16">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6205,12 +6288,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:BN46">
+  <conditionalFormatting sqref="K5:BN47">
     <cfRule type="expression" dxfId="2" priority="35">
       <formula>AND(TODAY()&gt;=K$5,TODAY()&lt;L$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K7:BN46">
+  <conditionalFormatting sqref="K7:BN47">
     <cfRule type="expression" dxfId="1" priority="29">
       <formula>AND(Fecha_incio&lt;=K$5,ROUNDDOWN((Fecha_final-Fecha_incio+1)*Progresos,0)+Fecha_incio-1&gt;=K$5)</formula>
     </cfRule>
@@ -6245,7 +6328,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>F7:F47</xm:sqref>
+          <xm:sqref>F7:F48</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -6275,70 +6358,70 @@
       <c r="E1" s="107"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="103" t="s">
+      <c r="A2" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="103" t="s">
+      <c r="B2" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="103" t="s">
+      <c r="C2" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="103" t="s">
+      <c r="D2" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="103" t="s">
+      <c r="E2" s="96" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="104" t="s">
+      <c r="A3" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="104" t="s">
+      <c r="B3" s="97" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="105">
+      <c r="C3" s="98">
         <v>0.3</v>
       </c>
-      <c r="D3" s="106">
+      <c r="D3" s="99">
         <v>45830</v>
       </c>
-      <c r="E3" s="106">
+      <c r="E3" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="104" t="s">
+      <c r="A4" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="104" t="s">
+      <c r="B4" s="97" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="105">
+      <c r="C4" s="98">
         <v>0.8</v>
       </c>
-      <c r="D4" s="106">
+      <c r="D4" s="99">
         <v>45837</v>
       </c>
-      <c r="E4" s="106">
+      <c r="E4" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="104" t="s">
+      <c r="A5" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B5" s="104" t="s">
+      <c r="B5" s="97" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="105">
+      <c r="C5" s="98">
         <v>0.8</v>
       </c>
-      <c r="D5" s="106">
+      <c r="D5" s="99">
         <v>45837</v>
       </c>
-      <c r="E5" s="106">
+      <c r="E5" s="99">
         <v>45931</v>
       </c>
     </row>
@@ -6352,189 +6435,189 @@
       <c r="E7" s="107"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="103" t="s">
+      <c r="A8" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="B8" s="103" t="s">
+      <c r="B8" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="103" t="s">
+      <c r="C8" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="103" t="s">
+      <c r="D8" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="103" t="s">
+      <c r="E8" s="96" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="104" t="s">
+      <c r="A9" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="104" t="s">
+      <c r="B9" s="97" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="105">
+      <c r="C9" s="98">
         <v>0.8</v>
       </c>
-      <c r="D9" s="106">
+      <c r="D9" s="99">
         <v>45822</v>
       </c>
-      <c r="E9" s="106">
+      <c r="E9" s="99">
         <v>45931</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="104" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="104" t="s">
+      <c r="B10" s="97" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="105">
+      <c r="C10" s="98">
         <v>0.8</v>
       </c>
-      <c r="D10" s="106">
+      <c r="D10" s="99">
         <v>45837</v>
       </c>
-      <c r="E10" s="106">
+      <c r="E10" s="99">
         <v>45837</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="104" t="s">
+      <c r="A11" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="104" t="s">
+      <c r="B11" s="97" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="105">
+      <c r="C11" s="98">
         <v>0.1</v>
       </c>
-      <c r="D11" s="106">
+      <c r="D11" s="99">
         <v>45851</v>
       </c>
-      <c r="E11" s="106">
+      <c r="E11" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="104" t="s">
+      <c r="A12" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="104" t="s">
+      <c r="B12" s="97" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="105">
+      <c r="C12" s="98">
         <v>0.2</v>
       </c>
-      <c r="D12" s="106">
+      <c r="D12" s="99">
         <v>45837</v>
       </c>
-      <c r="E12" s="106">
+      <c r="E12" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="104" t="s">
+      <c r="A13" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B13" s="104" t="s">
+      <c r="B13" s="97" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="105">
+      <c r="C13" s="98">
         <v>1</v>
       </c>
-      <c r="D13" s="106">
+      <c r="D13" s="99">
         <v>45828</v>
       </c>
-      <c r="E13" s="106">
+      <c r="E13" s="99">
         <v>45830</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="104" t="s">
+      <c r="A14" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B14" s="104" t="s">
+      <c r="B14" s="97" t="s">
         <v>107</v>
       </c>
-      <c r="C14" s="105">
+      <c r="C14" s="98">
         <v>0</v>
       </c>
-      <c r="D14" s="106">
+      <c r="D14" s="99">
         <v>45830</v>
       </c>
-      <c r="E14" s="106">
+      <c r="E14" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="104" t="s">
+      <c r="A15" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="104" t="s">
+      <c r="B15" s="97" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="105">
+      <c r="C15" s="98">
         <v>1</v>
       </c>
-      <c r="D15" s="106">
+      <c r="D15" s="99">
         <v>45834</v>
       </c>
-      <c r="E15" s="106">
+      <c r="E15" s="99">
         <v>45838</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="104" t="s">
+      <c r="A16" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B16" s="104" t="s">
+      <c r="B16" s="97" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="105">
+      <c r="C16" s="98">
         <v>0.5</v>
       </c>
-      <c r="D16" s="106">
+      <c r="D16" s="99">
         <v>45834</v>
       </c>
-      <c r="E16" s="106">
+      <c r="E16" s="99">
         <v>45839</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="104" t="s">
+      <c r="A17" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="104" t="s">
+      <c r="B17" s="97" t="s">
         <v>110</v>
       </c>
-      <c r="C17" s="105">
+      <c r="C17" s="98">
         <v>0.5</v>
       </c>
-      <c r="D17" s="106">
+      <c r="D17" s="99">
         <v>45829</v>
       </c>
-      <c r="E17" s="106">
+      <c r="E17" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="104" t="s">
+      <c r="A18" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="104" t="s">
+      <c r="B18" s="97" t="s">
         <v>111</v>
       </c>
-      <c r="C18" s="105">
+      <c r="C18" s="98">
         <v>0.75</v>
       </c>
-      <c r="D18" s="106">
+      <c r="D18" s="99">
         <v>45829</v>
       </c>
-      <c r="E18" s="106">
+      <c r="E18" s="99">
         <v>45931</v>
       </c>
     </row>
@@ -6548,138 +6631,138 @@
       <c r="E20" s="108"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="103" t="s">
+      <c r="A21" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="103" t="s">
+      <c r="B21" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="103" t="s">
+      <c r="C21" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="D21" s="103" t="s">
+      <c r="D21" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="E21" s="103" t="s">
+      <c r="E21" s="96" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="104" t="s">
+      <c r="A22" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B22" s="104" t="s">
+      <c r="B22" s="97" t="s">
         <v>112</v>
       </c>
-      <c r="C22" s="105">
+      <c r="C22" s="98">
         <v>1</v>
       </c>
-      <c r="D22" s="106">
+      <c r="D22" s="99">
         <v>45858</v>
       </c>
-      <c r="E22" s="106">
+      <c r="E22" s="99">
         <v>45862</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="104" t="s">
+      <c r="A23" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B23" s="104" t="s">
+      <c r="B23" s="97" t="s">
         <v>113</v>
       </c>
-      <c r="C23" s="105">
+      <c r="C23" s="98">
         <v>1</v>
       </c>
-      <c r="D23" s="106">
+      <c r="D23" s="99">
         <v>45858</v>
       </c>
-      <c r="E23" s="106">
+      <c r="E23" s="99">
         <v>45862</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="104" t="s">
+      <c r="A24" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B24" s="104" t="s">
+      <c r="B24" s="97" t="s">
         <v>114</v>
       </c>
-      <c r="C24" s="105">
+      <c r="C24" s="98">
         <v>1</v>
       </c>
-      <c r="D24" s="106">
+      <c r="D24" s="99">
         <v>45829</v>
       </c>
-      <c r="E24" s="106">
+      <c r="E24" s="99">
         <v>45829</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="104" t="s">
+      <c r="A25" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="104" t="s">
+      <c r="B25" s="97" t="s">
         <v>115</v>
       </c>
-      <c r="C25" s="105">
+      <c r="C25" s="98">
         <v>1</v>
       </c>
-      <c r="D25" s="106">
+      <c r="D25" s="99">
         <v>45830</v>
       </c>
-      <c r="E25" s="106">
+      <c r="E25" s="99">
         <v>45834</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="104" t="s">
+      <c r="A26" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B26" s="104" t="s">
+      <c r="B26" s="97" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="105">
+      <c r="C26" s="98">
         <v>1</v>
       </c>
-      <c r="D26" s="106">
+      <c r="D26" s="99">
         <v>45858</v>
       </c>
-      <c r="E26" s="106">
+      <c r="E26" s="99">
         <v>45858</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="104" t="s">
+      <c r="A27" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="B27" s="104" t="s">
+      <c r="B27" s="97" t="s">
         <v>117</v>
       </c>
-      <c r="C27" s="105">
+      <c r="C27" s="98">
         <v>0</v>
       </c>
-      <c r="D27" s="106" t="s">
+      <c r="D27" s="99" t="s">
         <v>105</v>
       </c>
-      <c r="E27" s="106">
+      <c r="E27" s="99">
         <v>45931</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="104" t="s">
+      <c r="A28" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="104" t="s">
+      <c r="B28" s="97" t="s">
         <v>118</v>
       </c>
-      <c r="C28" s="105">
+      <c r="C28" s="98">
         <v>0</v>
       </c>
-      <c r="D28" s="106" t="s">
+      <c r="D28" s="99" t="s">
         <v>105</v>
       </c>
-      <c r="E28" s="106">
+      <c r="E28" s="99">
         <v>45931</v>
       </c>
     </row>
@@ -6693,104 +6776,104 @@
       <c r="E30" s="107"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="103" t="s">
+      <c r="A31" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="B31" s="103" t="s">
+      <c r="B31" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C31" s="103" t="s">
+      <c r="C31" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="D31" s="103" t="s">
+      <c r="D31" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="E31" s="103" t="s">
+      <c r="E31" s="96" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="104" t="s">
+      <c r="A32" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="104" t="s">
+      <c r="B32" s="97" t="s">
         <v>121</v>
       </c>
-      <c r="C32" s="105">
+      <c r="C32" s="98">
         <v>1</v>
       </c>
-      <c r="D32" s="106">
+      <c r="D32" s="99">
         <v>45829</v>
       </c>
-      <c r="E32" s="106">
+      <c r="E32" s="99">
         <v>45829</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="104" t="s">
+      <c r="A33" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B33" s="104" t="s">
+      <c r="B33" s="97" t="s">
         <v>122</v>
       </c>
-      <c r="C33" s="105">
+      <c r="C33" s="98">
         <v>1</v>
       </c>
-      <c r="D33" s="106">
+      <c r="D33" s="99">
         <v>45837</v>
       </c>
-      <c r="E33" s="106">
+      <c r="E33" s="99">
         <v>45842</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="104" t="s">
+      <c r="A34" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B34" s="104" t="s">
+      <c r="B34" s="97" t="s">
         <v>123</v>
       </c>
-      <c r="C34" s="105">
+      <c r="C34" s="98">
         <v>1</v>
       </c>
-      <c r="D34" s="106">
+      <c r="D34" s="99">
         <v>45829</v>
       </c>
-      <c r="E34" s="106">
+      <c r="E34" s="99">
         <v>45829</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="104" t="s">
+      <c r="A35" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="104" t="s">
+      <c r="B35" s="97" t="s">
         <v>124</v>
       </c>
-      <c r="C35" s="105">
+      <c r="C35" s="98">
         <v>1</v>
       </c>
-      <c r="D35" s="106">
+      <c r="D35" s="99">
         <v>45837</v>
       </c>
-      <c r="E35" s="106">
+      <c r="E35" s="99">
         <v>45851</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A36" s="104" t="s">
+      <c r="A36" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="104" t="s">
+      <c r="B36" s="97" t="s">
         <v>132</v>
       </c>
-      <c r="C36" s="105">
+      <c r="C36" s="98">
         <v>1</v>
       </c>
-      <c r="D36" s="106">
+      <c r="D36" s="99">
         <v>45837</v>
       </c>
-      <c r="E36" s="106">
+      <c r="E36" s="99">
         <v>45851</v>
       </c>
     </row>
@@ -6804,121 +6887,121 @@
       <c r="E38" s="107"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="103" t="s">
+      <c r="A39" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="B39" s="103" t="s">
+      <c r="B39" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C39" s="103" t="s">
+      <c r="C39" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="D39" s="103" t="s">
+      <c r="D39" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="E39" s="103" t="s">
+      <c r="E39" s="96" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="104" t="s">
+      <c r="A40" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="104" t="s">
+      <c r="B40" s="97" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="105">
+      <c r="C40" s="98">
         <v>1</v>
       </c>
-      <c r="D40" s="106">
+      <c r="D40" s="99">
         <v>45837</v>
       </c>
-      <c r="E40" s="106">
+      <c r="E40" s="99">
         <v>45837</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="104" t="s">
+      <c r="A41" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B41" s="104" t="s">
+      <c r="B41" s="97" t="s">
         <v>127</v>
       </c>
-      <c r="C41" s="105">
+      <c r="C41" s="98">
         <v>1</v>
       </c>
-      <c r="D41" s="106">
+      <c r="D41" s="99">
         <v>45837</v>
       </c>
-      <c r="E41" s="106">
+      <c r="E41" s="99">
         <v>45837</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="104" t="s">
+      <c r="A42" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B42" s="104" t="s">
+      <c r="B42" s="97" t="s">
         <v>128</v>
       </c>
-      <c r="C42" s="105">
+      <c r="C42" s="98">
         <v>1</v>
       </c>
-      <c r="D42" s="106">
+      <c r="D42" s="99">
         <v>45837</v>
       </c>
-      <c r="E42" s="106">
+      <c r="E42" s="99">
         <v>45837</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="104" t="s">
+      <c r="A43" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B43" s="104" t="s">
+      <c r="B43" s="97" t="s">
         <v>129</v>
       </c>
-      <c r="C43" s="105">
+      <c r="C43" s="98">
         <v>1</v>
       </c>
-      <c r="D43" s="106">
+      <c r="D43" s="99">
         <v>45837</v>
       </c>
-      <c r="E43" s="106">
+      <c r="E43" s="99">
         <v>45837</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="104" t="s">
+      <c r="A44" s="97" t="s">
         <v>78</v>
       </c>
-      <c r="B44" s="104" t="s">
+      <c r="B44" s="97" t="s">
         <v>130</v>
       </c>
-      <c r="C44" s="105">
+      <c r="C44" s="98">
         <v>1</v>
       </c>
-      <c r="D44" s="106">
+      <c r="D44" s="99">
         <v>45837</v>
       </c>
-      <c r="E44" s="106">
+      <c r="E44" s="99">
         <v>45837</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="104" t="s">
+      <c r="A45" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="104" t="s">
+      <c r="B45" s="97" t="s">
         <v>131</v>
       </c>
-      <c r="C45" s="105">
+      <c r="C45" s="98">
         <v>0</v>
       </c>
-      <c r="D45" s="106">
+      <c r="D45" s="99">
         <v>45837</v>
       </c>
-      <c r="E45" s="106">
+      <c r="E45" s="99">
         <v>45931</v>
       </c>
     </row>

</xml_diff>